<commit_message>
versão atual flask + htmx
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="LjW3JD/1QGFiHUIMpmQSIlS+VWTI5JrYWhRAQN5qqsk="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="g92YoGyz9TbpAesj0bHD7JqmwjJ/ajMmkP0Wlw/eQtQ="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="282">
   <si>
     <t>nome</t>
   </si>
@@ -748,15 +748,6 @@
     <t>Rosca spider</t>
   </si>
   <si>
-    <t>Salto de corda</t>
-  </si>
-  <si>
-    <t>Sem equipamento</t>
-  </si>
-  <si>
-    <t>gastrocnêmio, sóleo</t>
-  </si>
-  <si>
     <t>Serrote</t>
   </si>
   <si>
@@ -1011,7 +1002,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1078,9 +1069,6 @@
     </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="12" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="13" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="12" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="13" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1089,38 +1077,14 @@
     <xf borderId="0" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="14" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf borderId="0" fillId="14" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="9" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="15" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1131,9 +1095,6 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3245,7 +3206,7 @@
       <c r="AA33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="26" t="s">
+      <c r="A34" s="10" t="s">
         <v>127</v>
       </c>
       <c r="B34" s="11" t="s">
@@ -3862,10 +3823,10 @@
         <v>155</v>
       </c>
       <c r="D45" s="2"/>
-      <c r="E45" s="27" t="s">
+      <c r="E45" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="F45" s="27" t="s">
+      <c r="F45" s="26" t="s">
         <v>28</v>
       </c>
       <c r="G45" s="11" t="s">
@@ -3883,7 +3844,7 @@
       <c r="K45" s="21">
         <v>3.0</v>
       </c>
-      <c r="L45" s="28" t="s">
+      <c r="L45" s="27" t="s">
         <v>30</v>
       </c>
       <c r="M45" s="2" t="s">
@@ -3917,10 +3878,10 @@
         <v>157</v>
       </c>
       <c r="D46" s="4"/>
-      <c r="E46" s="29" t="s">
+      <c r="E46" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="F46" s="29" t="s">
+      <c r="F46" s="28" t="s">
         <v>28</v>
       </c>
       <c r="G46" s="11" t="s">
@@ -3938,7 +3899,7 @@
       <c r="K46" s="7">
         <v>4.0</v>
       </c>
-      <c r="L46" s="30" t="s">
+      <c r="L46" s="29" t="s">
         <v>30</v>
       </c>
       <c r="M46" s="4" t="s">
@@ -4612,39 +4573,39 @@
       <c r="AA58" s="4"/>
     </row>
     <row r="59">
-      <c r="A59" s="31" t="s">
+      <c r="A59" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B59" s="32"/>
-      <c r="C59" s="31" t="s">
+      <c r="B59" s="4"/>
+      <c r="C59" s="9" t="s">
         <v>189</v>
       </c>
       <c r="D59" s="2"/>
-      <c r="E59" s="33" t="s">
+      <c r="E59" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F59" s="34" t="s">
+      <c r="F59" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G59" s="35" t="s">
+      <c r="G59" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H59" s="36" t="s">
+      <c r="H59" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I59" s="36" t="s">
+      <c r="I59" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J59" s="37">
+      <c r="J59" s="31">
         <v>1.0</v>
       </c>
-      <c r="K59" s="38">
+      <c r="K59" s="31">
         <v>2.0</v>
       </c>
-      <c r="L59" s="36" t="s">
+      <c r="L59" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M59" s="35" t="s">
+      <c r="M59" s="2" t="s">
         <v>23</v>
       </c>
       <c r="N59" s="9" t="s">
@@ -4665,36 +4626,36 @@
       <c r="AA59" s="4"/>
     </row>
     <row r="60">
-      <c r="A60" s="26" t="s">
+      <c r="A60" s="10" t="s">
         <v>190</v>
       </c>
       <c r="B60" s="2"/>
-      <c r="C60" s="26" t="s">
+      <c r="C60" s="10" t="s">
         <v>17</v>
       </c>
       <c r="D60" s="10"/>
-      <c r="E60" s="39" t="s">
+      <c r="E60" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F60" s="39" t="s">
+      <c r="F60" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="G60" s="40" t="s">
+      <c r="G60" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="H60" s="40" t="s">
+      <c r="H60" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="I60" s="40" t="s">
+      <c r="I60" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="J60" s="40">
+      <c r="J60" s="11">
         <v>1.0</v>
       </c>
-      <c r="K60" s="40">
+      <c r="K60" s="11">
         <v>1.0</v>
       </c>
-      <c r="L60" s="41" t="s">
+      <c r="L60" s="16" t="s">
         <v>22</v>
       </c>
       <c r="M60" s="11" t="s">
@@ -5696,7 +5657,7 @@
       <c r="K78" s="21">
         <v>3.0</v>
       </c>
-      <c r="L78" s="42" t="s">
+      <c r="L78" s="32" t="s">
         <v>30</v>
       </c>
       <c r="M78" s="2" t="s">
@@ -6274,157 +6235,157 @@
       <c r="AA88" s="2"/>
     </row>
     <row r="89">
-      <c r="A89" s="10" t="s">
+      <c r="A89" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="B89" s="11"/>
-      <c r="C89" s="10" t="s">
+      <c r="B89" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E89" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F89" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="G89" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I89" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="J89" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="K89" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="L89" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="M89" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="N89" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="O89" s="3"/>
+      <c r="P89" s="4"/>
+      <c r="Q89" s="4"/>
+      <c r="R89" s="4"/>
+      <c r="S89" s="4"/>
+      <c r="T89" s="4"/>
+      <c r="U89" s="4"/>
+      <c r="V89" s="4"/>
+      <c r="W89" s="4"/>
+      <c r="X89" s="4"/>
+      <c r="Y89" s="4"/>
+      <c r="Z89" s="4"/>
+      <c r="AA89" s="4"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="D89" s="10"/>
-      <c r="E89" s="15" t="s">
+      <c r="B90" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C90" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D90" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E90" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="F89" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="G89" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="H89" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="I89" s="13" t="s">
+      <c r="F90" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G90" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="H90" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I90" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="J89" s="11">
+      <c r="J90" s="11">
         <v>1.0</v>
       </c>
-      <c r="K89" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="L89" s="16" t="s">
+      <c r="K90" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="L90" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="M89" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="N89" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="O89" s="10"/>
-      <c r="P89" s="2"/>
-      <c r="Q89" s="2"/>
-      <c r="R89" s="2"/>
-      <c r="S89" s="2"/>
-      <c r="T89" s="2"/>
-      <c r="U89" s="2"/>
-      <c r="V89" s="2"/>
-      <c r="W89" s="2"/>
-      <c r="X89" s="2"/>
-      <c r="Y89" s="2"/>
-      <c r="Z89" s="2"/>
-      <c r="AA89" s="2"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="B90" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E90" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="F90" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="G90" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H90" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I90" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="J90" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="K90" s="7">
-        <v>4.0</v>
-      </c>
-      <c r="L90" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="M90" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="N90" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="O90" s="3"/>
-      <c r="P90" s="4"/>
-      <c r="Q90" s="4"/>
-      <c r="R90" s="4"/>
-      <c r="S90" s="4"/>
-      <c r="T90" s="4"/>
-      <c r="U90" s="4"/>
-      <c r="V90" s="4"/>
-      <c r="W90" s="4"/>
-      <c r="X90" s="4"/>
-      <c r="Y90" s="4"/>
-      <c r="Z90" s="4"/>
-      <c r="AA90" s="4"/>
+      <c r="M90" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="N90" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="O90" s="10"/>
+      <c r="P90" s="2"/>
+      <c r="Q90" s="2"/>
+      <c r="R90" s="2"/>
+      <c r="S90" s="2"/>
+      <c r="T90" s="2"/>
+      <c r="U90" s="2"/>
+      <c r="V90" s="2"/>
+      <c r="W90" s="2"/>
+      <c r="X90" s="2"/>
+      <c r="Y90" s="2"/>
+      <c r="Z90" s="2"/>
+      <c r="AA90" s="2"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B91" s="11"/>
+      <c r="C91" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="D91" s="10"/>
+      <c r="E91" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F91" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G91" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H91" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I91" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J91" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="K91" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="L91" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="M91" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="B91" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C91" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="D91" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E91" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="F91" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="G91" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="H91" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I91" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="J91" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="K91" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="L91" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="M91" s="11" t="s">
-        <v>35</v>
-      </c>
       <c r="N91" s="10" t="s">
-        <v>32</v>
+        <v>248</v>
       </c>
       <c r="O91" s="10"/>
       <c r="P91" s="2"/>
@@ -6441,126 +6402,128 @@
       <c r="AA91" s="2"/>
     </row>
     <row r="92">
-      <c r="A92" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="B92" s="11"/>
-      <c r="C92" s="10" t="s">
+      <c r="A92" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="D92" s="10"/>
-      <c r="E92" s="12" t="s">
+      <c r="B92" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C92" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D92" s="9"/>
+      <c r="E92" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="F92" s="12" t="s">
+      <c r="F92" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G92" s="11" t="s">
+      <c r="G92" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H92" s="40" t="s">
-        <v>63</v>
-      </c>
-      <c r="I92" s="13" t="s">
+      <c r="H92" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I92" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J92" s="11">
+      <c r="J92" s="34">
         <v>3.0</v>
       </c>
-      <c r="K92" s="11">
+      <c r="K92" s="35">
         <v>3.0</v>
       </c>
-      <c r="L92" s="16" t="s">
+      <c r="L92" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M92" s="11" t="s">
+      <c r="M92" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N92" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="O92" s="2"/>
+      <c r="P92" s="4"/>
+      <c r="Q92" s="4"/>
+      <c r="R92" s="4"/>
+      <c r="S92" s="4"/>
+      <c r="T92" s="4"/>
+      <c r="U92" s="4"/>
+      <c r="V92" s="4"/>
+      <c r="W92" s="4"/>
+      <c r="X92" s="4"/>
+      <c r="Y92" s="4"/>
+      <c r="Z92" s="4"/>
+      <c r="AA92" s="4"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="N92" s="10" t="s">
+      <c r="B93" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="O92" s="10"/>
-      <c r="P92" s="2"/>
-      <c r="Q92" s="2"/>
-      <c r="R92" s="2"/>
-      <c r="S92" s="2"/>
-      <c r="T92" s="2"/>
-      <c r="U92" s="2"/>
-      <c r="V92" s="2"/>
-      <c r="W92" s="2"/>
-      <c r="X92" s="2"/>
-      <c r="Y92" s="2"/>
-      <c r="Z92" s="2"/>
-      <c r="AA92" s="2"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="31" t="s">
-        <v>252</v>
-      </c>
-      <c r="B93" s="35" t="s">
-        <v>252</v>
-      </c>
-      <c r="C93" s="9" t="s">
+      <c r="C93" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D93" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D93" s="9"/>
-      <c r="E93" s="27" t="s">
+      <c r="E93" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F93" s="44" t="s">
+      <c r="F93" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G93" s="2" t="s">
+      <c r="G93" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="H93" s="2" t="s">
+      <c r="H93" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="I93" s="2" t="s">
+      <c r="I93" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J93" s="45">
+      <c r="J93" s="11">
         <v>3.0</v>
       </c>
-      <c r="K93" s="46">
+      <c r="K93" s="11">
         <v>3.0</v>
       </c>
-      <c r="L93" s="2" t="s">
+      <c r="L93" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="M93" s="2" t="s">
+      <c r="M93" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="N93" s="9" t="s">
+      <c r="N93" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="O93" s="2"/>
-      <c r="P93" s="4"/>
-      <c r="Q93" s="4"/>
-      <c r="R93" s="4"/>
-      <c r="S93" s="4"/>
-      <c r="T93" s="4"/>
-      <c r="U93" s="4"/>
-      <c r="V93" s="4"/>
-      <c r="W93" s="4"/>
-      <c r="X93" s="4"/>
-      <c r="Y93" s="4"/>
-      <c r="Z93" s="4"/>
-      <c r="AA93" s="4"/>
+      <c r="O93" s="10"/>
+      <c r="P93" s="2"/>
+      <c r="Q93" s="2"/>
+      <c r="R93" s="2"/>
+      <c r="S93" s="2"/>
+      <c r="T93" s="2"/>
+      <c r="U93" s="2"/>
+      <c r="V93" s="2"/>
+      <c r="W93" s="2"/>
+      <c r="X93" s="2"/>
+      <c r="Y93" s="2"/>
+      <c r="Z93" s="2"/>
+      <c r="AA93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C94" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="D94" s="10" t="s">
-        <v>44</v>
-      </c>
+      <c r="D94" s="10"/>
       <c r="E94" s="12" t="s">
         <v>27</v>
       </c>
@@ -6571,9 +6534,9 @@
         <v>46</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="I94" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="I94" s="33" t="s">
         <v>8</v>
       </c>
       <c r="J94" s="11">
@@ -6586,7 +6549,7 @@
         <v>22</v>
       </c>
       <c r="M94" s="11" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="N94" s="10" t="s">
         <v>49</v>
@@ -6607,44 +6570,44 @@
     </row>
     <row r="95">
       <c r="A95" s="10" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B95" s="11" t="s">
         <v>254</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="D95" s="10"/>
       <c r="E95" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F95" s="12" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G95" s="11" t="s">
-        <v>46</v>
+        <v>159</v>
       </c>
       <c r="H95" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="I95" s="43" t="s">
-        <v>8</v>
+        <v>47</v>
+      </c>
+      <c r="I95" s="11" t="s">
+        <v>21</v>
       </c>
       <c r="J95" s="11">
         <v>3.0</v>
       </c>
       <c r="K95" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="L95" s="16" t="s">
-        <v>22</v>
+        <v>4.0</v>
+      </c>
+      <c r="L95" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="M95" s="11" t="s">
-        <v>85</v>
+        <v>162</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>49</v>
+        <v>174</v>
       </c>
       <c r="O95" s="10"/>
       <c r="P95" s="2"/>
@@ -6662,13 +6625,13 @@
     </row>
     <row r="96">
       <c r="A96" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C96" s="10" t="s">
-        <v>123</v>
+        <v>44</v>
       </c>
       <c r="D96" s="10"/>
       <c r="E96" s="12" t="s">
@@ -6690,7 +6653,7 @@
         <v>3.0</v>
       </c>
       <c r="K96" s="11">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="L96" s="11" t="s">
         <v>30</v>
@@ -6717,44 +6680,44 @@
     </row>
     <row r="97">
       <c r="A97" s="10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>257</v>
+        <v>51</v>
       </c>
       <c r="C97" s="10" t="s">
         <v>44</v>
       </c>
       <c r="D97" s="10"/>
-      <c r="E97" s="12" t="s">
+      <c r="E97" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="F97" s="12" t="s">
-        <v>28</v>
+      <c r="F97" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="G97" s="11" t="s">
-        <v>159</v>
+        <v>41</v>
       </c>
       <c r="H97" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="I97" s="11" t="s">
+      <c r="I97" s="13" t="s">
         <v>21</v>
       </c>
       <c r="J97" s="11">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K97" s="11">
         <v>3.0</v>
       </c>
-      <c r="L97" s="11" t="s">
-        <v>30</v>
+      <c r="L97" s="16" t="s">
+        <v>22</v>
       </c>
       <c r="M97" s="11" t="s">
-        <v>162</v>
+        <v>257</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>174</v>
+        <v>258</v>
       </c>
       <c r="O97" s="10"/>
       <c r="P97" s="2"/>
@@ -6771,129 +6734,131 @@
       <c r="AA97" s="2"/>
     </row>
     <row r="98">
-      <c r="A98" s="10" t="s">
+      <c r="A98" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="B98" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C98" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D98" s="10"/>
-      <c r="E98" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="F98" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="G98" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="H98" s="11" t="s">
+      <c r="B98" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C98" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D98" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E98" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F98" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H98" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I98" s="13" t="s">
+      <c r="I98" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="J98" s="11">
+      <c r="J98" s="21">
         <v>2.0</v>
       </c>
-      <c r="K98" s="11">
+      <c r="K98" s="21">
         <v>3.0</v>
       </c>
-      <c r="L98" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="M98" s="11" t="s">
+      <c r="L98" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="M98" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="N98" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="O98" s="2"/>
+      <c r="P98" s="4"/>
+      <c r="Q98" s="4"/>
+      <c r="R98" s="4"/>
+      <c r="S98" s="4"/>
+      <c r="T98" s="4"/>
+      <c r="U98" s="4"/>
+      <c r="V98" s="4"/>
+      <c r="W98" s="4"/>
+      <c r="X98" s="4"/>
+      <c r="Y98" s="4"/>
+      <c r="Z98" s="4"/>
+      <c r="AA98" s="4"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="B99" s="11" t="s">
         <v>260</v>
       </c>
-      <c r="N98" s="10" t="s">
+      <c r="C99" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D99" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E99" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F99" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="G99" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="H99" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="I99" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J99" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="K99" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="L99" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="M99" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="N99" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="O98" s="10"/>
-      <c r="P98" s="2"/>
-      <c r="Q98" s="2"/>
-      <c r="R98" s="2"/>
-      <c r="S98" s="2"/>
-      <c r="T98" s="2"/>
-      <c r="U98" s="2"/>
-      <c r="V98" s="2"/>
-      <c r="W98" s="2"/>
-      <c r="X98" s="2"/>
-      <c r="Y98" s="2"/>
-      <c r="Z98" s="2"/>
-      <c r="AA98" s="2"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="B99" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C99" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="D99" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="E99" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="F99" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G99" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="H99" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I99" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="J99" s="21">
-        <v>2.0</v>
-      </c>
-      <c r="K99" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="L99" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="M99" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="N99" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="O99" s="2"/>
-      <c r="P99" s="4"/>
-      <c r="Q99" s="4"/>
-      <c r="R99" s="4"/>
-      <c r="S99" s="4"/>
-      <c r="T99" s="4"/>
-      <c r="U99" s="4"/>
-      <c r="V99" s="4"/>
-      <c r="W99" s="4"/>
-      <c r="X99" s="4"/>
-      <c r="Y99" s="4"/>
-      <c r="Z99" s="4"/>
-      <c r="AA99" s="4"/>
+      <c r="O99" s="10"/>
+      <c r="P99" s="2"/>
+      <c r="Q99" s="2"/>
+      <c r="R99" s="2"/>
+      <c r="S99" s="2"/>
+      <c r="T99" s="2"/>
+      <c r="U99" s="2"/>
+      <c r="V99" s="2"/>
+      <c r="W99" s="2"/>
+      <c r="X99" s="2"/>
+      <c r="Y99" s="2"/>
+      <c r="Z99" s="2"/>
+      <c r="AA99" s="2"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C100" s="10" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="D100" s="10" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E100" s="14" t="s">
         <v>68</v>
@@ -6923,7 +6888,7 @@
         <v>71</v>
       </c>
       <c r="N100" s="10" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="O100" s="10"/>
       <c r="P100" s="2"/>
@@ -6941,16 +6906,16 @@
     </row>
     <row r="101">
       <c r="A101" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>94</v>
+        <v>58</v>
       </c>
       <c r="D101" s="10" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="E101" s="14" t="s">
         <v>68</v>
@@ -6968,7 +6933,7 @@
         <v>21</v>
       </c>
       <c r="J101" s="11">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="K101" s="11">
         <v>3.0</v>
@@ -6980,7 +6945,7 @@
         <v>71</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>264</v>
+        <v>72</v>
       </c>
       <c r="O101" s="10"/>
       <c r="P101" s="2"/>
@@ -6998,46 +6963,46 @@
     </row>
     <row r="102">
       <c r="A102" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D102" s="10" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E102" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F102" s="14" t="s">
-        <v>69</v>
+        <v>232</v>
       </c>
       <c r="G102" s="11" t="s">
-        <v>70</v>
+        <v>267</v>
       </c>
       <c r="H102" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="I102" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="I102" s="33" t="s">
+        <v>8</v>
       </c>
       <c r="J102" s="11">
         <v>2.0</v>
       </c>
       <c r="K102" s="11">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="L102" s="11" t="s">
         <v>30</v>
       </c>
       <c r="M102" s="11" t="s">
-        <v>71</v>
+        <v>268</v>
       </c>
       <c r="N102" s="10" t="s">
-        <v>72</v>
+        <v>269</v>
       </c>
       <c r="O102" s="10"/>
       <c r="P102" s="2"/>
@@ -7054,49 +7019,49 @@
       <c r="AA102" s="2"/>
     </row>
     <row r="103">
-      <c r="A103" s="10" t="s">
+      <c r="A103" s="37" t="s">
+        <v>270</v>
+      </c>
+      <c r="B103" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="C103" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="D103" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E103" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F103" s="37" t="s">
+        <v>232</v>
+      </c>
+      <c r="G103" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="H103" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="I103" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="J103" s="37">
+        <v>2.0</v>
+      </c>
+      <c r="K103" s="37">
+        <v>2.0</v>
+      </c>
+      <c r="L103" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="M103" s="37" t="s">
         <v>268</v>
       </c>
-      <c r="B103" s="11" t="s">
+      <c r="N103" s="37" t="s">
         <v>269</v>
       </c>
-      <c r="C103" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="D103" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="E103" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F103" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="G103" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="H103" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I103" s="43" t="s">
-        <v>8</v>
-      </c>
-      <c r="J103" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="K103" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="L103" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="M103" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="N103" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="O103" s="10"/>
+      <c r="O103" s="37"/>
       <c r="P103" s="2"/>
       <c r="Q103" s="2"/>
       <c r="R103" s="2"/>
@@ -7111,49 +7076,47 @@
       <c r="AA103" s="2"/>
     </row>
     <row r="104">
-      <c r="A104" s="48" t="s">
-        <v>273</v>
-      </c>
-      <c r="B104" s="48" t="s">
+      <c r="A104" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="C104" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D104" s="10"/>
+      <c r="E104" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F104" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="G104" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I104" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J104" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="K104" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="L104" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="M104" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="N104" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="C104" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="D104" s="48" t="s">
-        <v>94</v>
-      </c>
-      <c r="E104" s="48" t="s">
-        <v>68</v>
-      </c>
-      <c r="F104" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="G104" s="48" t="s">
-        <v>270</v>
-      </c>
-      <c r="H104" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="I104" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="J104" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="K104" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="L104" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="M104" s="48" t="s">
-        <v>271</v>
-      </c>
-      <c r="N104" s="48" t="s">
-        <v>272</v>
-      </c>
-      <c r="O104" s="48"/>
+      <c r="O104" s="10"/>
       <c r="P104" s="2"/>
       <c r="Q104" s="2"/>
       <c r="R104" s="2"/>
@@ -7168,47 +7131,47 @@
       <c r="AA104" s="2"/>
     </row>
     <row r="105">
-      <c r="A105" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="B105" s="11" t="s">
+      <c r="A105" s="37" t="s">
+        <v>272</v>
+      </c>
+      <c r="B105" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="C105" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="D105" s="2"/>
+      <c r="E105" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F105" s="37" t="s">
+        <v>232</v>
+      </c>
+      <c r="G105" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="H105" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="I105" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="J105" s="37">
+        <v>1.0</v>
+      </c>
+      <c r="K105" s="37">
+        <v>2.0</v>
+      </c>
+      <c r="L105" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="M105" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="N105" s="37" t="s">
         <v>269</v>
       </c>
-      <c r="C105" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="D105" s="10"/>
-      <c r="E105" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F105" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="G105" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="H105" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I105" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="J105" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="K105" s="11">
-        <v>3.0</v>
-      </c>
-      <c r="L105" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="M105" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="N105" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="O105" s="10"/>
+      <c r="O105" s="37"/>
       <c r="P105" s="2"/>
       <c r="Q105" s="2"/>
       <c r="R105" s="2"/>
@@ -7223,47 +7186,49 @@
       <c r="AA105" s="2"/>
     </row>
     <row r="106">
-      <c r="A106" s="48" t="s">
-        <v>275</v>
-      </c>
-      <c r="B106" s="48" t="s">
+      <c r="A106" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="B106" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="C106" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D106" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="E106" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F106" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="G106" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="H106" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I106" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J106" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="K106" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="L106" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="M106" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="N106" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="C106" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="D106" s="2"/>
-      <c r="E106" s="48" t="s">
-        <v>68</v>
-      </c>
-      <c r="F106" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="G106" s="48" t="s">
-        <v>270</v>
-      </c>
-      <c r="H106" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="I106" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="J106" s="48">
-        <v>1.0</v>
-      </c>
-      <c r="K106" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="L106" s="48" t="s">
-        <v>22</v>
-      </c>
-      <c r="M106" s="48" t="s">
-        <v>271</v>
-      </c>
-      <c r="N106" s="48" t="s">
-        <v>272</v>
-      </c>
-      <c r="O106" s="48"/>
+      <c r="O106" s="10"/>
       <c r="P106" s="2"/>
       <c r="Q106" s="2"/>
       <c r="R106" s="2"/>
@@ -7279,16 +7244,16 @@
     </row>
     <row r="107">
       <c r="A107" s="10" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="D107" s="10" t="s">
-        <v>222</v>
+        <v>94</v>
       </c>
       <c r="E107" s="14" t="s">
         <v>68</v>
@@ -7297,7 +7262,7 @@
         <v>232</v>
       </c>
       <c r="G107" s="11" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H107" s="11" t="s">
         <v>20</v>
@@ -7306,7 +7271,7 @@
         <v>21</v>
       </c>
       <c r="J107" s="11">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="K107" s="11">
         <v>2.0</v>
@@ -7315,10 +7280,10 @@
         <v>30</v>
       </c>
       <c r="M107" s="11" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="N107" s="10" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="O107" s="10"/>
       <c r="P107" s="2"/>
@@ -7335,49 +7300,47 @@
       <c r="AA107" s="2"/>
     </row>
     <row r="108">
-      <c r="A108" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="B108" s="11" t="s">
+      <c r="A108" s="37" t="s">
+        <v>275</v>
+      </c>
+      <c r="B108" s="37" t="s">
+        <v>266</v>
+      </c>
+      <c r="C108" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="D108" s="2"/>
+      <c r="E108" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F108" s="37" t="s">
+        <v>232</v>
+      </c>
+      <c r="G108" s="37" t="s">
+        <v>267</v>
+      </c>
+      <c r="H108" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="I108" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="J108" s="37">
+        <v>1.0</v>
+      </c>
+      <c r="K108" s="37">
+        <v>2.0</v>
+      </c>
+      <c r="L108" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="M108" s="37" t="s">
+        <v>268</v>
+      </c>
+      <c r="N108" s="37" t="s">
         <v>269</v>
       </c>
-      <c r="C108" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D108" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="E108" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F108" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="G108" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="H108" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I108" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="J108" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="K108" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="L108" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="M108" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="N108" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="O108" s="10"/>
+      <c r="O108" s="37"/>
       <c r="P108" s="2"/>
       <c r="Q108" s="2"/>
       <c r="R108" s="2"/>
@@ -7392,102 +7355,102 @@
       <c r="AA108" s="2"/>
     </row>
     <row r="109">
-      <c r="A109" s="48" t="s">
+      <c r="A109" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D109" s="4"/>
+      <c r="E109" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F109" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G109" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H109" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I109" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="J109" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="K109" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="L109" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M109" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N109" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="O109" s="4"/>
+      <c r="P109" s="4"/>
+      <c r="Q109" s="4"/>
+      <c r="R109" s="4"/>
+      <c r="S109" s="4"/>
+      <c r="T109" s="4"/>
+      <c r="U109" s="4"/>
+      <c r="V109" s="4"/>
+      <c r="W109" s="4"/>
+      <c r="X109" s="4"/>
+      <c r="Y109" s="4"/>
+      <c r="Z109" s="4"/>
+      <c r="AA109" s="4"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="B109" s="48" t="s">
-        <v>269</v>
-      </c>
-      <c r="C109" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="D109" s="2"/>
-      <c r="E109" s="48" t="s">
-        <v>68</v>
-      </c>
-      <c r="F109" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="G109" s="48" t="s">
-        <v>270</v>
-      </c>
-      <c r="H109" s="48" t="s">
+      <c r="B110" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C110" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="2"/>
+      <c r="E110" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F110" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H110" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I109" s="48" t="s">
+      <c r="I110" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J109" s="48">
-        <v>1.0</v>
-      </c>
-      <c r="K109" s="48">
+      <c r="J110" s="21">
         <v>2.0</v>
       </c>
-      <c r="L109" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="M109" s="48" t="s">
-        <v>271</v>
-      </c>
-      <c r="N109" s="48" t="s">
-        <v>272</v>
-      </c>
-      <c r="O109" s="48"/>
-      <c r="P109" s="2"/>
-      <c r="Q109" s="2"/>
-      <c r="R109" s="2"/>
-      <c r="S109" s="2"/>
-      <c r="T109" s="2"/>
-      <c r="U109" s="2"/>
-      <c r="V109" s="2"/>
-      <c r="W109" s="2"/>
-      <c r="X109" s="2"/>
-      <c r="Y109" s="2"/>
-      <c r="Z109" s="2"/>
-      <c r="AA109" s="2"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D110" s="4"/>
-      <c r="E110" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F110" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G110" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H110" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I110" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J110" s="7">
-        <v>2.0</v>
-      </c>
-      <c r="K110" s="7">
-        <v>4.0</v>
-      </c>
-      <c r="L110" s="8" t="s">
+      <c r="K110" s="21">
+        <v>3.0</v>
+      </c>
+      <c r="L110" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="M110" s="4" t="s">
+      <c r="M110" s="2" t="s">
         <v>23</v>
       </c>
       <c r="N110" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="O110" s="4"/>
+      <c r="O110" s="2"/>
       <c r="P110" s="4"/>
       <c r="Q110" s="4"/>
       <c r="R110" s="4"/>
@@ -7501,60 +7464,34 @@
       <c r="Z110" s="4"/>
       <c r="AA110" s="4"/>
     </row>
-    <row r="111">
-      <c r="A111" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="B111" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="C111" s="9" t="s">
-        <v>17</v>
-      </c>
+    <row r="111" ht="15.75" customHeight="1">
+      <c r="A111" s="2"/>
+      <c r="B111" s="2"/>
+      <c r="C111" s="2"/>
       <c r="D111" s="2"/>
-      <c r="E111" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="F111" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="G111" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H111" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I111" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="J111" s="21">
-        <v>2.0</v>
-      </c>
-      <c r="K111" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="L111" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="M111" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N111" s="9" t="s">
-        <v>24</v>
-      </c>
+      <c r="E111" s="2"/>
+      <c r="F111" s="2"/>
+      <c r="G111" s="2"/>
+      <c r="H111" s="2"/>
+      <c r="I111" s="37"/>
+      <c r="J111" s="2"/>
+      <c r="K111" s="2"/>
+      <c r="L111" s="2"/>
+      <c r="M111" s="2"/>
+      <c r="N111" s="2"/>
       <c r="O111" s="2"/>
-      <c r="P111" s="4"/>
-      <c r="Q111" s="4"/>
-      <c r="R111" s="4"/>
-      <c r="S111" s="4"/>
-      <c r="T111" s="4"/>
-      <c r="U111" s="4"/>
-      <c r="V111" s="4"/>
-      <c r="W111" s="4"/>
-      <c r="X111" s="4"/>
-      <c r="Y111" s="4"/>
-      <c r="Z111" s="4"/>
-      <c r="AA111" s="4"/>
+      <c r="P111" s="2"/>
+      <c r="Q111" s="2"/>
+      <c r="R111" s="2"/>
+      <c r="S111" s="2"/>
+      <c r="T111" s="2"/>
+      <c r="U111" s="2"/>
+      <c r="V111" s="2"/>
+      <c r="W111" s="2"/>
+      <c r="X111" s="2"/>
+      <c r="Y111" s="2"/>
+      <c r="Z111" s="2"/>
+      <c r="AA111" s="2"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="2"/>
@@ -7565,7 +7502,7 @@
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
-      <c r="I112" s="48"/>
+      <c r="I112" s="37"/>
       <c r="J112" s="2"/>
       <c r="K112" s="2"/>
       <c r="L112" s="2"/>
@@ -7594,7 +7531,7 @@
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
-      <c r="I113" s="48"/>
+      <c r="I113" s="37"/>
       <c r="J113" s="2"/>
       <c r="K113" s="2"/>
       <c r="L113" s="2"/>
@@ -7623,7 +7560,7 @@
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
-      <c r="I114" s="48"/>
+      <c r="I114" s="37"/>
       <c r="J114" s="2"/>
       <c r="K114" s="2"/>
       <c r="L114" s="2"/>
@@ -7652,7 +7589,7 @@
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
-      <c r="I115" s="48"/>
+      <c r="I115" s="37"/>
       <c r="J115" s="2"/>
       <c r="K115" s="2"/>
       <c r="L115" s="2"/>
@@ -7681,7 +7618,7 @@
       <c r="F116" s="2"/>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
-      <c r="I116" s="48"/>
+      <c r="I116" s="37"/>
       <c r="J116" s="2"/>
       <c r="K116" s="2"/>
       <c r="L116" s="2"/>
@@ -7710,7 +7647,7 @@
       <c r="F117" s="2"/>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
-      <c r="I117" s="48"/>
+      <c r="I117" s="37"/>
       <c r="J117" s="2"/>
       <c r="K117" s="2"/>
       <c r="L117" s="2"/>
@@ -7739,7 +7676,7 @@
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
-      <c r="I118" s="48"/>
+      <c r="I118" s="37"/>
       <c r="J118" s="2"/>
       <c r="K118" s="2"/>
       <c r="L118" s="2"/>
@@ -7768,7 +7705,7 @@
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
-      <c r="I119" s="48"/>
+      <c r="I119" s="37"/>
       <c r="J119" s="2"/>
       <c r="K119" s="2"/>
       <c r="L119" s="2"/>
@@ -7797,7 +7734,7 @@
       <c r="F120" s="2"/>
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
-      <c r="I120" s="48"/>
+      <c r="I120" s="37"/>
       <c r="J120" s="2"/>
       <c r="K120" s="2"/>
       <c r="L120" s="2"/>
@@ -7826,7 +7763,7 @@
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
-      <c r="I121" s="48"/>
+      <c r="I121" s="37"/>
       <c r="J121" s="2"/>
       <c r="K121" s="2"/>
       <c r="L121" s="2"/>
@@ -7855,7 +7792,7 @@
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
-      <c r="I122" s="48"/>
+      <c r="I122" s="37"/>
       <c r="J122" s="2"/>
       <c r="K122" s="2"/>
       <c r="L122" s="2"/>
@@ -7884,7 +7821,7 @@
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
-      <c r="I123" s="48"/>
+      <c r="I123" s="37"/>
       <c r="J123" s="2"/>
       <c r="K123" s="2"/>
       <c r="L123" s="2"/>
@@ -7913,7 +7850,7 @@
       <c r="F124" s="2"/>
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
-      <c r="I124" s="48"/>
+      <c r="I124" s="37"/>
       <c r="J124" s="2"/>
       <c r="K124" s="2"/>
       <c r="L124" s="2"/>
@@ -7942,7 +7879,7 @@
       <c r="F125" s="2"/>
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
-      <c r="I125" s="48"/>
+      <c r="I125" s="37"/>
       <c r="J125" s="2"/>
       <c r="K125" s="2"/>
       <c r="L125" s="2"/>
@@ -7971,7 +7908,7 @@
       <c r="F126" s="2"/>
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
-      <c r="I126" s="48"/>
+      <c r="I126" s="37"/>
       <c r="J126" s="2"/>
       <c r="K126" s="2"/>
       <c r="L126" s="2"/>
@@ -8000,7 +7937,7 @@
       <c r="F127" s="2"/>
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
-      <c r="I127" s="48"/>
+      <c r="I127" s="37"/>
       <c r="J127" s="2"/>
       <c r="K127" s="2"/>
       <c r="L127" s="2"/>
@@ -8029,7 +7966,7 @@
       <c r="F128" s="2"/>
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
-      <c r="I128" s="48"/>
+      <c r="I128" s="37"/>
       <c r="J128" s="2"/>
       <c r="K128" s="2"/>
       <c r="L128" s="2"/>
@@ -8058,7 +7995,7 @@
       <c r="F129" s="2"/>
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
-      <c r="I129" s="48"/>
+      <c r="I129" s="37"/>
       <c r="J129" s="2"/>
       <c r="K129" s="2"/>
       <c r="L129" s="2"/>
@@ -8087,7 +8024,7 @@
       <c r="F130" s="2"/>
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
-      <c r="I130" s="48"/>
+      <c r="I130" s="37"/>
       <c r="J130" s="2"/>
       <c r="K130" s="2"/>
       <c r="L130" s="2"/>
@@ -8116,7 +8053,7 @@
       <c r="F131" s="2"/>
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
-      <c r="I131" s="48"/>
+      <c r="I131" s="37"/>
       <c r="J131" s="2"/>
       <c r="K131" s="2"/>
       <c r="L131" s="2"/>
@@ -8145,7 +8082,7 @@
       <c r="F132" s="2"/>
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
-      <c r="I132" s="48"/>
+      <c r="I132" s="37"/>
       <c r="J132" s="2"/>
       <c r="K132" s="2"/>
       <c r="L132" s="2"/>
@@ -8174,7 +8111,7 @@
       <c r="F133" s="2"/>
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
-      <c r="I133" s="48"/>
+      <c r="I133" s="37"/>
       <c r="J133" s="2"/>
       <c r="K133" s="2"/>
       <c r="L133" s="2"/>
@@ -8203,7 +8140,7 @@
       <c r="F134" s="2"/>
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
-      <c r="I134" s="48"/>
+      <c r="I134" s="37"/>
       <c r="J134" s="2"/>
       <c r="K134" s="2"/>
       <c r="L134" s="2"/>
@@ -8232,7 +8169,7 @@
       <c r="F135" s="2"/>
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
-      <c r="I135" s="48"/>
+      <c r="I135" s="37"/>
       <c r="J135" s="2"/>
       <c r="K135" s="2"/>
       <c r="L135" s="2"/>
@@ -8261,7 +8198,7 @@
       <c r="F136" s="2"/>
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
-      <c r="I136" s="48"/>
+      <c r="I136" s="37"/>
       <c r="J136" s="2"/>
       <c r="K136" s="2"/>
       <c r="L136" s="2"/>
@@ -8290,7 +8227,7 @@
       <c r="F137" s="2"/>
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
-      <c r="I137" s="48"/>
+      <c r="I137" s="37"/>
       <c r="J137" s="2"/>
       <c r="K137" s="2"/>
       <c r="L137" s="2"/>
@@ -8319,7 +8256,7 @@
       <c r="F138" s="2"/>
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
-      <c r="I138" s="48"/>
+      <c r="I138" s="37"/>
       <c r="J138" s="2"/>
       <c r="K138" s="2"/>
       <c r="L138" s="2"/>
@@ -8348,7 +8285,7 @@
       <c r="F139" s="2"/>
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
-      <c r="I139" s="48"/>
+      <c r="I139" s="37"/>
       <c r="J139" s="2"/>
       <c r="K139" s="2"/>
       <c r="L139" s="2"/>
@@ -8377,7 +8314,7 @@
       <c r="F140" s="2"/>
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
-      <c r="I140" s="48"/>
+      <c r="I140" s="37"/>
       <c r="J140" s="2"/>
       <c r="K140" s="2"/>
       <c r="L140" s="2"/>
@@ -8406,7 +8343,7 @@
       <c r="F141" s="2"/>
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
-      <c r="I141" s="48"/>
+      <c r="I141" s="37"/>
       <c r="J141" s="2"/>
       <c r="K141" s="2"/>
       <c r="L141" s="2"/>
@@ -8435,7 +8372,7 @@
       <c r="F142" s="2"/>
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
-      <c r="I142" s="48"/>
+      <c r="I142" s="37"/>
       <c r="J142" s="2"/>
       <c r="K142" s="2"/>
       <c r="L142" s="2"/>
@@ -8464,7 +8401,7 @@
       <c r="F143" s="2"/>
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
-      <c r="I143" s="48"/>
+      <c r="I143" s="37"/>
       <c r="J143" s="2"/>
       <c r="K143" s="2"/>
       <c r="L143" s="2"/>
@@ -8493,7 +8430,7 @@
       <c r="F144" s="2"/>
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
-      <c r="I144" s="48"/>
+      <c r="I144" s="37"/>
       <c r="J144" s="2"/>
       <c r="K144" s="2"/>
       <c r="L144" s="2"/>
@@ -8522,7 +8459,7 @@
       <c r="F145" s="2"/>
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
-      <c r="I145" s="48"/>
+      <c r="I145" s="37"/>
       <c r="J145" s="2"/>
       <c r="K145" s="2"/>
       <c r="L145" s="2"/>
@@ -8551,7 +8488,7 @@
       <c r="F146" s="2"/>
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
-      <c r="I146" s="48"/>
+      <c r="I146" s="37"/>
       <c r="J146" s="2"/>
       <c r="K146" s="2"/>
       <c r="L146" s="2"/>
@@ -8580,7 +8517,7 @@
       <c r="F147" s="2"/>
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
-      <c r="I147" s="48"/>
+      <c r="I147" s="37"/>
       <c r="J147" s="2"/>
       <c r="K147" s="2"/>
       <c r="L147" s="2"/>
@@ -8609,7 +8546,7 @@
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
-      <c r="I148" s="48"/>
+      <c r="I148" s="37"/>
       <c r="J148" s="2"/>
       <c r="K148" s="2"/>
       <c r="L148" s="2"/>
@@ -8638,7 +8575,7 @@
       <c r="F149" s="2"/>
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
-      <c r="I149" s="48"/>
+      <c r="I149" s="37"/>
       <c r="J149" s="2"/>
       <c r="K149" s="2"/>
       <c r="L149" s="2"/>
@@ -8667,7 +8604,7 @@
       <c r="F150" s="2"/>
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
-      <c r="I150" s="48"/>
+      <c r="I150" s="37"/>
       <c r="J150" s="2"/>
       <c r="K150" s="2"/>
       <c r="L150" s="2"/>
@@ -8696,7 +8633,7 @@
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
-      <c r="I151" s="48"/>
+      <c r="I151" s="37"/>
       <c r="J151" s="2"/>
       <c r="K151" s="2"/>
       <c r="L151" s="2"/>
@@ -8725,7 +8662,7 @@
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
-      <c r="I152" s="48"/>
+      <c r="I152" s="37"/>
       <c r="J152" s="2"/>
       <c r="K152" s="2"/>
       <c r="L152" s="2"/>
@@ -8754,7 +8691,7 @@
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
-      <c r="I153" s="48"/>
+      <c r="I153" s="37"/>
       <c r="J153" s="2"/>
       <c r="K153" s="2"/>
       <c r="L153" s="2"/>
@@ -8783,7 +8720,7 @@
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
-      <c r="I154" s="48"/>
+      <c r="I154" s="37"/>
       <c r="J154" s="2"/>
       <c r="K154" s="2"/>
       <c r="L154" s="2"/>
@@ -8812,7 +8749,7 @@
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
-      <c r="I155" s="48"/>
+      <c r="I155" s="37"/>
       <c r="J155" s="2"/>
       <c r="K155" s="2"/>
       <c r="L155" s="2"/>
@@ -8841,7 +8778,7 @@
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
-      <c r="I156" s="48"/>
+      <c r="I156" s="37"/>
       <c r="J156" s="2"/>
       <c r="K156" s="2"/>
       <c r="L156" s="2"/>
@@ -8870,7 +8807,7 @@
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
-      <c r="I157" s="48"/>
+      <c r="I157" s="37"/>
       <c r="J157" s="2"/>
       <c r="K157" s="2"/>
       <c r="L157" s="2"/>
@@ -8899,7 +8836,7 @@
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
-      <c r="I158" s="48"/>
+      <c r="I158" s="37"/>
       <c r="J158" s="2"/>
       <c r="K158" s="2"/>
       <c r="L158" s="2"/>
@@ -8928,7 +8865,7 @@
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
-      <c r="I159" s="48"/>
+      <c r="I159" s="37"/>
       <c r="J159" s="2"/>
       <c r="K159" s="2"/>
       <c r="L159" s="2"/>
@@ -8957,7 +8894,7 @@
       <c r="F160" s="2"/>
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
-      <c r="I160" s="48"/>
+      <c r="I160" s="37"/>
       <c r="J160" s="2"/>
       <c r="K160" s="2"/>
       <c r="L160" s="2"/>
@@ -8986,7 +8923,7 @@
       <c r="F161" s="2"/>
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
-      <c r="I161" s="48"/>
+      <c r="I161" s="37"/>
       <c r="J161" s="2"/>
       <c r="K161" s="2"/>
       <c r="L161" s="2"/>
@@ -9015,7 +8952,7 @@
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
-      <c r="I162" s="48"/>
+      <c r="I162" s="37"/>
       <c r="J162" s="2"/>
       <c r="K162" s="2"/>
       <c r="L162" s="2"/>
@@ -9044,7 +8981,7 @@
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
-      <c r="I163" s="48"/>
+      <c r="I163" s="37"/>
       <c r="J163" s="2"/>
       <c r="K163" s="2"/>
       <c r="L163" s="2"/>
@@ -9073,7 +9010,7 @@
       <c r="F164" s="2"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
-      <c r="I164" s="48"/>
+      <c r="I164" s="37"/>
       <c r="J164" s="2"/>
       <c r="K164" s="2"/>
       <c r="L164" s="2"/>
@@ -9102,7 +9039,7 @@
       <c r="F165" s="2"/>
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
-      <c r="I165" s="48"/>
+      <c r="I165" s="37"/>
       <c r="J165" s="2"/>
       <c r="K165" s="2"/>
       <c r="L165" s="2"/>
@@ -9131,7 +9068,7 @@
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
-      <c r="I166" s="48"/>
+      <c r="I166" s="37"/>
       <c r="J166" s="2"/>
       <c r="K166" s="2"/>
       <c r="L166" s="2"/>
@@ -9160,7 +9097,7 @@
       <c r="F167" s="2"/>
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
-      <c r="I167" s="48"/>
+      <c r="I167" s="37"/>
       <c r="J167" s="2"/>
       <c r="K167" s="2"/>
       <c r="L167" s="2"/>
@@ -9189,7 +9126,7 @@
       <c r="F168" s="2"/>
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
-      <c r="I168" s="48"/>
+      <c r="I168" s="37"/>
       <c r="J168" s="2"/>
       <c r="K168" s="2"/>
       <c r="L168" s="2"/>
@@ -9218,7 +9155,7 @@
       <c r="F169" s="2"/>
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
-      <c r="I169" s="48"/>
+      <c r="I169" s="37"/>
       <c r="J169" s="2"/>
       <c r="K169" s="2"/>
       <c r="L169" s="2"/>
@@ -9247,7 +9184,7 @@
       <c r="F170" s="2"/>
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
-      <c r="I170" s="48"/>
+      <c r="I170" s="37"/>
       <c r="J170" s="2"/>
       <c r="K170" s="2"/>
       <c r="L170" s="2"/>
@@ -9276,7 +9213,7 @@
       <c r="F171" s="2"/>
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
-      <c r="I171" s="48"/>
+      <c r="I171" s="37"/>
       <c r="J171" s="2"/>
       <c r="K171" s="2"/>
       <c r="L171" s="2"/>
@@ -9305,7 +9242,7 @@
       <c r="F172" s="2"/>
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
-      <c r="I172" s="48"/>
+      <c r="I172" s="37"/>
       <c r="J172" s="2"/>
       <c r="K172" s="2"/>
       <c r="L172" s="2"/>
@@ -9334,7 +9271,7 @@
       <c r="F173" s="2"/>
       <c r="G173" s="2"/>
       <c r="H173" s="2"/>
-      <c r="I173" s="48"/>
+      <c r="I173" s="37"/>
       <c r="J173" s="2"/>
       <c r="K173" s="2"/>
       <c r="L173" s="2"/>
@@ -9363,7 +9300,7 @@
       <c r="F174" s="2"/>
       <c r="G174" s="2"/>
       <c r="H174" s="2"/>
-      <c r="I174" s="48"/>
+      <c r="I174" s="37"/>
       <c r="J174" s="2"/>
       <c r="K174" s="2"/>
       <c r="L174" s="2"/>
@@ -9392,7 +9329,7 @@
       <c r="F175" s="2"/>
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
-      <c r="I175" s="48"/>
+      <c r="I175" s="37"/>
       <c r="J175" s="2"/>
       <c r="K175" s="2"/>
       <c r="L175" s="2"/>
@@ -9421,7 +9358,7 @@
       <c r="F176" s="2"/>
       <c r="G176" s="2"/>
       <c r="H176" s="2"/>
-      <c r="I176" s="48"/>
+      <c r="I176" s="37"/>
       <c r="J176" s="2"/>
       <c r="K176" s="2"/>
       <c r="L176" s="2"/>
@@ -9450,7 +9387,7 @@
       <c r="F177" s="2"/>
       <c r="G177" s="2"/>
       <c r="H177" s="2"/>
-      <c r="I177" s="48"/>
+      <c r="I177" s="37"/>
       <c r="J177" s="2"/>
       <c r="K177" s="2"/>
       <c r="L177" s="2"/>
@@ -9479,7 +9416,7 @@
       <c r="F178" s="2"/>
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
-      <c r="I178" s="48"/>
+      <c r="I178" s="37"/>
       <c r="J178" s="2"/>
       <c r="K178" s="2"/>
       <c r="L178" s="2"/>
@@ -9508,7 +9445,7 @@
       <c r="F179" s="2"/>
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
-      <c r="I179" s="48"/>
+      <c r="I179" s="37"/>
       <c r="J179" s="2"/>
       <c r="K179" s="2"/>
       <c r="L179" s="2"/>
@@ -9537,7 +9474,7 @@
       <c r="F180" s="2"/>
       <c r="G180" s="2"/>
       <c r="H180" s="2"/>
-      <c r="I180" s="48"/>
+      <c r="I180" s="37"/>
       <c r="J180" s="2"/>
       <c r="K180" s="2"/>
       <c r="L180" s="2"/>
@@ -9566,7 +9503,7 @@
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
-      <c r="I181" s="48"/>
+      <c r="I181" s="37"/>
       <c r="J181" s="2"/>
       <c r="K181" s="2"/>
       <c r="L181" s="2"/>
@@ -9595,7 +9532,7 @@
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
-      <c r="I182" s="48"/>
+      <c r="I182" s="37"/>
       <c r="J182" s="2"/>
       <c r="K182" s="2"/>
       <c r="L182" s="2"/>
@@ -9624,7 +9561,7 @@
       <c r="F183" s="2"/>
       <c r="G183" s="2"/>
       <c r="H183" s="2"/>
-      <c r="I183" s="48"/>
+      <c r="I183" s="37"/>
       <c r="J183" s="2"/>
       <c r="K183" s="2"/>
       <c r="L183" s="2"/>
@@ -9653,7 +9590,7 @@
       <c r="F184" s="2"/>
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
-      <c r="I184" s="48"/>
+      <c r="I184" s="37"/>
       <c r="J184" s="2"/>
       <c r="K184" s="2"/>
       <c r="L184" s="2"/>
@@ -9682,7 +9619,7 @@
       <c r="F185" s="2"/>
       <c r="G185" s="2"/>
       <c r="H185" s="2"/>
-      <c r="I185" s="48"/>
+      <c r="I185" s="37"/>
       <c r="J185" s="2"/>
       <c r="K185" s="2"/>
       <c r="L185" s="2"/>
@@ -9711,7 +9648,7 @@
       <c r="F186" s="2"/>
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
-      <c r="I186" s="48"/>
+      <c r="I186" s="37"/>
       <c r="J186" s="2"/>
       <c r="K186" s="2"/>
       <c r="L186" s="2"/>
@@ -9740,7 +9677,7 @@
       <c r="F187" s="2"/>
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
-      <c r="I187" s="48"/>
+      <c r="I187" s="37"/>
       <c r="J187" s="2"/>
       <c r="K187" s="2"/>
       <c r="L187" s="2"/>
@@ -9769,7 +9706,7 @@
       <c r="F188" s="2"/>
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
-      <c r="I188" s="48"/>
+      <c r="I188" s="37"/>
       <c r="J188" s="2"/>
       <c r="K188" s="2"/>
       <c r="L188" s="2"/>
@@ -9798,7 +9735,7 @@
       <c r="F189" s="2"/>
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
-      <c r="I189" s="48"/>
+      <c r="I189" s="37"/>
       <c r="J189" s="2"/>
       <c r="K189" s="2"/>
       <c r="L189" s="2"/>
@@ -9827,7 +9764,7 @@
       <c r="F190" s="2"/>
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
-      <c r="I190" s="48"/>
+      <c r="I190" s="37"/>
       <c r="J190" s="2"/>
       <c r="K190" s="2"/>
       <c r="L190" s="2"/>
@@ -9856,7 +9793,7 @@
       <c r="F191" s="2"/>
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
-      <c r="I191" s="48"/>
+      <c r="I191" s="37"/>
       <c r="J191" s="2"/>
       <c r="K191" s="2"/>
       <c r="L191" s="2"/>
@@ -9885,7 +9822,7 @@
       <c r="F192" s="2"/>
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
-      <c r="I192" s="48"/>
+      <c r="I192" s="37"/>
       <c r="J192" s="2"/>
       <c r="K192" s="2"/>
       <c r="L192" s="2"/>
@@ -9914,7 +9851,7 @@
       <c r="F193" s="2"/>
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
-      <c r="I193" s="48"/>
+      <c r="I193" s="37"/>
       <c r="J193" s="2"/>
       <c r="K193" s="2"/>
       <c r="L193" s="2"/>
@@ -9943,7 +9880,7 @@
       <c r="F194" s="2"/>
       <c r="G194" s="2"/>
       <c r="H194" s="2"/>
-      <c r="I194" s="48"/>
+      <c r="I194" s="37"/>
       <c r="J194" s="2"/>
       <c r="K194" s="2"/>
       <c r="L194" s="2"/>
@@ -9972,7 +9909,7 @@
       <c r="F195" s="2"/>
       <c r="G195" s="2"/>
       <c r="H195" s="2"/>
-      <c r="I195" s="48"/>
+      <c r="I195" s="37"/>
       <c r="J195" s="2"/>
       <c r="K195" s="2"/>
       <c r="L195" s="2"/>
@@ -10001,7 +9938,7 @@
       <c r="F196" s="2"/>
       <c r="G196" s="2"/>
       <c r="H196" s="2"/>
-      <c r="I196" s="48"/>
+      <c r="I196" s="37"/>
       <c r="J196" s="2"/>
       <c r="K196" s="2"/>
       <c r="L196" s="2"/>
@@ -10030,7 +9967,7 @@
       <c r="F197" s="2"/>
       <c r="G197" s="2"/>
       <c r="H197" s="2"/>
-      <c r="I197" s="48"/>
+      <c r="I197" s="37"/>
       <c r="J197" s="2"/>
       <c r="K197" s="2"/>
       <c r="L197" s="2"/>
@@ -10059,7 +9996,7 @@
       <c r="F198" s="2"/>
       <c r="G198" s="2"/>
       <c r="H198" s="2"/>
-      <c r="I198" s="48"/>
+      <c r="I198" s="37"/>
       <c r="J198" s="2"/>
       <c r="K198" s="2"/>
       <c r="L198" s="2"/>
@@ -10088,7 +10025,7 @@
       <c r="F199" s="2"/>
       <c r="G199" s="2"/>
       <c r="H199" s="2"/>
-      <c r="I199" s="48"/>
+      <c r="I199" s="37"/>
       <c r="J199" s="2"/>
       <c r="K199" s="2"/>
       <c r="L199" s="2"/>
@@ -10117,7 +10054,7 @@
       <c r="F200" s="2"/>
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
-      <c r="I200" s="48"/>
+      <c r="I200" s="37"/>
       <c r="J200" s="2"/>
       <c r="K200" s="2"/>
       <c r="L200" s="2"/>
@@ -10146,7 +10083,7 @@
       <c r="F201" s="2"/>
       <c r="G201" s="2"/>
       <c r="H201" s="2"/>
-      <c r="I201" s="48"/>
+      <c r="I201" s="37"/>
       <c r="J201" s="2"/>
       <c r="K201" s="2"/>
       <c r="L201" s="2"/>
@@ -10175,7 +10112,7 @@
       <c r="F202" s="2"/>
       <c r="G202" s="2"/>
       <c r="H202" s="2"/>
-      <c r="I202" s="48"/>
+      <c r="I202" s="37"/>
       <c r="J202" s="2"/>
       <c r="K202" s="2"/>
       <c r="L202" s="2"/>
@@ -10204,7 +10141,7 @@
       <c r="F203" s="2"/>
       <c r="G203" s="2"/>
       <c r="H203" s="2"/>
-      <c r="I203" s="48"/>
+      <c r="I203" s="37"/>
       <c r="J203" s="2"/>
       <c r="K203" s="2"/>
       <c r="L203" s="2"/>
@@ -10233,7 +10170,7 @@
       <c r="F204" s="2"/>
       <c r="G204" s="2"/>
       <c r="H204" s="2"/>
-      <c r="I204" s="48"/>
+      <c r="I204" s="37"/>
       <c r="J204" s="2"/>
       <c r="K204" s="2"/>
       <c r="L204" s="2"/>
@@ -10262,7 +10199,7 @@
       <c r="F205" s="2"/>
       <c r="G205" s="2"/>
       <c r="H205" s="2"/>
-      <c r="I205" s="48"/>
+      <c r="I205" s="37"/>
       <c r="J205" s="2"/>
       <c r="K205" s="2"/>
       <c r="L205" s="2"/>
@@ -10291,7 +10228,7 @@
       <c r="F206" s="2"/>
       <c r="G206" s="2"/>
       <c r="H206" s="2"/>
-      <c r="I206" s="48"/>
+      <c r="I206" s="37"/>
       <c r="J206" s="2"/>
       <c r="K206" s="2"/>
       <c r="L206" s="2"/>
@@ -10320,7 +10257,7 @@
       <c r="F207" s="2"/>
       <c r="G207" s="2"/>
       <c r="H207" s="2"/>
-      <c r="I207" s="48"/>
+      <c r="I207" s="37"/>
       <c r="J207" s="2"/>
       <c r="K207" s="2"/>
       <c r="L207" s="2"/>
@@ -10349,7 +10286,7 @@
       <c r="F208" s="2"/>
       <c r="G208" s="2"/>
       <c r="H208" s="2"/>
-      <c r="I208" s="48"/>
+      <c r="I208" s="37"/>
       <c r="J208" s="2"/>
       <c r="K208" s="2"/>
       <c r="L208" s="2"/>
@@ -10378,7 +10315,7 @@
       <c r="F209" s="2"/>
       <c r="G209" s="2"/>
       <c r="H209" s="2"/>
-      <c r="I209" s="48"/>
+      <c r="I209" s="37"/>
       <c r="J209" s="2"/>
       <c r="K209" s="2"/>
       <c r="L209" s="2"/>
@@ -10407,7 +10344,7 @@
       <c r="F210" s="2"/>
       <c r="G210" s="2"/>
       <c r="H210" s="2"/>
-      <c r="I210" s="48"/>
+      <c r="I210" s="37"/>
       <c r="J210" s="2"/>
       <c r="K210" s="2"/>
       <c r="L210" s="2"/>
@@ -10436,7 +10373,7 @@
       <c r="F211" s="2"/>
       <c r="G211" s="2"/>
       <c r="H211" s="2"/>
-      <c r="I211" s="48"/>
+      <c r="I211" s="37"/>
       <c r="J211" s="2"/>
       <c r="K211" s="2"/>
       <c r="L211" s="2"/>
@@ -10465,7 +10402,7 @@
       <c r="F212" s="2"/>
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
-      <c r="I212" s="48"/>
+      <c r="I212" s="37"/>
       <c r="J212" s="2"/>
       <c r="K212" s="2"/>
       <c r="L212" s="2"/>
@@ -10494,7 +10431,7 @@
       <c r="F213" s="2"/>
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
-      <c r="I213" s="48"/>
+      <c r="I213" s="37"/>
       <c r="J213" s="2"/>
       <c r="K213" s="2"/>
       <c r="L213" s="2"/>
@@ -10523,7 +10460,7 @@
       <c r="F214" s="2"/>
       <c r="G214" s="2"/>
       <c r="H214" s="2"/>
-      <c r="I214" s="48"/>
+      <c r="I214" s="37"/>
       <c r="J214" s="2"/>
       <c r="K214" s="2"/>
       <c r="L214" s="2"/>
@@ -10552,7 +10489,7 @@
       <c r="F215" s="2"/>
       <c r="G215" s="2"/>
       <c r="H215" s="2"/>
-      <c r="I215" s="48"/>
+      <c r="I215" s="37"/>
       <c r="J215" s="2"/>
       <c r="K215" s="2"/>
       <c r="L215" s="2"/>
@@ -10581,7 +10518,7 @@
       <c r="F216" s="2"/>
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
-      <c r="I216" s="48"/>
+      <c r="I216" s="37"/>
       <c r="J216" s="2"/>
       <c r="K216" s="2"/>
       <c r="L216" s="2"/>
@@ -10610,7 +10547,7 @@
       <c r="F217" s="2"/>
       <c r="G217" s="2"/>
       <c r="H217" s="2"/>
-      <c r="I217" s="48"/>
+      <c r="I217" s="37"/>
       <c r="J217" s="2"/>
       <c r="K217" s="2"/>
       <c r="L217" s="2"/>
@@ -10639,7 +10576,7 @@
       <c r="F218" s="2"/>
       <c r="G218" s="2"/>
       <c r="H218" s="2"/>
-      <c r="I218" s="48"/>
+      <c r="I218" s="37"/>
       <c r="J218" s="2"/>
       <c r="K218" s="2"/>
       <c r="L218" s="2"/>
@@ -10668,7 +10605,7 @@
       <c r="F219" s="2"/>
       <c r="G219" s="2"/>
       <c r="H219" s="2"/>
-      <c r="I219" s="48"/>
+      <c r="I219" s="37"/>
       <c r="J219" s="2"/>
       <c r="K219" s="2"/>
       <c r="L219" s="2"/>
@@ -10697,7 +10634,7 @@
       <c r="F220" s="2"/>
       <c r="G220" s="2"/>
       <c r="H220" s="2"/>
-      <c r="I220" s="48"/>
+      <c r="I220" s="37"/>
       <c r="J220" s="2"/>
       <c r="K220" s="2"/>
       <c r="L220" s="2"/>
@@ -10726,7 +10663,7 @@
       <c r="F221" s="2"/>
       <c r="G221" s="2"/>
       <c r="H221" s="2"/>
-      <c r="I221" s="48"/>
+      <c r="I221" s="37"/>
       <c r="J221" s="2"/>
       <c r="K221" s="2"/>
       <c r="L221" s="2"/>
@@ -10755,7 +10692,7 @@
       <c r="F222" s="2"/>
       <c r="G222" s="2"/>
       <c r="H222" s="2"/>
-      <c r="I222" s="48"/>
+      <c r="I222" s="37"/>
       <c r="J222" s="2"/>
       <c r="K222" s="2"/>
       <c r="L222" s="2"/>
@@ -10784,7 +10721,7 @@
       <c r="F223" s="2"/>
       <c r="G223" s="2"/>
       <c r="H223" s="2"/>
-      <c r="I223" s="48"/>
+      <c r="I223" s="37"/>
       <c r="J223" s="2"/>
       <c r="K223" s="2"/>
       <c r="L223" s="2"/>
@@ -10813,7 +10750,7 @@
       <c r="F224" s="2"/>
       <c r="G224" s="2"/>
       <c r="H224" s="2"/>
-      <c r="I224" s="48"/>
+      <c r="I224" s="37"/>
       <c r="J224" s="2"/>
       <c r="K224" s="2"/>
       <c r="L224" s="2"/>
@@ -10842,7 +10779,7 @@
       <c r="F225" s="2"/>
       <c r="G225" s="2"/>
       <c r="H225" s="2"/>
-      <c r="I225" s="48"/>
+      <c r="I225" s="37"/>
       <c r="J225" s="2"/>
       <c r="K225" s="2"/>
       <c r="L225" s="2"/>
@@ -10871,7 +10808,7 @@
       <c r="F226" s="2"/>
       <c r="G226" s="2"/>
       <c r="H226" s="2"/>
-      <c r="I226" s="48"/>
+      <c r="I226" s="37"/>
       <c r="J226" s="2"/>
       <c r="K226" s="2"/>
       <c r="L226" s="2"/>
@@ -10900,7 +10837,7 @@
       <c r="F227" s="2"/>
       <c r="G227" s="2"/>
       <c r="H227" s="2"/>
-      <c r="I227" s="48"/>
+      <c r="I227" s="37"/>
       <c r="J227" s="2"/>
       <c r="K227" s="2"/>
       <c r="L227" s="2"/>
@@ -10929,7 +10866,7 @@
       <c r="F228" s="2"/>
       <c r="G228" s="2"/>
       <c r="H228" s="2"/>
-      <c r="I228" s="48"/>
+      <c r="I228" s="37"/>
       <c r="J228" s="2"/>
       <c r="K228" s="2"/>
       <c r="L228" s="2"/>
@@ -10958,7 +10895,7 @@
       <c r="F229" s="2"/>
       <c r="G229" s="2"/>
       <c r="H229" s="2"/>
-      <c r="I229" s="48"/>
+      <c r="I229" s="37"/>
       <c r="J229" s="2"/>
       <c r="K229" s="2"/>
       <c r="L229" s="2"/>
@@ -10987,7 +10924,7 @@
       <c r="F230" s="2"/>
       <c r="G230" s="2"/>
       <c r="H230" s="2"/>
-      <c r="I230" s="48"/>
+      <c r="I230" s="37"/>
       <c r="J230" s="2"/>
       <c r="K230" s="2"/>
       <c r="L230" s="2"/>
@@ -11016,7 +10953,7 @@
       <c r="F231" s="2"/>
       <c r="G231" s="2"/>
       <c r="H231" s="2"/>
-      <c r="I231" s="48"/>
+      <c r="I231" s="37"/>
       <c r="J231" s="2"/>
       <c r="K231" s="2"/>
       <c r="L231" s="2"/>
@@ -11045,7 +10982,7 @@
       <c r="F232" s="2"/>
       <c r="G232" s="2"/>
       <c r="H232" s="2"/>
-      <c r="I232" s="48"/>
+      <c r="I232" s="37"/>
       <c r="J232" s="2"/>
       <c r="K232" s="2"/>
       <c r="L232" s="2"/>
@@ -11074,7 +11011,7 @@
       <c r="F233" s="2"/>
       <c r="G233" s="2"/>
       <c r="H233" s="2"/>
-      <c r="I233" s="48"/>
+      <c r="I233" s="37"/>
       <c r="J233" s="2"/>
       <c r="K233" s="2"/>
       <c r="L233" s="2"/>
@@ -11103,7 +11040,7 @@
       <c r="F234" s="2"/>
       <c r="G234" s="2"/>
       <c r="H234" s="2"/>
-      <c r="I234" s="48"/>
+      <c r="I234" s="37"/>
       <c r="J234" s="2"/>
       <c r="K234" s="2"/>
       <c r="L234" s="2"/>
@@ -11132,7 +11069,7 @@
       <c r="F235" s="2"/>
       <c r="G235" s="2"/>
       <c r="H235" s="2"/>
-      <c r="I235" s="48"/>
+      <c r="I235" s="37"/>
       <c r="J235" s="2"/>
       <c r="K235" s="2"/>
       <c r="L235" s="2"/>
@@ -11161,7 +11098,7 @@
       <c r="F236" s="2"/>
       <c r="G236" s="2"/>
       <c r="H236" s="2"/>
-      <c r="I236" s="48"/>
+      <c r="I236" s="37"/>
       <c r="J236" s="2"/>
       <c r="K236" s="2"/>
       <c r="L236" s="2"/>
@@ -11190,7 +11127,7 @@
       <c r="F237" s="2"/>
       <c r="G237" s="2"/>
       <c r="H237" s="2"/>
-      <c r="I237" s="48"/>
+      <c r="I237" s="37"/>
       <c r="J237" s="2"/>
       <c r="K237" s="2"/>
       <c r="L237" s="2"/>
@@ -11219,7 +11156,7 @@
       <c r="F238" s="2"/>
       <c r="G238" s="2"/>
       <c r="H238" s="2"/>
-      <c r="I238" s="48"/>
+      <c r="I238" s="37"/>
       <c r="J238" s="2"/>
       <c r="K238" s="2"/>
       <c r="L238" s="2"/>
@@ -11248,7 +11185,7 @@
       <c r="F239" s="2"/>
       <c r="G239" s="2"/>
       <c r="H239" s="2"/>
-      <c r="I239" s="48"/>
+      <c r="I239" s="37"/>
       <c r="J239" s="2"/>
       <c r="K239" s="2"/>
       <c r="L239" s="2"/>
@@ -11277,7 +11214,7 @@
       <c r="F240" s="2"/>
       <c r="G240" s="2"/>
       <c r="H240" s="2"/>
-      <c r="I240" s="48"/>
+      <c r="I240" s="37"/>
       <c r="J240" s="2"/>
       <c r="K240" s="2"/>
       <c r="L240" s="2"/>
@@ -11306,7 +11243,7 @@
       <c r="F241" s="2"/>
       <c r="G241" s="2"/>
       <c r="H241" s="2"/>
-      <c r="I241" s="48"/>
+      <c r="I241" s="37"/>
       <c r="J241" s="2"/>
       <c r="K241" s="2"/>
       <c r="L241" s="2"/>
@@ -11335,7 +11272,7 @@
       <c r="F242" s="2"/>
       <c r="G242" s="2"/>
       <c r="H242" s="2"/>
-      <c r="I242" s="48"/>
+      <c r="I242" s="37"/>
       <c r="J242" s="2"/>
       <c r="K242" s="2"/>
       <c r="L242" s="2"/>
@@ -11364,7 +11301,7 @@
       <c r="F243" s="2"/>
       <c r="G243" s="2"/>
       <c r="H243" s="2"/>
-      <c r="I243" s="48"/>
+      <c r="I243" s="37"/>
       <c r="J243" s="2"/>
       <c r="K243" s="2"/>
       <c r="L243" s="2"/>
@@ -11393,7 +11330,7 @@
       <c r="F244" s="2"/>
       <c r="G244" s="2"/>
       <c r="H244" s="2"/>
-      <c r="I244" s="48"/>
+      <c r="I244" s="37"/>
       <c r="J244" s="2"/>
       <c r="K244" s="2"/>
       <c r="L244" s="2"/>
@@ -11422,7 +11359,7 @@
       <c r="F245" s="2"/>
       <c r="G245" s="2"/>
       <c r="H245" s="2"/>
-      <c r="I245" s="48"/>
+      <c r="I245" s="37"/>
       <c r="J245" s="2"/>
       <c r="K245" s="2"/>
       <c r="L245" s="2"/>
@@ -11451,7 +11388,7 @@
       <c r="F246" s="2"/>
       <c r="G246" s="2"/>
       <c r="H246" s="2"/>
-      <c r="I246" s="48"/>
+      <c r="I246" s="37"/>
       <c r="J246" s="2"/>
       <c r="K246" s="2"/>
       <c r="L246" s="2"/>
@@ -11480,7 +11417,7 @@
       <c r="F247" s="2"/>
       <c r="G247" s="2"/>
       <c r="H247" s="2"/>
-      <c r="I247" s="48"/>
+      <c r="I247" s="37"/>
       <c r="J247" s="2"/>
       <c r="K247" s="2"/>
       <c r="L247" s="2"/>
@@ -11509,7 +11446,7 @@
       <c r="F248" s="2"/>
       <c r="G248" s="2"/>
       <c r="H248" s="2"/>
-      <c r="I248" s="48"/>
+      <c r="I248" s="37"/>
       <c r="J248" s="2"/>
       <c r="K248" s="2"/>
       <c r="L248" s="2"/>
@@ -11538,7 +11475,7 @@
       <c r="F249" s="2"/>
       <c r="G249" s="2"/>
       <c r="H249" s="2"/>
-      <c r="I249" s="48"/>
+      <c r="I249" s="37"/>
       <c r="J249" s="2"/>
       <c r="K249" s="2"/>
       <c r="L249" s="2"/>
@@ -11567,7 +11504,7 @@
       <c r="F250" s="2"/>
       <c r="G250" s="2"/>
       <c r="H250" s="2"/>
-      <c r="I250" s="48"/>
+      <c r="I250" s="37"/>
       <c r="J250" s="2"/>
       <c r="K250" s="2"/>
       <c r="L250" s="2"/>
@@ -11596,7 +11533,7 @@
       <c r="F251" s="2"/>
       <c r="G251" s="2"/>
       <c r="H251" s="2"/>
-      <c r="I251" s="48"/>
+      <c r="I251" s="37"/>
       <c r="J251" s="2"/>
       <c r="K251" s="2"/>
       <c r="L251" s="2"/>
@@ -11625,7 +11562,7 @@
       <c r="F252" s="2"/>
       <c r="G252" s="2"/>
       <c r="H252" s="2"/>
-      <c r="I252" s="48"/>
+      <c r="I252" s="37"/>
       <c r="J252" s="2"/>
       <c r="K252" s="2"/>
       <c r="L252" s="2"/>
@@ -11654,7 +11591,7 @@
       <c r="F253" s="2"/>
       <c r="G253" s="2"/>
       <c r="H253" s="2"/>
-      <c r="I253" s="48"/>
+      <c r="I253" s="37"/>
       <c r="J253" s="2"/>
       <c r="K253" s="2"/>
       <c r="L253" s="2"/>
@@ -11683,7 +11620,7 @@
       <c r="F254" s="2"/>
       <c r="G254" s="2"/>
       <c r="H254" s="2"/>
-      <c r="I254" s="48"/>
+      <c r="I254" s="37"/>
       <c r="J254" s="2"/>
       <c r="K254" s="2"/>
       <c r="L254" s="2"/>
@@ -11712,7 +11649,7 @@
       <c r="F255" s="2"/>
       <c r="G255" s="2"/>
       <c r="H255" s="2"/>
-      <c r="I255" s="48"/>
+      <c r="I255" s="37"/>
       <c r="J255" s="2"/>
       <c r="K255" s="2"/>
       <c r="L255" s="2"/>
@@ -11741,7 +11678,7 @@
       <c r="F256" s="2"/>
       <c r="G256" s="2"/>
       <c r="H256" s="2"/>
-      <c r="I256" s="48"/>
+      <c r="I256" s="37"/>
       <c r="J256" s="2"/>
       <c r="K256" s="2"/>
       <c r="L256" s="2"/>
@@ -11770,7 +11707,7 @@
       <c r="F257" s="2"/>
       <c r="G257" s="2"/>
       <c r="H257" s="2"/>
-      <c r="I257" s="48"/>
+      <c r="I257" s="37"/>
       <c r="J257" s="2"/>
       <c r="K257" s="2"/>
       <c r="L257" s="2"/>
@@ -11799,7 +11736,7 @@
       <c r="F258" s="2"/>
       <c r="G258" s="2"/>
       <c r="H258" s="2"/>
-      <c r="I258" s="48"/>
+      <c r="I258" s="37"/>
       <c r="J258" s="2"/>
       <c r="K258" s="2"/>
       <c r="L258" s="2"/>
@@ -11828,7 +11765,7 @@
       <c r="F259" s="2"/>
       <c r="G259" s="2"/>
       <c r="H259" s="2"/>
-      <c r="I259" s="48"/>
+      <c r="I259" s="37"/>
       <c r="J259" s="2"/>
       <c r="K259" s="2"/>
       <c r="L259" s="2"/>
@@ -11857,7 +11794,7 @@
       <c r="F260" s="2"/>
       <c r="G260" s="2"/>
       <c r="H260" s="2"/>
-      <c r="I260" s="48"/>
+      <c r="I260" s="37"/>
       <c r="J260" s="2"/>
       <c r="K260" s="2"/>
       <c r="L260" s="2"/>
@@ -11886,7 +11823,7 @@
       <c r="F261" s="2"/>
       <c r="G261" s="2"/>
       <c r="H261" s="2"/>
-      <c r="I261" s="48"/>
+      <c r="I261" s="37"/>
       <c r="J261" s="2"/>
       <c r="K261" s="2"/>
       <c r="L261" s="2"/>
@@ -11915,7 +11852,7 @@
       <c r="F262" s="2"/>
       <c r="G262" s="2"/>
       <c r="H262" s="2"/>
-      <c r="I262" s="48"/>
+      <c r="I262" s="37"/>
       <c r="J262" s="2"/>
       <c r="K262" s="2"/>
       <c r="L262" s="2"/>
@@ -11944,7 +11881,7 @@
       <c r="F263" s="2"/>
       <c r="G263" s="2"/>
       <c r="H263" s="2"/>
-      <c r="I263" s="48"/>
+      <c r="I263" s="37"/>
       <c r="J263" s="2"/>
       <c r="K263" s="2"/>
       <c r="L263" s="2"/>
@@ -11973,7 +11910,7 @@
       <c r="F264" s="2"/>
       <c r="G264" s="2"/>
       <c r="H264" s="2"/>
-      <c r="I264" s="48"/>
+      <c r="I264" s="37"/>
       <c r="J264" s="2"/>
       <c r="K264" s="2"/>
       <c r="L264" s="2"/>
@@ -12002,7 +11939,7 @@
       <c r="F265" s="2"/>
       <c r="G265" s="2"/>
       <c r="H265" s="2"/>
-      <c r="I265" s="48"/>
+      <c r="I265" s="37"/>
       <c r="J265" s="2"/>
       <c r="K265" s="2"/>
       <c r="L265" s="2"/>
@@ -12031,7 +11968,7 @@
       <c r="F266" s="2"/>
       <c r="G266" s="2"/>
       <c r="H266" s="2"/>
-      <c r="I266" s="48"/>
+      <c r="I266" s="37"/>
       <c r="J266" s="2"/>
       <c r="K266" s="2"/>
       <c r="L266" s="2"/>
@@ -12060,7 +11997,7 @@
       <c r="F267" s="2"/>
       <c r="G267" s="2"/>
       <c r="H267" s="2"/>
-      <c r="I267" s="48"/>
+      <c r="I267" s="37"/>
       <c r="J267" s="2"/>
       <c r="K267" s="2"/>
       <c r="L267" s="2"/>
@@ -12089,7 +12026,7 @@
       <c r="F268" s="2"/>
       <c r="G268" s="2"/>
       <c r="H268" s="2"/>
-      <c r="I268" s="48"/>
+      <c r="I268" s="37"/>
       <c r="J268" s="2"/>
       <c r="K268" s="2"/>
       <c r="L268" s="2"/>
@@ -12118,7 +12055,7 @@
       <c r="F269" s="2"/>
       <c r="G269" s="2"/>
       <c r="H269" s="2"/>
-      <c r="I269" s="48"/>
+      <c r="I269" s="37"/>
       <c r="J269" s="2"/>
       <c r="K269" s="2"/>
       <c r="L269" s="2"/>
@@ -12147,7 +12084,7 @@
       <c r="F270" s="2"/>
       <c r="G270" s="2"/>
       <c r="H270" s="2"/>
-      <c r="I270" s="48"/>
+      <c r="I270" s="37"/>
       <c r="J270" s="2"/>
       <c r="K270" s="2"/>
       <c r="L270" s="2"/>
@@ -12176,7 +12113,7 @@
       <c r="F271" s="2"/>
       <c r="G271" s="2"/>
       <c r="H271" s="2"/>
-      <c r="I271" s="48"/>
+      <c r="I271" s="37"/>
       <c r="J271" s="2"/>
       <c r="K271" s="2"/>
       <c r="L271" s="2"/>
@@ -12205,7 +12142,7 @@
       <c r="F272" s="2"/>
       <c r="G272" s="2"/>
       <c r="H272" s="2"/>
-      <c r="I272" s="48"/>
+      <c r="I272" s="37"/>
       <c r="J272" s="2"/>
       <c r="K272" s="2"/>
       <c r="L272" s="2"/>
@@ -12234,7 +12171,7 @@
       <c r="F273" s="2"/>
       <c r="G273" s="2"/>
       <c r="H273" s="2"/>
-      <c r="I273" s="48"/>
+      <c r="I273" s="37"/>
       <c r="J273" s="2"/>
       <c r="K273" s="2"/>
       <c r="L273" s="2"/>
@@ -12263,7 +12200,7 @@
       <c r="F274" s="2"/>
       <c r="G274" s="2"/>
       <c r="H274" s="2"/>
-      <c r="I274" s="48"/>
+      <c r="I274" s="37"/>
       <c r="J274" s="2"/>
       <c r="K274" s="2"/>
       <c r="L274" s="2"/>
@@ -12292,7 +12229,7 @@
       <c r="F275" s="2"/>
       <c r="G275" s="2"/>
       <c r="H275" s="2"/>
-      <c r="I275" s="48"/>
+      <c r="I275" s="37"/>
       <c r="J275" s="2"/>
       <c r="K275" s="2"/>
       <c r="L275" s="2"/>
@@ -12321,7 +12258,7 @@
       <c r="F276" s="2"/>
       <c r="G276" s="2"/>
       <c r="H276" s="2"/>
-      <c r="I276" s="48"/>
+      <c r="I276" s="37"/>
       <c r="J276" s="2"/>
       <c r="K276" s="2"/>
       <c r="L276" s="2"/>
@@ -12350,7 +12287,7 @@
       <c r="F277" s="2"/>
       <c r="G277" s="2"/>
       <c r="H277" s="2"/>
-      <c r="I277" s="48"/>
+      <c r="I277" s="37"/>
       <c r="J277" s="2"/>
       <c r="K277" s="2"/>
       <c r="L277" s="2"/>
@@ -12379,7 +12316,7 @@
       <c r="F278" s="2"/>
       <c r="G278" s="2"/>
       <c r="H278" s="2"/>
-      <c r="I278" s="48"/>
+      <c r="I278" s="37"/>
       <c r="J278" s="2"/>
       <c r="K278" s="2"/>
       <c r="L278" s="2"/>
@@ -12408,7 +12345,7 @@
       <c r="F279" s="2"/>
       <c r="G279" s="2"/>
       <c r="H279" s="2"/>
-      <c r="I279" s="48"/>
+      <c r="I279" s="37"/>
       <c r="J279" s="2"/>
       <c r="K279" s="2"/>
       <c r="L279" s="2"/>
@@ -12437,7 +12374,7 @@
       <c r="F280" s="2"/>
       <c r="G280" s="2"/>
       <c r="H280" s="2"/>
-      <c r="I280" s="48"/>
+      <c r="I280" s="37"/>
       <c r="J280" s="2"/>
       <c r="K280" s="2"/>
       <c r="L280" s="2"/>
@@ -12466,7 +12403,7 @@
       <c r="F281" s="2"/>
       <c r="G281" s="2"/>
       <c r="H281" s="2"/>
-      <c r="I281" s="48"/>
+      <c r="I281" s="37"/>
       <c r="J281" s="2"/>
       <c r="K281" s="2"/>
       <c r="L281" s="2"/>
@@ -12495,7 +12432,7 @@
       <c r="F282" s="2"/>
       <c r="G282" s="2"/>
       <c r="H282" s="2"/>
-      <c r="I282" s="48"/>
+      <c r="I282" s="37"/>
       <c r="J282" s="2"/>
       <c r="K282" s="2"/>
       <c r="L282" s="2"/>
@@ -12524,7 +12461,7 @@
       <c r="F283" s="2"/>
       <c r="G283" s="2"/>
       <c r="H283" s="2"/>
-      <c r="I283" s="48"/>
+      <c r="I283" s="37"/>
       <c r="J283" s="2"/>
       <c r="K283" s="2"/>
       <c r="L283" s="2"/>
@@ -12553,7 +12490,7 @@
       <c r="F284" s="2"/>
       <c r="G284" s="2"/>
       <c r="H284" s="2"/>
-      <c r="I284" s="48"/>
+      <c r="I284" s="37"/>
       <c r="J284" s="2"/>
       <c r="K284" s="2"/>
       <c r="L284" s="2"/>
@@ -12582,7 +12519,7 @@
       <c r="F285" s="2"/>
       <c r="G285" s="2"/>
       <c r="H285" s="2"/>
-      <c r="I285" s="48"/>
+      <c r="I285" s="37"/>
       <c r="J285" s="2"/>
       <c r="K285" s="2"/>
       <c r="L285" s="2"/>
@@ -12611,7 +12548,7 @@
       <c r="F286" s="2"/>
       <c r="G286" s="2"/>
       <c r="H286" s="2"/>
-      <c r="I286" s="48"/>
+      <c r="I286" s="37"/>
       <c r="J286" s="2"/>
       <c r="K286" s="2"/>
       <c r="L286" s="2"/>
@@ -12640,7 +12577,7 @@
       <c r="F287" s="2"/>
       <c r="G287" s="2"/>
       <c r="H287" s="2"/>
-      <c r="I287" s="48"/>
+      <c r="I287" s="37"/>
       <c r="J287" s="2"/>
       <c r="K287" s="2"/>
       <c r="L287" s="2"/>
@@ -12669,7 +12606,7 @@
       <c r="F288" s="2"/>
       <c r="G288" s="2"/>
       <c r="H288" s="2"/>
-      <c r="I288" s="48"/>
+      <c r="I288" s="37"/>
       <c r="J288" s="2"/>
       <c r="K288" s="2"/>
       <c r="L288" s="2"/>
@@ -12698,7 +12635,7 @@
       <c r="F289" s="2"/>
       <c r="G289" s="2"/>
       <c r="H289" s="2"/>
-      <c r="I289" s="48"/>
+      <c r="I289" s="37"/>
       <c r="J289" s="2"/>
       <c r="K289" s="2"/>
       <c r="L289" s="2"/>
@@ -12727,7 +12664,7 @@
       <c r="F290" s="2"/>
       <c r="G290" s="2"/>
       <c r="H290" s="2"/>
-      <c r="I290" s="48"/>
+      <c r="I290" s="37"/>
       <c r="J290" s="2"/>
       <c r="K290" s="2"/>
       <c r="L290" s="2"/>
@@ -12756,7 +12693,7 @@
       <c r="F291" s="2"/>
       <c r="G291" s="2"/>
       <c r="H291" s="2"/>
-      <c r="I291" s="48"/>
+      <c r="I291" s="37"/>
       <c r="J291" s="2"/>
       <c r="K291" s="2"/>
       <c r="L291" s="2"/>
@@ -12785,7 +12722,7 @@
       <c r="F292" s="2"/>
       <c r="G292" s="2"/>
       <c r="H292" s="2"/>
-      <c r="I292" s="48"/>
+      <c r="I292" s="37"/>
       <c r="J292" s="2"/>
       <c r="K292" s="2"/>
       <c r="L292" s="2"/>
@@ -12814,7 +12751,7 @@
       <c r="F293" s="2"/>
       <c r="G293" s="2"/>
       <c r="H293" s="2"/>
-      <c r="I293" s="48"/>
+      <c r="I293" s="37"/>
       <c r="J293" s="2"/>
       <c r="K293" s="2"/>
       <c r="L293" s="2"/>
@@ -12843,7 +12780,7 @@
       <c r="F294" s="2"/>
       <c r="G294" s="2"/>
       <c r="H294" s="2"/>
-      <c r="I294" s="48"/>
+      <c r="I294" s="37"/>
       <c r="J294" s="2"/>
       <c r="K294" s="2"/>
       <c r="L294" s="2"/>
@@ -12872,7 +12809,7 @@
       <c r="F295" s="2"/>
       <c r="G295" s="2"/>
       <c r="H295" s="2"/>
-      <c r="I295" s="48"/>
+      <c r="I295" s="37"/>
       <c r="J295" s="2"/>
       <c r="K295" s="2"/>
       <c r="L295" s="2"/>
@@ -12901,7 +12838,7 @@
       <c r="F296" s="2"/>
       <c r="G296" s="2"/>
       <c r="H296" s="2"/>
-      <c r="I296" s="48"/>
+      <c r="I296" s="37"/>
       <c r="J296" s="2"/>
       <c r="K296" s="2"/>
       <c r="L296" s="2"/>
@@ -12930,7 +12867,7 @@
       <c r="F297" s="2"/>
       <c r="G297" s="2"/>
       <c r="H297" s="2"/>
-      <c r="I297" s="48"/>
+      <c r="I297" s="37"/>
       <c r="J297" s="2"/>
       <c r="K297" s="2"/>
       <c r="L297" s="2"/>
@@ -12959,7 +12896,7 @@
       <c r="F298" s="2"/>
       <c r="G298" s="2"/>
       <c r="H298" s="2"/>
-      <c r="I298" s="48"/>
+      <c r="I298" s="37"/>
       <c r="J298" s="2"/>
       <c r="K298" s="2"/>
       <c r="L298" s="2"/>
@@ -12988,7 +12925,7 @@
       <c r="F299" s="2"/>
       <c r="G299" s="2"/>
       <c r="H299" s="2"/>
-      <c r="I299" s="48"/>
+      <c r="I299" s="37"/>
       <c r="J299" s="2"/>
       <c r="K299" s="2"/>
       <c r="L299" s="2"/>
@@ -13017,7 +12954,7 @@
       <c r="F300" s="2"/>
       <c r="G300" s="2"/>
       <c r="H300" s="2"/>
-      <c r="I300" s="48"/>
+      <c r="I300" s="37"/>
       <c r="J300" s="2"/>
       <c r="K300" s="2"/>
       <c r="L300" s="2"/>
@@ -13046,7 +12983,7 @@
       <c r="F301" s="2"/>
       <c r="G301" s="2"/>
       <c r="H301" s="2"/>
-      <c r="I301" s="48"/>
+      <c r="I301" s="37"/>
       <c r="J301" s="2"/>
       <c r="K301" s="2"/>
       <c r="L301" s="2"/>
@@ -13075,7 +13012,7 @@
       <c r="F302" s="2"/>
       <c r="G302" s="2"/>
       <c r="H302" s="2"/>
-      <c r="I302" s="48"/>
+      <c r="I302" s="37"/>
       <c r="J302" s="2"/>
       <c r="K302" s="2"/>
       <c r="L302" s="2"/>
@@ -13104,7 +13041,7 @@
       <c r="F303" s="2"/>
       <c r="G303" s="2"/>
       <c r="H303" s="2"/>
-      <c r="I303" s="48"/>
+      <c r="I303" s="37"/>
       <c r="J303" s="2"/>
       <c r="K303" s="2"/>
       <c r="L303" s="2"/>
@@ -13133,7 +13070,7 @@
       <c r="F304" s="2"/>
       <c r="G304" s="2"/>
       <c r="H304" s="2"/>
-      <c r="I304" s="48"/>
+      <c r="I304" s="37"/>
       <c r="J304" s="2"/>
       <c r="K304" s="2"/>
       <c r="L304" s="2"/>
@@ -13162,7 +13099,7 @@
       <c r="F305" s="2"/>
       <c r="G305" s="2"/>
       <c r="H305" s="2"/>
-      <c r="I305" s="48"/>
+      <c r="I305" s="37"/>
       <c r="J305" s="2"/>
       <c r="K305" s="2"/>
       <c r="L305" s="2"/>
@@ -13191,7 +13128,7 @@
       <c r="F306" s="2"/>
       <c r="G306" s="2"/>
       <c r="H306" s="2"/>
-      <c r="I306" s="48"/>
+      <c r="I306" s="37"/>
       <c r="J306" s="2"/>
       <c r="K306" s="2"/>
       <c r="L306" s="2"/>
@@ -13220,7 +13157,7 @@
       <c r="F307" s="2"/>
       <c r="G307" s="2"/>
       <c r="H307" s="2"/>
-      <c r="I307" s="48"/>
+      <c r="I307" s="37"/>
       <c r="J307" s="2"/>
       <c r="K307" s="2"/>
       <c r="L307" s="2"/>
@@ -13249,7 +13186,7 @@
       <c r="F308" s="2"/>
       <c r="G308" s="2"/>
       <c r="H308" s="2"/>
-      <c r="I308" s="48"/>
+      <c r="I308" s="37"/>
       <c r="J308" s="2"/>
       <c r="K308" s="2"/>
       <c r="L308" s="2"/>
@@ -13278,7 +13215,7 @@
       <c r="F309" s="2"/>
       <c r="G309" s="2"/>
       <c r="H309" s="2"/>
-      <c r="I309" s="48"/>
+      <c r="I309" s="37"/>
       <c r="J309" s="2"/>
       <c r="K309" s="2"/>
       <c r="L309" s="2"/>
@@ -13307,7 +13244,7 @@
       <c r="F310" s="2"/>
       <c r="G310" s="2"/>
       <c r="H310" s="2"/>
-      <c r="I310" s="48"/>
+      <c r="I310" s="37"/>
       <c r="J310" s="2"/>
       <c r="K310" s="2"/>
       <c r="L310" s="2"/>
@@ -13336,7 +13273,7 @@
       <c r="F311" s="2"/>
       <c r="G311" s="2"/>
       <c r="H311" s="2"/>
-      <c r="I311" s="48"/>
+      <c r="I311" s="2"/>
       <c r="J311" s="2"/>
       <c r="K311" s="2"/>
       <c r="L311" s="2"/>
@@ -13354,7 +13291,6 @@
       <c r="X311" s="2"/>
       <c r="Y311" s="2"/>
       <c r="Z311" s="2"/>
-      <c r="AA311" s="2"/>
     </row>
     <row r="312" ht="15.75" customHeight="1">
       <c r="A312" s="2"/>
@@ -32676,66 +32612,38 @@
       <c r="Y1001" s="2"/>
       <c r="Z1001" s="2"/>
     </row>
-    <row r="1002" ht="15.75" customHeight="1">
-      <c r="A1002" s="2"/>
-      <c r="B1002" s="2"/>
-      <c r="C1002" s="2"/>
-      <c r="D1002" s="2"/>
-      <c r="E1002" s="2"/>
-      <c r="F1002" s="2"/>
-      <c r="G1002" s="2"/>
-      <c r="H1002" s="2"/>
-      <c r="I1002" s="2"/>
-      <c r="J1002" s="2"/>
-      <c r="K1002" s="2"/>
-      <c r="L1002" s="2"/>
-      <c r="M1002" s="2"/>
-      <c r="N1002" s="2"/>
-      <c r="O1002" s="2"/>
-      <c r="P1002" s="2"/>
-      <c r="Q1002" s="2"/>
-      <c r="R1002" s="2"/>
-      <c r="S1002" s="2"/>
-      <c r="T1002" s="2"/>
-      <c r="U1002" s="2"/>
-      <c r="V1002" s="2"/>
-      <c r="W1002" s="2"/>
-      <c r="X1002" s="2"/>
-      <c r="Y1002" s="2"/>
-      <c r="Z1002" s="2"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E108">
+  <conditionalFormatting sqref="E2:E107">
     <cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="c">
       <formula>LEFT((E2),LEN("c"))=("c")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E108">
+  <conditionalFormatting sqref="E2:E107">
     <cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="u">
       <formula>LEFT((E2),LEN("u"))=("u")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E108">
+  <conditionalFormatting sqref="E2:E107">
     <cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="l">
       <formula>LEFT((E2),LEN("l"))=("l")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E108">
+  <conditionalFormatting sqref="E2:E107">
     <cfRule type="beginsWith" dxfId="3" priority="4" operator="beginsWith" text="f">
       <formula>LEFT((E2),LEN("f"))=("f")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H142">
+  <conditionalFormatting sqref="H2:H141">
     <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>"unilateral"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H142">
+  <conditionalFormatting sqref="H2:H141">
     <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>"bilateral"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J1:J1002">
+  <conditionalFormatting sqref="J1:J1001">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -32745,7 +32653,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:K1002">
+  <conditionalFormatting sqref="K1:K1001">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -32756,26 +32664,26 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F1002">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F1001">
       <formula1>'Referência'!$D$2:$D$11</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H202">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M2:M1001">
+      <formula1>'Referência'!$K$2:$K$28</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="L2:L1001">
+      <formula1>'Referência'!$I$2:$I$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="H2:H201">
       <formula1>'Referência'!$E$2:$E$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I1002">
-      <formula1>'Referência'!$G$2:$G$3</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L2:L1002">
-      <formula1>'Referência'!$I$2:$I$3</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E2:E202">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E201">
       <formula1>'Referência'!$A$2:$A$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G202">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G201">
       <formula1>'Referência'!$C$2:$C$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M2:M1002">
-      <formula1>'Referência'!$K$2:$K$28</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I1001">
+      <formula1>'Referência'!$G$2:$G$3</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions/>
@@ -32807,33 +32715,33 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="38" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="49" t="s">
+      <c r="C1" s="38" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="49" t="s">
+      <c r="E1" s="38" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="2"/>
-      <c r="G1" s="49" t="s">
+      <c r="G1" s="38" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="2"/>
-      <c r="I1" s="49" t="s">
+      <c r="I1" s="38" t="s">
         <v>11</v>
       </c>
       <c r="J1" s="2"/>
-      <c r="K1" s="49" t="s">
+      <c r="K1" s="38" t="s">
         <v>12</v>
       </c>
       <c r="L1" s="2"/>
-      <c r="M1" s="49" t="s">
+      <c r="M1" s="38" t="s">
         <v>11</v>
       </c>
       <c r="N1" s="2"/>
@@ -32851,33 +32759,33 @@
       <c r="Z1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="37" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="37" t="s">
         <v>46</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="48" t="s">
+      <c r="E2" s="37" t="s">
         <v>47</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="G2" s="48" t="s">
+      <c r="G2" s="37" t="s">
         <v>8</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="48" t="s">
+      <c r="I2" s="37" t="s">
         <v>22</v>
       </c>
       <c r="J2" s="2"/>
-      <c r="K2" s="48" t="s">
-        <v>282</v>
+      <c r="K2" s="37" t="s">
+        <v>279</v>
       </c>
       <c r="L2" s="2"/>
-      <c r="M2" s="48" t="s">
+      <c r="M2" s="37" t="s">
         <v>22</v>
       </c>
       <c r="N2" s="2"/>
@@ -32895,33 +32803,33 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="37" t="s">
         <v>68</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="37" t="s">
         <v>159</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="37" t="s">
         <v>20</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="48" t="s">
+      <c r="G3" s="37" t="s">
         <v>21</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="48" t="s">
+      <c r="I3" s="37" t="s">
         <v>30</v>
       </c>
       <c r="J3" s="2"/>
-      <c r="K3" s="48" t="s">
+      <c r="K3" s="37" t="s">
         <v>87</v>
       </c>
       <c r="L3" s="2"/>
-      <c r="M3" s="48" t="s">
+      <c r="M3" s="37" t="s">
         <v>30</v>
       </c>
       <c r="N3" s="2"/>
@@ -32939,17 +32847,17 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="37" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="48" t="s">
+      <c r="C4" s="37" t="s">
         <v>90</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E4" s="48" t="s">
+      <c r="E4" s="37" t="s">
         <v>66</v>
       </c>
       <c r="F4" s="2"/>
@@ -32957,7 +32865,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="48" t="s">
+      <c r="K4" s="37" t="s">
         <v>162</v>
       </c>
       <c r="L4" s="2"/>
@@ -32977,17 +32885,17 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="48" t="s">
-        <v>283</v>
+      <c r="A5" s="37" t="s">
+        <v>280</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="37" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="E5" s="48" t="s">
+      <c r="E5" s="37" t="s">
         <v>63</v>
       </c>
       <c r="F5" s="2"/>
@@ -32995,7 +32903,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="48" t="s">
+      <c r="K5" s="37" t="s">
         <v>31</v>
       </c>
       <c r="L5" s="2"/>
@@ -33017,7 +32925,7 @@
     <row r="6">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="37" t="s">
         <v>41</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -33029,7 +32937,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="48" t="s">
+      <c r="K6" s="37" t="s">
         <v>91</v>
       </c>
       <c r="L6" s="2"/>
@@ -33051,7 +32959,7 @@
     <row r="7">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="37" t="s">
         <v>136</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -33063,7 +32971,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="48" t="s">
+      <c r="K7" s="37" t="s">
         <v>166</v>
       </c>
       <c r="L7" s="2"/>
@@ -33085,7 +32993,7 @@
     <row r="8">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
-      <c r="C8" s="48" t="s">
+      <c r="C8" s="37" t="s">
         <v>70</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -33097,7 +33005,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="48" t="s">
+      <c r="K8" s="37" t="s">
         <v>71</v>
       </c>
       <c r="L8" s="2"/>
@@ -33119,7 +33027,7 @@
     <row r="9">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="37" t="s">
         <v>97</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -33131,7 +33039,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="48" t="s">
+      <c r="K9" s="37" t="s">
         <v>214</v>
       </c>
       <c r="L9" s="2"/>
@@ -33153,7 +33061,7 @@
     <row r="10">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="37" t="s">
         <v>213</v>
       </c>
       <c r="D10" s="2" t="s">
@@ -33165,7 +33073,7 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="48" t="s">
+      <c r="K10" s="37" t="s">
         <v>80</v>
       </c>
       <c r="L10" s="2"/>
@@ -33187,7 +33095,7 @@
     <row r="11">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="37" t="s">
         <v>79</v>
       </c>
       <c r="D11" s="2" t="s">
@@ -33199,7 +33107,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="48" t="s">
+      <c r="K11" s="37" t="s">
         <v>125</v>
       </c>
       <c r="L11" s="2"/>
@@ -33221,7 +33129,7 @@
     <row r="12">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="37" t="s">
         <v>124</v>
       </c>
       <c r="D12" s="2"/>
@@ -33231,7 +33139,7 @@
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="48" t="s">
+      <c r="K12" s="37" t="s">
         <v>107</v>
       </c>
       <c r="L12" s="2"/>
@@ -33253,7 +33161,7 @@
     <row r="13">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="37" t="s">
         <v>142</v>
       </c>
       <c r="D13" s="2"/>
@@ -33263,7 +33171,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="48" t="s">
+      <c r="K13" s="37" t="s">
         <v>234</v>
       </c>
       <c r="L13" s="2"/>
@@ -33285,7 +33193,7 @@
     <row r="14">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
-      <c r="C14" s="48" t="s">
+      <c r="C14" s="37" t="s">
         <v>106</v>
       </c>
       <c r="D14" s="2"/>
@@ -33295,8 +33203,8 @@
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="48" t="s">
-        <v>271</v>
+      <c r="K14" s="37" t="s">
+        <v>268</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
@@ -33317,7 +33225,7 @@
     <row r="15">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="37" t="s">
         <v>233</v>
       </c>
       <c r="D15" s="2"/>
@@ -33327,7 +33235,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="50" t="s">
+      <c r="K15" s="37" t="s">
         <v>185</v>
       </c>
       <c r="L15" s="2"/>
@@ -33350,7 +33258,7 @@
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -33359,7 +33267,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="48" t="s">
+      <c r="K16" s="37" t="s">
         <v>116</v>
       </c>
       <c r="L16" s="2"/>
@@ -33391,8 +33299,8 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="48" t="s">
-        <v>284</v>
+      <c r="K17" s="37" t="s">
+        <v>281</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
@@ -33423,7 +33331,7 @@
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="48" t="s">
+      <c r="K18" s="37" t="s">
         <v>23</v>
       </c>
       <c r="L18" s="2"/>
@@ -33455,7 +33363,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="48" t="s">
+      <c r="K19" s="37" t="s">
         <v>62</v>
       </c>
       <c r="L19" s="2"/>
@@ -33485,7 +33393,7 @@
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="48" t="s">
+      <c r="K20" s="37" t="s">
         <v>54</v>
       </c>
       <c r="L20" s="2"/>
@@ -33515,7 +33423,7 @@
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="48" t="s">
+      <c r="K21" s="37" t="s">
         <v>48</v>
       </c>
       <c r="L21" s="2"/>
@@ -33545,7 +33453,7 @@
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="48" t="s">
+      <c r="K22" s="37" t="s">
         <v>85</v>
       </c>
       <c r="L22" s="2"/>
@@ -33575,8 +33483,8 @@
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
-      <c r="K23" s="48" t="s">
-        <v>250</v>
+      <c r="K23" s="37" t="s">
+        <v>247</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -33605,7 +33513,7 @@
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="48" t="s">
+      <c r="K24" s="37" t="s">
         <v>35</v>
       </c>
       <c r="L24" s="2"/>
@@ -33635,7 +33543,7 @@
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="48" t="s">
+      <c r="K25" s="37" t="s">
         <v>131</v>
       </c>
       <c r="L25" s="2"/>
@@ -33665,7 +33573,7 @@
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
-      <c r="K26" s="48" t="s">
+      <c r="K26" s="37" t="s">
         <v>42</v>
       </c>
       <c r="L26" s="2"/>
@@ -33695,8 +33603,8 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
-      <c r="K27" s="48" t="s">
-        <v>260</v>
+      <c r="K27" s="37" t="s">
+        <v>257</v>
       </c>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
@@ -33725,7 +33633,7 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="48" t="s">
+      <c r="K28" s="37" t="s">
         <v>137</v>
       </c>
       <c r="L28" s="2"/>

</xml_diff>

<commit_message>
redesign HUB-centric: sidebar, rotina ativa por aluno, comparacao periodos
- HUB como pagina principal com seletor de aluno e rotina ativa
- toggle Atual/Anterior/Lado a lado para comparar periodos
- sidebar fixa de navegacao (desktop) + barra horizontal (mobile)
- rotina_ativa_id na tabela alunos, auto-setado ao salvar historico
- paginas wrapper (alunos_page, historico_page) extendem base
- gerador context-aware via query params (aluno_id/acao/treino)
- organizacao do historico melhorada + botoes mobile

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="282">
   <si>
     <t>nome</t>
   </si>
@@ -172,10 +172,10 @@
     <t>Agachamento búlgaro</t>
   </si>
   <si>
-    <t>Agachamento</t>
+    <t>Agachamento goblet</t>
   </si>
   <si>
-    <t>Agachamento goblet</t>
+    <t>Agachamento</t>
   </si>
   <si>
     <t>Halter</t>
@@ -1781,9 +1781,7 @@
       <c r="A8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>51</v>
-      </c>
+      <c r="B8" s="11"/>
       <c r="C8" s="10" t="s">
         <v>44</v>
       </c>
@@ -1834,10 +1832,10 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>52</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>51</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>53</v>
@@ -1892,7 +1890,7 @@
         <v>55</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>56</v>
@@ -1947,7 +1945,7 @@
         <v>57</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>58</v>
@@ -6683,7 +6681,7 @@
         <v>256</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C97" s="10" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
settings.local e banco atualizado
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -1771,7 +1771,7 @@
       <c r="Z1" s="2"/>
       <c r="AA1" s="2"/>
     </row>
-    <row r="2">
+    <row r="2" hidden="1">
       <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
@@ -1832,7 +1832,7 @@
       <c r="Z2" s="4"/>
       <c r="AA2" s="4"/>
     </row>
-    <row r="3">
+    <row r="3" hidden="1">
       <c r="A3" s="10" t="s">
         <v>28</v>
       </c>
@@ -1893,7 +1893,7 @@
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" hidden="1">
       <c r="A4" s="10" t="s">
         <v>37</v>
       </c>
@@ -1954,7 +1954,7 @@
       <c r="Z4" s="2"/>
       <c r="AA4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" hidden="1">
       <c r="A5" s="9" t="s">
         <v>42</v>
       </c>
@@ -2015,7 +2015,7 @@
       <c r="Z5" s="4"/>
       <c r="AA5" s="4"/>
     </row>
-    <row r="6">
+    <row r="6" hidden="1">
       <c r="A6" s="10" t="s">
         <v>50</v>
       </c>
@@ -2074,7 +2074,7 @@
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" hidden="1">
       <c r="A7" s="10" t="s">
         <v>53</v>
       </c>
@@ -2135,7 +2135,7 @@
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" hidden="1">
       <c r="A8" s="10" t="s">
         <v>58</v>
       </c>
@@ -2196,7 +2196,7 @@
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
     </row>
-    <row r="9">
+    <row r="9" hidden="1">
       <c r="A9" s="10" t="s">
         <v>60</v>
       </c>
@@ -2257,7 +2257,7 @@
       <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
     </row>
-    <row r="10">
+    <row r="10" hidden="1">
       <c r="A10" s="10" t="s">
         <v>62</v>
       </c>
@@ -2318,7 +2318,7 @@
       <c r="Z10" s="2"/>
       <c r="AA10" s="2"/>
     </row>
-    <row r="11">
+    <row r="11" hidden="1">
       <c r="A11" s="10" t="s">
         <v>67</v>
       </c>
@@ -2379,7 +2379,7 @@
       <c r="Z11" s="2"/>
       <c r="AA11" s="2"/>
     </row>
-    <row r="12">
+    <row r="12" hidden="1">
       <c r="A12" s="10" t="s">
         <v>69</v>
       </c>
@@ -2438,7 +2438,7 @@
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
     </row>
-    <row r="13">
+    <row r="13" hidden="1">
       <c r="A13" s="3" t="s">
         <v>75</v>
       </c>
@@ -2497,7 +2497,7 @@
       <c r="Z13" s="4"/>
       <c r="AA13" s="4"/>
     </row>
-    <row r="14">
+    <row r="14" hidden="1">
       <c r="A14" s="9" t="s">
         <v>76</v>
       </c>
@@ -2556,7 +2556,7 @@
       <c r="Z14" s="4"/>
       <c r="AA14" s="4"/>
     </row>
-    <row r="15">
+    <row r="15" hidden="1">
       <c r="A15" s="10" t="s">
         <v>77</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="Z15" s="2"/>
       <c r="AA15" s="2"/>
     </row>
-    <row r="16">
+    <row r="16" hidden="1">
       <c r="A16" s="10" t="s">
         <v>84</v>
       </c>
@@ -2678,7 +2678,7 @@
       <c r="Z16" s="2"/>
       <c r="AA16" s="2"/>
     </row>
-    <row r="17">
+    <row r="17" hidden="1">
       <c r="A17" s="10" t="s">
         <v>85</v>
       </c>
@@ -2739,7 +2739,7 @@
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
     </row>
-    <row r="18">
+    <row r="18" hidden="1">
       <c r="A18" s="10" t="s">
         <v>92</v>
       </c>
@@ -2802,7 +2802,7 @@
       <c r="Z18" s="2"/>
       <c r="AA18" s="2"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="15.75" hidden="1" customHeight="1">
       <c r="A19" s="9" t="s">
         <v>94</v>
       </c>
@@ -2863,7 +2863,7 @@
       <c r="Z19" s="4"/>
       <c r="AA19" s="4"/>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" ht="15.75" hidden="1" customHeight="1">
       <c r="A20" s="10" t="s">
         <v>95</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="Z20" s="2"/>
       <c r="AA20" s="2"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="15.75" hidden="1" customHeight="1">
       <c r="A21" s="10" t="s">
         <v>96</v>
       </c>
@@ -2985,7 +2985,7 @@
       <c r="Z21" s="2"/>
       <c r="AA21" s="2"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="15.75" hidden="1" customHeight="1">
       <c r="A22" s="10" t="s">
         <v>97</v>
       </c>
@@ -3046,7 +3046,7 @@
       <c r="Z22" s="2"/>
       <c r="AA22" s="2"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="15.75" hidden="1" customHeight="1">
       <c r="A23" s="10" t="s">
         <v>99</v>
       </c>
@@ -3105,7 +3105,7 @@
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="15.75" hidden="1" customHeight="1">
       <c r="A24" s="10" t="s">
         <v>102</v>
       </c>
@@ -3223,7 +3223,7 @@
       <c r="Z25" s="2"/>
       <c r="AA25" s="2"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" ht="15.75" hidden="1" customHeight="1">
       <c r="A26" s="9" t="s">
         <v>111</v>
       </c>
@@ -3282,7 +3282,7 @@
       <c r="Z26" s="4"/>
       <c r="AA26" s="4"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" ht="15.75" hidden="1" customHeight="1">
       <c r="A27" s="10" t="s">
         <v>113</v>
       </c>
@@ -3345,7 +3345,7 @@
       <c r="Z27" s="2"/>
       <c r="AA27" s="2"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="15.75" hidden="1" customHeight="1">
       <c r="A28" s="10" t="s">
         <v>114</v>
       </c>
@@ -3406,7 +3406,7 @@
       <c r="Z28" s="2"/>
       <c r="AA28" s="2"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="15.75" hidden="1" customHeight="1">
       <c r="A29" s="9" t="s">
         <v>118</v>
       </c>
@@ -3469,7 +3469,7 @@
       <c r="Z29" s="4"/>
       <c r="AA29" s="4"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" ht="15.75" hidden="1" customHeight="1">
       <c r="A30" s="10" t="s">
         <v>120</v>
       </c>
@@ -3532,7 +3532,7 @@
       <c r="Z30" s="2"/>
       <c r="AA30" s="2"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="15.75" hidden="1" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>122</v>
       </c>
@@ -3591,7 +3591,7 @@
       <c r="Z31" s="4"/>
       <c r="AA31" s="4"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="15.75" hidden="1" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>127</v>
       </c>
@@ -3652,7 +3652,7 @@
       <c r="Z32" s="4"/>
       <c r="AA32" s="4"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="15.75" hidden="1" customHeight="1">
       <c r="A33" s="10" t="s">
         <v>128</v>
       </c>
@@ -3713,7 +3713,7 @@
       <c r="Z33" s="2"/>
       <c r="AA33" s="2"/>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" ht="15.75" hidden="1" customHeight="1">
       <c r="A34" s="10" t="s">
         <v>130</v>
       </c>
@@ -3774,7 +3774,7 @@
       <c r="Z34" s="2"/>
       <c r="AA34" s="2"/>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" ht="15.75" hidden="1" customHeight="1">
       <c r="A35" s="10" t="s">
         <v>132</v>
       </c>
@@ -3835,7 +3835,7 @@
       <c r="Z35" s="2"/>
       <c r="AA35" s="2"/>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" ht="15.75" hidden="1" customHeight="1">
       <c r="A36" s="10" t="s">
         <v>136</v>
       </c>
@@ -3898,7 +3898,7 @@
       <c r="Z36" s="2"/>
       <c r="AA36" s="2"/>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="15.75" hidden="1" customHeight="1">
       <c r="A37" s="10" t="s">
         <v>138</v>
       </c>
@@ -3959,7 +3959,7 @@
       <c r="Z37" s="2"/>
       <c r="AA37" s="2"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="15.75" hidden="1" customHeight="1">
       <c r="A38" s="10" t="s">
         <v>139</v>
       </c>
@@ -4022,7 +4022,7 @@
       <c r="Z38" s="2"/>
       <c r="AA38" s="2"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="15.75" hidden="1" customHeight="1">
       <c r="A39" s="9" t="s">
         <v>144</v>
       </c>
@@ -4085,7 +4085,7 @@
       <c r="Z39" s="4"/>
       <c r="AA39" s="4"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" ht="15.75" hidden="1" customHeight="1">
       <c r="A40" s="3" t="s">
         <v>147</v>
       </c>
@@ -4148,7 +4148,7 @@
       <c r="Z40" s="4"/>
       <c r="AA40" s="4"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="15.75" hidden="1" customHeight="1">
       <c r="A41" s="9" t="s">
         <v>149</v>
       </c>
@@ -4211,7 +4211,7 @@
       <c r="Z41" s="4"/>
       <c r="AA41" s="4"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" ht="15.75" hidden="1" customHeight="1">
       <c r="A42" s="10" t="s">
         <v>151</v>
       </c>
@@ -4272,7 +4272,7 @@
       <c r="Z42" s="2"/>
       <c r="AA42" s="2"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" ht="15.75" hidden="1" customHeight="1">
       <c r="A43" s="10" t="s">
         <v>152</v>
       </c>
@@ -4331,7 +4331,7 @@
       <c r="Z43" s="2"/>
       <c r="AA43" s="2"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="15.75" hidden="1" customHeight="1">
       <c r="A44" s="10" t="s">
         <v>155</v>
       </c>
@@ -4392,7 +4392,7 @@
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="15.75" hidden="1" customHeight="1">
       <c r="A45" s="9" t="s">
         <v>161</v>
       </c>
@@ -4453,7 +4453,7 @@
       <c r="Z45" s="4"/>
       <c r="AA45" s="4"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" ht="15.75" hidden="1" customHeight="1">
       <c r="A46" s="10" t="s">
         <v>165</v>
       </c>
@@ -4514,7 +4514,7 @@
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" ht="15.75" hidden="1" customHeight="1">
       <c r="A47" s="10" t="s">
         <v>166</v>
       </c>
@@ -4575,7 +4575,7 @@
       <c r="Z47" s="2"/>
       <c r="AA47" s="2"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" ht="15.75" hidden="1" customHeight="1">
       <c r="A48" s="10" t="s">
         <v>169</v>
       </c>
@@ -4636,7 +4636,7 @@
       <c r="Z48" s="2"/>
       <c r="AA48" s="2"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" ht="15.75" hidden="1" customHeight="1">
       <c r="A49" s="9" t="s">
         <v>170</v>
       </c>
@@ -4699,7 +4699,7 @@
       <c r="Z49" s="4"/>
       <c r="AA49" s="4"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" ht="15.75" hidden="1" customHeight="1">
       <c r="A50" s="10" t="s">
         <v>171</v>
       </c>
@@ -4760,7 +4760,7 @@
       <c r="Z50" s="2"/>
       <c r="AA50" s="2"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" ht="15.75" hidden="1" customHeight="1">
       <c r="A51" s="10" t="s">
         <v>172</v>
       </c>
@@ -5248,7 +5248,7 @@
       <c r="Z58" s="2"/>
       <c r="AA58" s="2"/>
     </row>
-    <row r="59" ht="15.75" customHeight="1">
+    <row r="59" ht="15.75" hidden="1" customHeight="1">
       <c r="A59" s="10" t="s">
         <v>194</v>
       </c>
@@ -5307,7 +5307,7 @@
       <c r="Z59" s="2"/>
       <c r="AA59" s="2"/>
     </row>
-    <row r="60" ht="15.75" customHeight="1">
+    <row r="60" ht="15.75" hidden="1" customHeight="1">
       <c r="A60" s="10" t="s">
         <v>195</v>
       </c>
@@ -5610,7 +5610,7 @@
       <c r="Z64" s="2"/>
       <c r="AA64" s="2"/>
     </row>
-    <row r="65" ht="15.75" customHeight="1">
+    <row r="65" ht="15.75" hidden="1" customHeight="1">
       <c r="A65" s="10" t="s">
         <v>205</v>
       </c>
@@ -5669,7 +5669,7 @@
       <c r="Z65" s="2"/>
       <c r="AA65" s="2"/>
     </row>
-    <row r="66" ht="15.75" customHeight="1">
+    <row r="66" ht="15.75" hidden="1" customHeight="1">
       <c r="A66" s="3" t="s">
         <v>208</v>
       </c>
@@ -5730,7 +5730,7 @@
       <c r="Z66" s="4"/>
       <c r="AA66" s="4"/>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
+    <row r="67" ht="15.75" hidden="1" customHeight="1">
       <c r="A67" s="3" t="s">
         <v>210</v>
       </c>
@@ -6169,7 +6169,7 @@
       <c r="Z73" s="4"/>
       <c r="AA73" s="4"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
+    <row r="74" ht="15.75" hidden="1" customHeight="1">
       <c r="A74" s="9" t="s">
         <v>220</v>
       </c>
@@ -6228,7 +6228,7 @@
       <c r="Z74" s="4"/>
       <c r="AA74" s="4"/>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
+    <row r="75" ht="15.75" hidden="1" customHeight="1">
       <c r="A75" s="10" t="s">
         <v>221</v>
       </c>
@@ -6289,7 +6289,7 @@
       <c r="Z75" s="2"/>
       <c r="AA75" s="2"/>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
+    <row r="76" ht="15.75" hidden="1" customHeight="1">
       <c r="A76" s="10" t="s">
         <v>223</v>
       </c>
@@ -6350,7 +6350,7 @@
       <c r="Z76" s="2"/>
       <c r="AA76" s="2"/>
     </row>
-    <row r="77" ht="15.75" customHeight="1">
+    <row r="77" ht="15.75" hidden="1" customHeight="1">
       <c r="A77" s="10" t="s">
         <v>224</v>
       </c>
@@ -6411,7 +6411,7 @@
       <c r="Z77" s="2"/>
       <c r="AA77" s="2"/>
     </row>
-    <row r="78" ht="15.75" customHeight="1">
+    <row r="78" ht="15.75" hidden="1" customHeight="1">
       <c r="A78" s="10" t="s">
         <v>226</v>
       </c>
@@ -6472,7 +6472,7 @@
       <c r="Z78" s="2"/>
       <c r="AA78" s="2"/>
     </row>
-    <row r="79" ht="15.75" customHeight="1">
+    <row r="79" ht="15.75" hidden="1" customHeight="1">
       <c r="A79" s="10" t="s">
         <v>227</v>
       </c>
@@ -6531,7 +6531,7 @@
       <c r="Z79" s="2"/>
       <c r="AA79" s="2"/>
     </row>
-    <row r="80" ht="15.75" customHeight="1">
+    <row r="80" ht="15.75" hidden="1" customHeight="1">
       <c r="A80" s="10" t="s">
         <v>229</v>
       </c>
@@ -6592,7 +6592,7 @@
       <c r="Z80" s="2"/>
       <c r="AA80" s="2"/>
     </row>
-    <row r="81" ht="15.75" customHeight="1">
+    <row r="81" ht="15.75" hidden="1" customHeight="1">
       <c r="A81" s="10" t="s">
         <v>230</v>
       </c>
@@ -6653,7 +6653,7 @@
       <c r="Z81" s="2"/>
       <c r="AA81" s="2"/>
     </row>
-    <row r="82" ht="15.75" customHeight="1">
+    <row r="82" ht="15.75" hidden="1" customHeight="1">
       <c r="A82" s="9" t="s">
         <v>231</v>
       </c>
@@ -6716,7 +6716,7 @@
       <c r="Z82" s="4"/>
       <c r="AA82" s="4"/>
     </row>
-    <row r="83" ht="15.75" customHeight="1">
+    <row r="83" ht="15.75" hidden="1" customHeight="1">
       <c r="A83" s="10" t="s">
         <v>234</v>
       </c>
@@ -6777,7 +6777,7 @@
       <c r="Z83" s="2"/>
       <c r="AA83" s="2"/>
     </row>
-    <row r="84" ht="15.75" customHeight="1">
+    <row r="84" ht="15.75" hidden="1" customHeight="1">
       <c r="A84" s="10" t="s">
         <v>235</v>
       </c>
@@ -6840,7 +6840,7 @@
       <c r="Z84" s="2"/>
       <c r="AA84" s="2"/>
     </row>
-    <row r="85" ht="15.75" customHeight="1">
+    <row r="85" ht="15.75" hidden="1" customHeight="1">
       <c r="A85" s="10" t="s">
         <v>239</v>
       </c>
@@ -6903,7 +6903,7 @@
       <c r="Z85" s="2"/>
       <c r="AA85" s="2"/>
     </row>
-    <row r="86" ht="15.75" customHeight="1">
+    <row r="86" ht="15.75" hidden="1" customHeight="1">
       <c r="A86" s="10" t="s">
         <v>241</v>
       </c>
@@ -6964,7 +6964,7 @@
       <c r="Z86" s="2"/>
       <c r="AA86" s="2"/>
     </row>
-    <row r="87" ht="15.75" customHeight="1">
+    <row r="87" ht="15.75" hidden="1" customHeight="1">
       <c r="A87" s="3" t="s">
         <v>242</v>
       </c>
@@ -7025,7 +7025,7 @@
       <c r="Z87" s="4"/>
       <c r="AA87" s="4"/>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
+    <row r="88" ht="15.75" hidden="1" customHeight="1">
       <c r="A88" s="9" t="s">
         <v>243</v>
       </c>
@@ -7086,7 +7086,7 @@
       <c r="Z88" s="4"/>
       <c r="AA88" s="4"/>
     </row>
-    <row r="89" ht="15.75" customHeight="1">
+    <row r="89" ht="15.75" hidden="1" customHeight="1">
       <c r="A89" s="3" t="s">
         <v>244</v>
       </c>
@@ -7147,7 +7147,7 @@
       <c r="Z89" s="4"/>
       <c r="AA89" s="4"/>
     </row>
-    <row r="90" ht="15.75" customHeight="1">
+    <row r="90" ht="15.75" hidden="1" customHeight="1">
       <c r="A90" s="10" t="s">
         <v>245</v>
       </c>
@@ -7206,7 +7206,7 @@
       <c r="Z90" s="2"/>
       <c r="AA90" s="2"/>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
+    <row r="91" ht="15.75" hidden="1" customHeight="1">
       <c r="A91" s="10" t="s">
         <v>250</v>
       </c>
@@ -7269,7 +7269,7 @@
       <c r="Z91" s="2"/>
       <c r="AA91" s="2"/>
     </row>
-    <row r="92" ht="15.75" customHeight="1">
+    <row r="92" ht="15.75" hidden="1" customHeight="1">
       <c r="A92" s="10" t="s">
         <v>253</v>
       </c>
@@ -7332,7 +7332,7 @@
       <c r="Z92" s="2"/>
       <c r="AA92" s="2"/>
     </row>
-    <row r="93" ht="15.75" customHeight="1">
+    <row r="93" ht="15.75" hidden="1" customHeight="1">
       <c r="A93" s="10" t="s">
         <v>255</v>
       </c>
@@ -7395,7 +7395,7 @@
       <c r="Z93" s="2"/>
       <c r="AA93" s="2"/>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
+    <row r="94" ht="15.75" hidden="1" customHeight="1">
       <c r="A94" s="10" t="s">
         <v>257</v>
       </c>
@@ -7456,7 +7456,7 @@
       <c r="Z94" s="2"/>
       <c r="AA94" s="2"/>
     </row>
-    <row r="95" ht="15.75" customHeight="1">
+    <row r="95" ht="15.75" hidden="1" customHeight="1">
       <c r="A95" s="3" t="s">
         <v>259</v>
       </c>
@@ -7517,7 +7517,7 @@
       <c r="Z95" s="4"/>
       <c r="AA95" s="4"/>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
+    <row r="96" ht="15.75" hidden="1" customHeight="1">
       <c r="A96" s="9" t="s">
         <v>260</v>
       </c>
@@ -7578,7 +7578,7 @@
       <c r="Z96" s="4"/>
       <c r="AA96" s="4"/>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
+    <row r="97" ht="15.75" hidden="1" customHeight="1">
       <c r="A97" s="10" t="s">
         <v>262</v>
       </c>
@@ -7641,7 +7641,7 @@
       <c r="Z97" s="2"/>
       <c r="AA97" s="2"/>
     </row>
-    <row r="98" ht="15.75" customHeight="1">
+    <row r="98" ht="15.75" hidden="1" customHeight="1">
       <c r="A98" s="9" t="s">
         <v>264</v>
       </c>
@@ -7700,7 +7700,7 @@
       <c r="Z98" s="4"/>
       <c r="AA98" s="4"/>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
+    <row r="99" ht="15.75" hidden="1" customHeight="1">
       <c r="A99" s="9" t="s">
         <v>265</v>
       </c>
@@ -7761,7 +7761,7 @@
       <c r="Z99" s="4"/>
       <c r="AA99" s="4"/>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
+    <row r="100" ht="15.75" hidden="1" customHeight="1">
       <c r="A100" s="9" t="s">
         <v>266</v>
       </c>
@@ -7822,7 +7822,7 @@
       <c r="Z100" s="4"/>
       <c r="AA100" s="4"/>
     </row>
-    <row r="101" ht="15.75" customHeight="1">
+    <row r="101" ht="15.75" hidden="1" customHeight="1">
       <c r="A101" s="10" t="s">
         <v>268</v>
       </c>
@@ -7883,7 +7883,7 @@
       <c r="Z101" s="2"/>
       <c r="AA101" s="2"/>
     </row>
-    <row r="102" ht="15.75" customHeight="1">
+    <row r="102" ht="15.75" hidden="1" customHeight="1">
       <c r="A102" s="3" t="s">
         <v>270</v>
       </c>
@@ -7946,7 +7946,7 @@
       <c r="Z102" s="4"/>
       <c r="AA102" s="4"/>
     </row>
-    <row r="103" ht="15.75" customHeight="1">
+    <row r="103" ht="15.75" hidden="1" customHeight="1">
       <c r="A103" s="10" t="s">
         <v>271</v>
       </c>
@@ -8007,7 +8007,7 @@
       <c r="Z103" s="2"/>
       <c r="AA103" s="2"/>
     </row>
-    <row r="104" ht="15.75" customHeight="1">
+    <row r="104" ht="15.75" hidden="1" customHeight="1">
       <c r="A104" s="10" t="s">
         <v>272</v>
       </c>
@@ -8068,7 +8068,7 @@
       <c r="Z104" s="2"/>
       <c r="AA104" s="2"/>
     </row>
-    <row r="105" ht="15.75" customHeight="1">
+    <row r="105" ht="15.75" hidden="1" customHeight="1">
       <c r="A105" s="10" t="s">
         <v>274</v>
       </c>
@@ -8131,7 +8131,7 @@
       <c r="Z105" s="2"/>
       <c r="AA105" s="2"/>
     </row>
-    <row r="106" ht="15.75" customHeight="1">
+    <row r="106" ht="15.75" hidden="1" customHeight="1">
       <c r="A106" s="10" t="s">
         <v>277</v>
       </c>
@@ -8499,7 +8499,7 @@
       <c r="Z111" s="4"/>
       <c r="AA111" s="4"/>
     </row>
-    <row r="112" ht="15.75" customHeight="1">
+    <row r="112" ht="15.75" hidden="1" customHeight="1">
       <c r="A112" s="9" t="s">
         <v>285</v>
       </c>
@@ -8562,7 +8562,7 @@
       <c r="Z112" s="4"/>
       <c r="AA112" s="4"/>
     </row>
-    <row r="113" ht="15.75" customHeight="1">
+    <row r="113" ht="15.75" hidden="1" customHeight="1">
       <c r="A113" s="10" t="s">
         <v>288</v>
       </c>
@@ -8625,7 +8625,7 @@
       <c r="Z113" s="2"/>
       <c r="AA113" s="2"/>
     </row>
-    <row r="114" ht="15.75" customHeight="1">
+    <row r="114" ht="15.75" hidden="1" customHeight="1">
       <c r="A114" s="10" t="s">
         <v>289</v>
       </c>
@@ -8688,7 +8688,7 @@
       <c r="Z114" s="2"/>
       <c r="AA114" s="2"/>
     </row>
-    <row r="115" ht="15.75" customHeight="1">
+    <row r="115" ht="15.75" hidden="1" customHeight="1">
       <c r="A115" s="10" t="s">
         <v>290</v>
       </c>
@@ -8751,7 +8751,7 @@
       <c r="Z115" s="2"/>
       <c r="AA115" s="2"/>
     </row>
-    <row r="116" ht="15.75" customHeight="1">
+    <row r="116" ht="15.75" hidden="1" customHeight="1">
       <c r="A116" s="10" t="s">
         <v>291</v>
       </c>
@@ -8812,7 +8812,7 @@
       <c r="Z116" s="2"/>
       <c r="AA116" s="2"/>
     </row>
-    <row r="117" ht="15.75" customHeight="1">
+    <row r="117" ht="15.75" hidden="1" customHeight="1">
       <c r="A117" s="9" t="s">
         <v>296</v>
       </c>
@@ -8873,7 +8873,7 @@
       <c r="Z117" s="4"/>
       <c r="AA117" s="4"/>
     </row>
-    <row r="118" ht="15.75" customHeight="1">
+    <row r="118" ht="15.75" hidden="1" customHeight="1">
       <c r="A118" s="63" t="s">
         <v>298</v>
       </c>
@@ -8936,7 +8936,7 @@
       <c r="Z118" s="2"/>
       <c r="AA118" s="2"/>
     </row>
-    <row r="119" ht="15.75" customHeight="1">
+    <row r="119" ht="15.75" hidden="1" customHeight="1">
       <c r="A119" s="63" t="s">
         <v>301</v>
       </c>
@@ -8997,7 +8997,7 @@
       <c r="Z119" s="2"/>
       <c r="AA119" s="2"/>
     </row>
-    <row r="120" ht="15.75" customHeight="1">
+    <row r="120" ht="15.75" hidden="1" customHeight="1">
       <c r="A120" s="10" t="s">
         <v>302</v>
       </c>
@@ -9058,7 +9058,7 @@
       <c r="Z120" s="2"/>
       <c r="AA120" s="2"/>
     </row>
-    <row r="121" ht="15.75" customHeight="1">
+    <row r="121" ht="15.75" hidden="1" customHeight="1">
       <c r="A121" s="10" t="s">
         <v>304</v>
       </c>
@@ -9121,7 +9121,7 @@
       <c r="Z121" s="2"/>
       <c r="AA121" s="2"/>
     </row>
-    <row r="122" ht="15.75" customHeight="1">
+    <row r="122" ht="15.75" hidden="1" customHeight="1">
       <c r="A122" s="10" t="s">
         <v>306</v>
       </c>
@@ -9184,7 +9184,7 @@
       <c r="Z122" s="2"/>
       <c r="AA122" s="2"/>
     </row>
-    <row r="123" ht="15.75" customHeight="1">
+    <row r="123" ht="15.75" hidden="1" customHeight="1">
       <c r="A123" s="63" t="s">
         <v>308</v>
       </c>
@@ -9245,7 +9245,7 @@
       <c r="Z123" s="2"/>
       <c r="AA123" s="2"/>
     </row>
-    <row r="124" ht="15.75" customHeight="1">
+    <row r="124" ht="15.75" hidden="1" customHeight="1">
       <c r="A124" s="3" t="s">
         <v>309</v>
       </c>
@@ -9306,7 +9306,7 @@
       <c r="Z124" s="4"/>
       <c r="AA124" s="4"/>
     </row>
-    <row r="125" ht="15.75" customHeight="1">
+    <row r="125" ht="15.75" hidden="1" customHeight="1">
       <c r="A125" s="9" t="s">
         <v>311</v>
       </c>
@@ -9367,7 +9367,7 @@
       <c r="Z125" s="4"/>
       <c r="AA125" s="4"/>
     </row>
-    <row r="126" ht="15.75" customHeight="1">
+    <row r="126" ht="15.75" hidden="1" customHeight="1">
       <c r="A126" s="3" t="s">
         <v>312</v>
       </c>
@@ -34101,7 +34101,14 @@
       <c r="Z1000" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$R$126"/>
+  <autoFilter ref="$A$1:$R$126">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="hinge"/>
+        <filter val="knee_flexion"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="E2:E126">
     <cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="co">
       <formula>LEFT((E2),LEN("co"))=("co")</formula>

</xml_diff>

<commit_message>
mds de inicio etapa 6
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -12,7 +12,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="340RZNeuHBGeotGKM/dXJ1npHZS4zP/DvD/MFWOMaec="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="P7CRpCEH7pi8xg7pMdH5Wq/2F7xjlo75XoD+mcYA5ss="/>
     </ext>
   </extLst>
 </workbook>
@@ -1771,7 +1771,7 @@
       <c r="Z1" s="2"/>
       <c r="AA1" s="2"/>
     </row>
-    <row r="2" hidden="1">
+    <row r="2">
       <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
@@ -3164,7 +3164,7 @@
       <c r="Z24" s="2"/>
       <c r="AA24" s="2"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" ht="15.75" hidden="1" customHeight="1">
       <c r="A25" s="10" t="s">
         <v>106</v>
       </c>
@@ -3223,7 +3223,7 @@
       <c r="Z25" s="2"/>
       <c r="AA25" s="2"/>
     </row>
-    <row r="26" ht="15.75" hidden="1" customHeight="1">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="9" t="s">
         <v>111</v>
       </c>
@@ -3591,7 +3591,7 @@
       <c r="Z31" s="4"/>
       <c r="AA31" s="4"/>
     </row>
-    <row r="32" ht="15.75" hidden="1" customHeight="1">
+    <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>127</v>
       </c>
@@ -3652,7 +3652,7 @@
       <c r="Z32" s="4"/>
       <c r="AA32" s="4"/>
     </row>
-    <row r="33" ht="15.75" hidden="1" customHeight="1">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="10" t="s">
         <v>128</v>
       </c>
@@ -3713,7 +3713,7 @@
       <c r="Z33" s="2"/>
       <c r="AA33" s="2"/>
     </row>
-    <row r="34" ht="15.75" hidden="1" customHeight="1">
+    <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="10" t="s">
         <v>130</v>
       </c>
@@ -3774,7 +3774,7 @@
       <c r="Z34" s="2"/>
       <c r="AA34" s="2"/>
     </row>
-    <row r="35" ht="15.75" hidden="1" customHeight="1">
+    <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="10" t="s">
         <v>132</v>
       </c>
@@ -3835,7 +3835,7 @@
       <c r="Z35" s="2"/>
       <c r="AA35" s="2"/>
     </row>
-    <row r="36" ht="15.75" hidden="1" customHeight="1">
+    <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="10" t="s">
         <v>136</v>
       </c>
@@ -3898,7 +3898,7 @@
       <c r="Z36" s="2"/>
       <c r="AA36" s="2"/>
     </row>
-    <row r="37" ht="15.75" hidden="1" customHeight="1">
+    <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="10" t="s">
         <v>138</v>
       </c>
@@ -4821,7 +4821,7 @@
       <c r="Z51" s="2"/>
       <c r="AA51" s="2"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" ht="15.75" hidden="1" customHeight="1">
       <c r="A52" s="9" t="s">
         <v>175</v>
       </c>
@@ -4882,7 +4882,7 @@
       <c r="Z52" s="4"/>
       <c r="AA52" s="4"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" ht="15.75" hidden="1" customHeight="1">
       <c r="A53" s="3" t="s">
         <v>178</v>
       </c>
@@ -4943,7 +4943,7 @@
       <c r="Z53" s="4"/>
       <c r="AA53" s="4"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" ht="15.75" hidden="1" customHeight="1">
       <c r="A54" s="10" t="s">
         <v>180</v>
       </c>
@@ -5002,7 +5002,7 @@
       <c r="Z54" s="2"/>
       <c r="AA54" s="2"/>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" ht="15.75" hidden="1" customHeight="1">
       <c r="A55" s="10" t="s">
         <v>184</v>
       </c>
@@ -5065,7 +5065,7 @@
       <c r="Z55" s="2"/>
       <c r="AA55" s="2"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
+    <row r="56" ht="15.75" hidden="1" customHeight="1">
       <c r="A56" s="3" t="s">
         <v>188</v>
       </c>
@@ -5128,7 +5128,7 @@
       <c r="Z56" s="4"/>
       <c r="AA56" s="4"/>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" ht="15.75" hidden="1" customHeight="1">
       <c r="A57" s="3" t="s">
         <v>190</v>
       </c>
@@ -5189,7 +5189,7 @@
       <c r="Z57" s="4"/>
       <c r="AA57" s="4"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" ht="15.75" hidden="1" customHeight="1">
       <c r="A58" s="10" t="s">
         <v>191</v>
       </c>
@@ -5248,7 +5248,7 @@
       <c r="Z58" s="2"/>
       <c r="AA58" s="2"/>
     </row>
-    <row r="59" ht="15.75" hidden="1" customHeight="1">
+    <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="10" t="s">
         <v>194</v>
       </c>
@@ -5366,7 +5366,7 @@
       <c r="Z60" s="2"/>
       <c r="AA60" s="2"/>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
+    <row r="61" ht="15.75" hidden="1" customHeight="1">
       <c r="A61" s="10" t="s">
         <v>196</v>
       </c>
@@ -5429,7 +5429,7 @@
       <c r="Z61" s="2"/>
       <c r="AA61" s="2"/>
     </row>
-    <row r="62" ht="15.75" customHeight="1">
+    <row r="62" ht="15.75" hidden="1" customHeight="1">
       <c r="A62" s="10" t="s">
         <v>200</v>
       </c>
@@ -5490,7 +5490,7 @@
       <c r="Z62" s="2"/>
       <c r="AA62" s="2"/>
     </row>
-    <row r="63" ht="15.75" customHeight="1">
+    <row r="63" ht="15.75" hidden="1" customHeight="1">
       <c r="A63" s="9" t="s">
         <v>203</v>
       </c>
@@ -5553,7 +5553,7 @@
       <c r="Z63" s="4"/>
       <c r="AA63" s="4"/>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
+    <row r="64" ht="15.75" hidden="1" customHeight="1">
       <c r="A64" s="10" t="s">
         <v>204</v>
       </c>
@@ -5610,7 +5610,7 @@
       <c r="Z64" s="2"/>
       <c r="AA64" s="2"/>
     </row>
-    <row r="65" ht="15.75" hidden="1" customHeight="1">
+    <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="10" t="s">
         <v>205</v>
       </c>
@@ -5793,7 +5793,7 @@
       <c r="Z67" s="4"/>
       <c r="AA67" s="4"/>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68" ht="15.75" hidden="1" customHeight="1">
       <c r="A68" s="9" t="s">
         <v>212</v>
       </c>
@@ -5856,7 +5856,7 @@
       <c r="Z68" s="4"/>
       <c r="AA68" s="4"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
+    <row r="69" ht="15.75" hidden="1" customHeight="1">
       <c r="A69" s="3" t="s">
         <v>214</v>
       </c>
@@ -5919,7 +5919,7 @@
       <c r="Z69" s="4"/>
       <c r="AA69" s="4"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70" ht="15.75" hidden="1" customHeight="1">
       <c r="A70" s="10" t="s">
         <v>216</v>
       </c>
@@ -5982,7 +5982,7 @@
       <c r="Z70" s="2"/>
       <c r="AA70" s="2"/>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
+    <row r="71" ht="15.75" hidden="1" customHeight="1">
       <c r="A71" s="3" t="s">
         <v>217</v>
       </c>
@@ -6045,7 +6045,7 @@
       <c r="Z71" s="4"/>
       <c r="AA71" s="4"/>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
+    <row r="72" ht="15.75" hidden="1" customHeight="1">
       <c r="A72" s="3" t="s">
         <v>218</v>
       </c>
@@ -6108,7 +6108,7 @@
       <c r="Z72" s="4"/>
       <c r="AA72" s="4"/>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
+    <row r="73" ht="15.75" hidden="1" customHeight="1">
       <c r="A73" s="3" t="s">
         <v>219</v>
       </c>
@@ -6228,7 +6228,7 @@
       <c r="Z74" s="4"/>
       <c r="AA74" s="4"/>
     </row>
-    <row r="75" ht="15.75" hidden="1" customHeight="1">
+    <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="10" t="s">
         <v>221</v>
       </c>
@@ -6289,7 +6289,7 @@
       <c r="Z75" s="2"/>
       <c r="AA75" s="2"/>
     </row>
-    <row r="76" ht="15.75" hidden="1" customHeight="1">
+    <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="10" t="s">
         <v>223</v>
       </c>
@@ -6350,7 +6350,7 @@
       <c r="Z76" s="2"/>
       <c r="AA76" s="2"/>
     </row>
-    <row r="77" ht="15.75" hidden="1" customHeight="1">
+    <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="10" t="s">
         <v>224</v>
       </c>
@@ -6411,7 +6411,7 @@
       <c r="Z77" s="2"/>
       <c r="AA77" s="2"/>
     </row>
-    <row r="78" ht="15.75" hidden="1" customHeight="1">
+    <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="10" t="s">
         <v>226</v>
       </c>
@@ -6472,7 +6472,7 @@
       <c r="Z78" s="2"/>
       <c r="AA78" s="2"/>
     </row>
-    <row r="79" ht="15.75" hidden="1" customHeight="1">
+    <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="10" t="s">
         <v>227</v>
       </c>
@@ -6531,7 +6531,7 @@
       <c r="Z79" s="2"/>
       <c r="AA79" s="2"/>
     </row>
-    <row r="80" ht="15.75" hidden="1" customHeight="1">
+    <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="10" t="s">
         <v>229</v>
       </c>
@@ -6592,7 +6592,7 @@
       <c r="Z80" s="2"/>
       <c r="AA80" s="2"/>
     </row>
-    <row r="81" ht="15.75" hidden="1" customHeight="1">
+    <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="10" t="s">
         <v>230</v>
       </c>
@@ -7822,7 +7822,7 @@
       <c r="Z100" s="4"/>
       <c r="AA100" s="4"/>
     </row>
-    <row r="101" ht="15.75" hidden="1" customHeight="1">
+    <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="10" t="s">
         <v>268</v>
       </c>
@@ -8194,7 +8194,7 @@
       <c r="Z106" s="2"/>
       <c r="AA106" s="2"/>
     </row>
-    <row r="107" ht="15.75" customHeight="1">
+    <row r="107" ht="15.75" hidden="1" customHeight="1">
       <c r="A107" s="9" t="s">
         <v>278</v>
       </c>
@@ -8255,7 +8255,7 @@
       <c r="Z107" s="4"/>
       <c r="AA107" s="4"/>
     </row>
-    <row r="108" ht="15.75" customHeight="1">
+    <row r="108" ht="15.75" hidden="1" customHeight="1">
       <c r="A108" s="10" t="s">
         <v>280</v>
       </c>
@@ -8316,7 +8316,7 @@
       <c r="Z108" s="2"/>
       <c r="AA108" s="2"/>
     </row>
-    <row r="109" ht="15.75" customHeight="1">
+    <row r="109" ht="15.75" hidden="1" customHeight="1">
       <c r="A109" s="10" t="s">
         <v>281</v>
       </c>
@@ -8377,7 +8377,7 @@
       <c r="Z109" s="2"/>
       <c r="AA109" s="2"/>
     </row>
-    <row r="110" ht="15.75" customHeight="1">
+    <row r="110" ht="15.75" hidden="1" customHeight="1">
       <c r="A110" s="10" t="s">
         <v>282</v>
       </c>
@@ -8438,7 +8438,7 @@
       <c r="Z110" s="2"/>
       <c r="AA110" s="2"/>
     </row>
-    <row r="111" ht="15.75" customHeight="1">
+    <row r="111" ht="15.75" hidden="1" customHeight="1">
       <c r="A111" s="9" t="s">
         <v>284</v>
       </c>
@@ -9245,7 +9245,7 @@
       <c r="Z123" s="2"/>
       <c r="AA123" s="2"/>
     </row>
-    <row r="124" ht="15.75" hidden="1" customHeight="1">
+    <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="3" t="s">
         <v>309</v>
       </c>
@@ -9306,7 +9306,7 @@
       <c r="Z124" s="4"/>
       <c r="AA124" s="4"/>
     </row>
-    <row r="125" ht="15.75" hidden="1" customHeight="1">
+    <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="9" t="s">
         <v>311</v>
       </c>
@@ -34102,10 +34102,9 @@
     </row>
   </sheetData>
   <autoFilter ref="$A$1:$R$126">
-    <filterColumn colId="6">
+    <filterColumn colId="4">
       <filters>
-        <filter val="hinge"/>
-        <filter val="knee_flexion"/>
+        <filter val="core"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
etapa 6 fase 2 - decisao filtro familia inter virar soft
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -6,13 +6,11 @@
     <sheet state="visible" name="Exercícios" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="Referência" sheetId="2" r:id="rId5"/>
   </sheets>
-  <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Exercícios'!$A$1:$R$126</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="P7CRpCEH7pi8xg7pMdH5Wq/2F7xjlo75XoD+mcYA5ss="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="YQLHIDdezskgxttbnkXAk/HNc8GeKEH/oj2nLju6zos="/>
     </ext>
   </extLst>
 </workbook>
@@ -1832,7 +1830,7 @@
       <c r="Z2" s="4"/>
       <c r="AA2" s="4"/>
     </row>
-    <row r="3" hidden="1">
+    <row r="3">
       <c r="A3" s="10" t="s">
         <v>28</v>
       </c>
@@ -1893,7 +1891,7 @@
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
     </row>
-    <row r="4" hidden="1">
+    <row r="4">
       <c r="A4" s="10" t="s">
         <v>37</v>
       </c>
@@ -1954,7 +1952,7 @@
       <c r="Z4" s="2"/>
       <c r="AA4" s="2"/>
     </row>
-    <row r="5" hidden="1">
+    <row r="5">
       <c r="A5" s="9" t="s">
         <v>42</v>
       </c>
@@ -2015,7 +2013,7 @@
       <c r="Z5" s="4"/>
       <c r="AA5" s="4"/>
     </row>
-    <row r="6" hidden="1">
+    <row r="6">
       <c r="A6" s="10" t="s">
         <v>50</v>
       </c>
@@ -2074,7 +2072,7 @@
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
     </row>
-    <row r="7" hidden="1">
+    <row r="7">
       <c r="A7" s="10" t="s">
         <v>53</v>
       </c>
@@ -2135,7 +2133,7 @@
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
     </row>
-    <row r="8" hidden="1">
+    <row r="8">
       <c r="A8" s="10" t="s">
         <v>58</v>
       </c>
@@ -2196,7 +2194,7 @@
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
     </row>
-    <row r="9" hidden="1">
+    <row r="9">
       <c r="A9" s="10" t="s">
         <v>60</v>
       </c>
@@ -2257,7 +2255,7 @@
       <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
     </row>
-    <row r="10" hidden="1">
+    <row r="10">
       <c r="A10" s="10" t="s">
         <v>62</v>
       </c>
@@ -2318,7 +2316,7 @@
       <c r="Z10" s="2"/>
       <c r="AA10" s="2"/>
     </row>
-    <row r="11" hidden="1">
+    <row r="11">
       <c r="A11" s="10" t="s">
         <v>67</v>
       </c>
@@ -2379,7 +2377,7 @@
       <c r="Z11" s="2"/>
       <c r="AA11" s="2"/>
     </row>
-    <row r="12" hidden="1">
+    <row r="12">
       <c r="A12" s="10" t="s">
         <v>69</v>
       </c>
@@ -2438,7 +2436,7 @@
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
     </row>
-    <row r="13" hidden="1">
+    <row r="13">
       <c r="A13" s="3" t="s">
         <v>75</v>
       </c>
@@ -2497,7 +2495,7 @@
       <c r="Z13" s="4"/>
       <c r="AA13" s="4"/>
     </row>
-    <row r="14" hidden="1">
+    <row r="14">
       <c r="A14" s="9" t="s">
         <v>76</v>
       </c>
@@ -2556,7 +2554,7 @@
       <c r="Z14" s="4"/>
       <c r="AA14" s="4"/>
     </row>
-    <row r="15" hidden="1">
+    <row r="15">
       <c r="A15" s="10" t="s">
         <v>77</v>
       </c>
@@ -2617,7 +2615,7 @@
       <c r="Z15" s="2"/>
       <c r="AA15" s="2"/>
     </row>
-    <row r="16" hidden="1">
+    <row r="16">
       <c r="A16" s="10" t="s">
         <v>84</v>
       </c>
@@ -2678,7 +2676,7 @@
       <c r="Z16" s="2"/>
       <c r="AA16" s="2"/>
     </row>
-    <row r="17" hidden="1">
+    <row r="17">
       <c r="A17" s="10" t="s">
         <v>85</v>
       </c>
@@ -2739,7 +2737,7 @@
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
     </row>
-    <row r="18" hidden="1">
+    <row r="18">
       <c r="A18" s="10" t="s">
         <v>92</v>
       </c>
@@ -2802,7 +2800,7 @@
       <c r="Z18" s="2"/>
       <c r="AA18" s="2"/>
     </row>
-    <row r="19" ht="15.75" hidden="1" customHeight="1">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="9" t="s">
         <v>94</v>
       </c>
@@ -2863,7 +2861,7 @@
       <c r="Z19" s="4"/>
       <c r="AA19" s="4"/>
     </row>
-    <row r="20" ht="15.75" hidden="1" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="10" t="s">
         <v>95</v>
       </c>
@@ -2924,7 +2922,7 @@
       <c r="Z20" s="2"/>
       <c r="AA20" s="2"/>
     </row>
-    <row r="21" ht="15.75" hidden="1" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="10" t="s">
         <v>96</v>
       </c>
@@ -2985,7 +2983,7 @@
       <c r="Z21" s="2"/>
       <c r="AA21" s="2"/>
     </row>
-    <row r="22" ht="15.75" hidden="1" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="10" t="s">
         <v>97</v>
       </c>
@@ -3046,7 +3044,7 @@
       <c r="Z22" s="2"/>
       <c r="AA22" s="2"/>
     </row>
-    <row r="23" ht="15.75" hidden="1" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="10" t="s">
         <v>99</v>
       </c>
@@ -3105,7 +3103,7 @@
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
     </row>
-    <row r="24" ht="15.75" hidden="1" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="10" t="s">
         <v>102</v>
       </c>
@@ -3164,7 +3162,7 @@
       <c r="Z24" s="2"/>
       <c r="AA24" s="2"/>
     </row>
-    <row r="25" ht="15.75" hidden="1" customHeight="1">
+    <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="10" t="s">
         <v>106</v>
       </c>
@@ -3282,7 +3280,7 @@
       <c r="Z26" s="4"/>
       <c r="AA26" s="4"/>
     </row>
-    <row r="27" ht="15.75" hidden="1" customHeight="1">
+    <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="10" t="s">
         <v>113</v>
       </c>
@@ -3345,7 +3343,7 @@
       <c r="Z27" s="2"/>
       <c r="AA27" s="2"/>
     </row>
-    <row r="28" ht="15.75" hidden="1" customHeight="1">
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="10" t="s">
         <v>114</v>
       </c>
@@ -3406,7 +3404,7 @@
       <c r="Z28" s="2"/>
       <c r="AA28" s="2"/>
     </row>
-    <row r="29" ht="15.75" hidden="1" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="9" t="s">
         <v>118</v>
       </c>
@@ -3469,7 +3467,7 @@
       <c r="Z29" s="4"/>
       <c r="AA29" s="4"/>
     </row>
-    <row r="30" ht="15.75" hidden="1" customHeight="1">
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="10" t="s">
         <v>120</v>
       </c>
@@ -3532,7 +3530,7 @@
       <c r="Z30" s="2"/>
       <c r="AA30" s="2"/>
     </row>
-    <row r="31" ht="15.75" hidden="1" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>122</v>
       </c>
@@ -3959,7 +3957,7 @@
       <c r="Z37" s="2"/>
       <c r="AA37" s="2"/>
     </row>
-    <row r="38" ht="15.75" hidden="1" customHeight="1">
+    <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="10" t="s">
         <v>139</v>
       </c>
@@ -4022,7 +4020,7 @@
       <c r="Z38" s="2"/>
       <c r="AA38" s="2"/>
     </row>
-    <row r="39" ht="15.75" hidden="1" customHeight="1">
+    <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="9" t="s">
         <v>144</v>
       </c>
@@ -4085,7 +4083,7 @@
       <c r="Z39" s="4"/>
       <c r="AA39" s="4"/>
     </row>
-    <row r="40" ht="15.75" hidden="1" customHeight="1">
+    <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3" t="s">
         <v>147</v>
       </c>
@@ -4148,7 +4146,7 @@
       <c r="Z40" s="4"/>
       <c r="AA40" s="4"/>
     </row>
-    <row r="41" ht="15.75" hidden="1" customHeight="1">
+    <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="9" t="s">
         <v>149</v>
       </c>
@@ -4211,7 +4209,7 @@
       <c r="Z41" s="4"/>
       <c r="AA41" s="4"/>
     </row>
-    <row r="42" ht="15.75" hidden="1" customHeight="1">
+    <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="10" t="s">
         <v>151</v>
       </c>
@@ -4272,7 +4270,7 @@
       <c r="Z42" s="2"/>
       <c r="AA42" s="2"/>
     </row>
-    <row r="43" ht="15.75" hidden="1" customHeight="1">
+    <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="10" t="s">
         <v>152</v>
       </c>
@@ -4331,7 +4329,7 @@
       <c r="Z43" s="2"/>
       <c r="AA43" s="2"/>
     </row>
-    <row r="44" ht="15.75" hidden="1" customHeight="1">
+    <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="10" t="s">
         <v>155</v>
       </c>
@@ -4392,7 +4390,7 @@
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
     </row>
-    <row r="45" ht="15.75" hidden="1" customHeight="1">
+    <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="9" t="s">
         <v>161</v>
       </c>
@@ -4453,7 +4451,7 @@
       <c r="Z45" s="4"/>
       <c r="AA45" s="4"/>
     </row>
-    <row r="46" ht="15.75" hidden="1" customHeight="1">
+    <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="10" t="s">
         <v>165</v>
       </c>
@@ -4514,7 +4512,7 @@
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
     </row>
-    <row r="47" ht="15.75" hidden="1" customHeight="1">
+    <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="10" t="s">
         <v>166</v>
       </c>
@@ -4575,7 +4573,7 @@
       <c r="Z47" s="2"/>
       <c r="AA47" s="2"/>
     </row>
-    <row r="48" ht="15.75" hidden="1" customHeight="1">
+    <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="10" t="s">
         <v>169</v>
       </c>
@@ -4636,7 +4634,7 @@
       <c r="Z48" s="2"/>
       <c r="AA48" s="2"/>
     </row>
-    <row r="49" ht="15.75" hidden="1" customHeight="1">
+    <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="9" t="s">
         <v>170</v>
       </c>
@@ -4699,7 +4697,7 @@
       <c r="Z49" s="4"/>
       <c r="AA49" s="4"/>
     </row>
-    <row r="50" ht="15.75" hidden="1" customHeight="1">
+    <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="10" t="s">
         <v>171</v>
       </c>
@@ -4760,7 +4758,7 @@
       <c r="Z50" s="2"/>
       <c r="AA50" s="2"/>
     </row>
-    <row r="51" ht="15.75" hidden="1" customHeight="1">
+    <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="10" t="s">
         <v>172</v>
       </c>
@@ -4821,7 +4819,7 @@
       <c r="Z51" s="2"/>
       <c r="AA51" s="2"/>
     </row>
-    <row r="52" ht="15.75" hidden="1" customHeight="1">
+    <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="9" t="s">
         <v>175</v>
       </c>
@@ -4882,7 +4880,7 @@
       <c r="Z52" s="4"/>
       <c r="AA52" s="4"/>
     </row>
-    <row r="53" ht="15.75" hidden="1" customHeight="1">
+    <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="3" t="s">
         <v>178</v>
       </c>
@@ -4943,7 +4941,7 @@
       <c r="Z53" s="4"/>
       <c r="AA53" s="4"/>
     </row>
-    <row r="54" ht="15.75" hidden="1" customHeight="1">
+    <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="10" t="s">
         <v>180</v>
       </c>
@@ -5002,7 +5000,7 @@
       <c r="Z54" s="2"/>
       <c r="AA54" s="2"/>
     </row>
-    <row r="55" ht="15.75" hidden="1" customHeight="1">
+    <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="10" t="s">
         <v>184</v>
       </c>
@@ -5065,7 +5063,7 @@
       <c r="Z55" s="2"/>
       <c r="AA55" s="2"/>
     </row>
-    <row r="56" ht="15.75" hidden="1" customHeight="1">
+    <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="3" t="s">
         <v>188</v>
       </c>
@@ -5128,7 +5126,7 @@
       <c r="Z56" s="4"/>
       <c r="AA56" s="4"/>
     </row>
-    <row r="57" ht="15.75" hidden="1" customHeight="1">
+    <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="3" t="s">
         <v>190</v>
       </c>
@@ -5189,7 +5187,7 @@
       <c r="Z57" s="4"/>
       <c r="AA57" s="4"/>
     </row>
-    <row r="58" ht="15.75" hidden="1" customHeight="1">
+    <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="10" t="s">
         <v>191</v>
       </c>
@@ -5307,7 +5305,7 @@
       <c r="Z59" s="2"/>
       <c r="AA59" s="2"/>
     </row>
-    <row r="60" ht="15.75" hidden="1" customHeight="1">
+    <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="10" t="s">
         <v>195</v>
       </c>
@@ -5366,7 +5364,7 @@
       <c r="Z60" s="2"/>
       <c r="AA60" s="2"/>
     </row>
-    <row r="61" ht="15.75" hidden="1" customHeight="1">
+    <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="10" t="s">
         <v>196</v>
       </c>
@@ -5429,7 +5427,7 @@
       <c r="Z61" s="2"/>
       <c r="AA61" s="2"/>
     </row>
-    <row r="62" ht="15.75" hidden="1" customHeight="1">
+    <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="10" t="s">
         <v>200</v>
       </c>
@@ -5490,7 +5488,7 @@
       <c r="Z62" s="2"/>
       <c r="AA62" s="2"/>
     </row>
-    <row r="63" ht="15.75" hidden="1" customHeight="1">
+    <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="9" t="s">
         <v>203</v>
       </c>
@@ -5553,7 +5551,7 @@
       <c r="Z63" s="4"/>
       <c r="AA63" s="4"/>
     </row>
-    <row r="64" ht="15.75" hidden="1" customHeight="1">
+    <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="10" t="s">
         <v>204</v>
       </c>
@@ -5669,7 +5667,7 @@
       <c r="Z65" s="2"/>
       <c r="AA65" s="2"/>
     </row>
-    <row r="66" ht="15.75" hidden="1" customHeight="1">
+    <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="3" t="s">
         <v>208</v>
       </c>
@@ -5730,7 +5728,7 @@
       <c r="Z66" s="4"/>
       <c r="AA66" s="4"/>
     </row>
-    <row r="67" ht="15.75" hidden="1" customHeight="1">
+    <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="3" t="s">
         <v>210</v>
       </c>
@@ -5793,7 +5791,7 @@
       <c r="Z67" s="4"/>
       <c r="AA67" s="4"/>
     </row>
-    <row r="68" ht="15.75" hidden="1" customHeight="1">
+    <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="9" t="s">
         <v>212</v>
       </c>
@@ -5856,7 +5854,7 @@
       <c r="Z68" s="4"/>
       <c r="AA68" s="4"/>
     </row>
-    <row r="69" ht="15.75" hidden="1" customHeight="1">
+    <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="3" t="s">
         <v>214</v>
       </c>
@@ -5919,7 +5917,7 @@
       <c r="Z69" s="4"/>
       <c r="AA69" s="4"/>
     </row>
-    <row r="70" ht="15.75" hidden="1" customHeight="1">
+    <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="10" t="s">
         <v>216</v>
       </c>
@@ -5982,7 +5980,7 @@
       <c r="Z70" s="2"/>
       <c r="AA70" s="2"/>
     </row>
-    <row r="71" ht="15.75" hidden="1" customHeight="1">
+    <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="3" t="s">
         <v>217</v>
       </c>
@@ -6045,7 +6043,7 @@
       <c r="Z71" s="4"/>
       <c r="AA71" s="4"/>
     </row>
-    <row r="72" ht="15.75" hidden="1" customHeight="1">
+    <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="3" t="s">
         <v>218</v>
       </c>
@@ -6108,7 +6106,7 @@
       <c r="Z72" s="4"/>
       <c r="AA72" s="4"/>
     </row>
-    <row r="73" ht="15.75" hidden="1" customHeight="1">
+    <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="3" t="s">
         <v>219</v>
       </c>
@@ -6169,7 +6167,7 @@
       <c r="Z73" s="4"/>
       <c r="AA73" s="4"/>
     </row>
-    <row r="74" ht="15.75" hidden="1" customHeight="1">
+    <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="9" t="s">
         <v>220</v>
       </c>
@@ -6653,7 +6651,7 @@
       <c r="Z81" s="2"/>
       <c r="AA81" s="2"/>
     </row>
-    <row r="82" ht="15.75" hidden="1" customHeight="1">
+    <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="9" t="s">
         <v>231</v>
       </c>
@@ -6716,7 +6714,7 @@
       <c r="Z82" s="4"/>
       <c r="AA82" s="4"/>
     </row>
-    <row r="83" ht="15.75" hidden="1" customHeight="1">
+    <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="10" t="s">
         <v>234</v>
       </c>
@@ -6777,7 +6775,7 @@
       <c r="Z83" s="2"/>
       <c r="AA83" s="2"/>
     </row>
-    <row r="84" ht="15.75" hidden="1" customHeight="1">
+    <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="10" t="s">
         <v>235</v>
       </c>
@@ -6840,7 +6838,7 @@
       <c r="Z84" s="2"/>
       <c r="AA84" s="2"/>
     </row>
-    <row r="85" ht="15.75" hidden="1" customHeight="1">
+    <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="10" t="s">
         <v>239</v>
       </c>
@@ -6903,7 +6901,7 @@
       <c r="Z85" s="2"/>
       <c r="AA85" s="2"/>
     </row>
-    <row r="86" ht="15.75" hidden="1" customHeight="1">
+    <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="10" t="s">
         <v>241</v>
       </c>
@@ -6964,7 +6962,7 @@
       <c r="Z86" s="2"/>
       <c r="AA86" s="2"/>
     </row>
-    <row r="87" ht="15.75" hidden="1" customHeight="1">
+    <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="3" t="s">
         <v>242</v>
       </c>
@@ -7025,7 +7023,7 @@
       <c r="Z87" s="4"/>
       <c r="AA87" s="4"/>
     </row>
-    <row r="88" ht="15.75" hidden="1" customHeight="1">
+    <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="9" t="s">
         <v>243</v>
       </c>
@@ -7086,7 +7084,7 @@
       <c r="Z88" s="4"/>
       <c r="AA88" s="4"/>
     </row>
-    <row r="89" ht="15.75" hidden="1" customHeight="1">
+    <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="3" t="s">
         <v>244</v>
       </c>
@@ -7147,7 +7145,7 @@
       <c r="Z89" s="4"/>
       <c r="AA89" s="4"/>
     </row>
-    <row r="90" ht="15.75" hidden="1" customHeight="1">
+    <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="10" t="s">
         <v>245</v>
       </c>
@@ -7206,7 +7204,7 @@
       <c r="Z90" s="2"/>
       <c r="AA90" s="2"/>
     </row>
-    <row r="91" ht="15.75" hidden="1" customHeight="1">
+    <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="10" t="s">
         <v>250</v>
       </c>
@@ -7269,7 +7267,7 @@
       <c r="Z91" s="2"/>
       <c r="AA91" s="2"/>
     </row>
-    <row r="92" ht="15.75" hidden="1" customHeight="1">
+    <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="10" t="s">
         <v>253</v>
       </c>
@@ -7332,7 +7330,7 @@
       <c r="Z92" s="2"/>
       <c r="AA92" s="2"/>
     </row>
-    <row r="93" ht="15.75" hidden="1" customHeight="1">
+    <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="10" t="s">
         <v>255</v>
       </c>
@@ -7395,7 +7393,7 @@
       <c r="Z93" s="2"/>
       <c r="AA93" s="2"/>
     </row>
-    <row r="94" ht="15.75" hidden="1" customHeight="1">
+    <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="10" t="s">
         <v>257</v>
       </c>
@@ -7456,7 +7454,7 @@
       <c r="Z94" s="2"/>
       <c r="AA94" s="2"/>
     </row>
-    <row r="95" ht="15.75" hidden="1" customHeight="1">
+    <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="3" t="s">
         <v>259</v>
       </c>
@@ -7517,7 +7515,7 @@
       <c r="Z95" s="4"/>
       <c r="AA95" s="4"/>
     </row>
-    <row r="96" ht="15.75" hidden="1" customHeight="1">
+    <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="9" t="s">
         <v>260</v>
       </c>
@@ -7578,7 +7576,7 @@
       <c r="Z96" s="4"/>
       <c r="AA96" s="4"/>
     </row>
-    <row r="97" ht="15.75" hidden="1" customHeight="1">
+    <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="10" t="s">
         <v>262</v>
       </c>
@@ -7641,7 +7639,7 @@
       <c r="Z97" s="2"/>
       <c r="AA97" s="2"/>
     </row>
-    <row r="98" ht="15.75" hidden="1" customHeight="1">
+    <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="9" t="s">
         <v>264</v>
       </c>
@@ -7700,7 +7698,7 @@
       <c r="Z98" s="4"/>
       <c r="AA98" s="4"/>
     </row>
-    <row r="99" ht="15.75" hidden="1" customHeight="1">
+    <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="9" t="s">
         <v>265</v>
       </c>
@@ -7761,7 +7759,7 @@
       <c r="Z99" s="4"/>
       <c r="AA99" s="4"/>
     </row>
-    <row r="100" ht="15.75" hidden="1" customHeight="1">
+    <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="9" t="s">
         <v>266</v>
       </c>
@@ -7883,7 +7881,7 @@
       <c r="Z101" s="2"/>
       <c r="AA101" s="2"/>
     </row>
-    <row r="102" ht="15.75" hidden="1" customHeight="1">
+    <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="3" t="s">
         <v>270</v>
       </c>
@@ -7946,7 +7944,7 @@
       <c r="Z102" s="4"/>
       <c r="AA102" s="4"/>
     </row>
-    <row r="103" ht="15.75" hidden="1" customHeight="1">
+    <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="10" t="s">
         <v>271</v>
       </c>
@@ -8007,7 +8005,7 @@
       <c r="Z103" s="2"/>
       <c r="AA103" s="2"/>
     </row>
-    <row r="104" ht="15.75" hidden="1" customHeight="1">
+    <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="10" t="s">
         <v>272</v>
       </c>
@@ -8068,7 +8066,7 @@
       <c r="Z104" s="2"/>
       <c r="AA104" s="2"/>
     </row>
-    <row r="105" ht="15.75" hidden="1" customHeight="1">
+    <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="10" t="s">
         <v>274</v>
       </c>
@@ -8131,7 +8129,7 @@
       <c r="Z105" s="2"/>
       <c r="AA105" s="2"/>
     </row>
-    <row r="106" ht="15.75" hidden="1" customHeight="1">
+    <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="10" t="s">
         <v>277</v>
       </c>
@@ -8194,7 +8192,7 @@
       <c r="Z106" s="2"/>
       <c r="AA106" s="2"/>
     </row>
-    <row r="107" ht="15.75" hidden="1" customHeight="1">
+    <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="9" t="s">
         <v>278</v>
       </c>
@@ -8255,7 +8253,7 @@
       <c r="Z107" s="4"/>
       <c r="AA107" s="4"/>
     </row>
-    <row r="108" ht="15.75" hidden="1" customHeight="1">
+    <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="10" t="s">
         <v>280</v>
       </c>
@@ -8316,7 +8314,7 @@
       <c r="Z108" s="2"/>
       <c r="AA108" s="2"/>
     </row>
-    <row r="109" ht="15.75" hidden="1" customHeight="1">
+    <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="10" t="s">
         <v>281</v>
       </c>
@@ -8377,7 +8375,7 @@
       <c r="Z109" s="2"/>
       <c r="AA109" s="2"/>
     </row>
-    <row r="110" ht="15.75" hidden="1" customHeight="1">
+    <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="10" t="s">
         <v>282</v>
       </c>
@@ -8438,7 +8436,7 @@
       <c r="Z110" s="2"/>
       <c r="AA110" s="2"/>
     </row>
-    <row r="111" ht="15.75" hidden="1" customHeight="1">
+    <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="9" t="s">
         <v>284</v>
       </c>
@@ -8499,7 +8497,7 @@
       <c r="Z111" s="4"/>
       <c r="AA111" s="4"/>
     </row>
-    <row r="112" ht="15.75" hidden="1" customHeight="1">
+    <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="9" t="s">
         <v>285</v>
       </c>
@@ -8562,7 +8560,7 @@
       <c r="Z112" s="4"/>
       <c r="AA112" s="4"/>
     </row>
-    <row r="113" ht="15.75" hidden="1" customHeight="1">
+    <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="10" t="s">
         <v>288</v>
       </c>
@@ -8625,7 +8623,7 @@
       <c r="Z113" s="2"/>
       <c r="AA113" s="2"/>
     </row>
-    <row r="114" ht="15.75" hidden="1" customHeight="1">
+    <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="10" t="s">
         <v>289</v>
       </c>
@@ -8688,7 +8686,7 @@
       <c r="Z114" s="2"/>
       <c r="AA114" s="2"/>
     </row>
-    <row r="115" ht="15.75" hidden="1" customHeight="1">
+    <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="10" t="s">
         <v>290</v>
       </c>
@@ -8751,7 +8749,7 @@
       <c r="Z115" s="2"/>
       <c r="AA115" s="2"/>
     </row>
-    <row r="116" ht="15.75" hidden="1" customHeight="1">
+    <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="10" t="s">
         <v>291</v>
       </c>
@@ -8812,7 +8810,7 @@
       <c r="Z116" s="2"/>
       <c r="AA116" s="2"/>
     </row>
-    <row r="117" ht="15.75" hidden="1" customHeight="1">
+    <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="9" t="s">
         <v>296</v>
       </c>
@@ -8873,7 +8871,7 @@
       <c r="Z117" s="4"/>
       <c r="AA117" s="4"/>
     </row>
-    <row r="118" ht="15.75" hidden="1" customHeight="1">
+    <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="63" t="s">
         <v>298</v>
       </c>
@@ -8936,7 +8934,7 @@
       <c r="Z118" s="2"/>
       <c r="AA118" s="2"/>
     </row>
-    <row r="119" ht="15.75" hidden="1" customHeight="1">
+    <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="63" t="s">
         <v>301</v>
       </c>
@@ -8997,7 +8995,7 @@
       <c r="Z119" s="2"/>
       <c r="AA119" s="2"/>
     </row>
-    <row r="120" ht="15.75" hidden="1" customHeight="1">
+    <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="10" t="s">
         <v>302</v>
       </c>
@@ -9058,7 +9056,7 @@
       <c r="Z120" s="2"/>
       <c r="AA120" s="2"/>
     </row>
-    <row r="121" ht="15.75" hidden="1" customHeight="1">
+    <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="10" t="s">
         <v>304</v>
       </c>
@@ -9121,7 +9119,7 @@
       <c r="Z121" s="2"/>
       <c r="AA121" s="2"/>
     </row>
-    <row r="122" ht="15.75" hidden="1" customHeight="1">
+    <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="10" t="s">
         <v>306</v>
       </c>
@@ -9184,7 +9182,7 @@
       <c r="Z122" s="2"/>
       <c r="AA122" s="2"/>
     </row>
-    <row r="123" ht="15.75" hidden="1" customHeight="1">
+    <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="63" t="s">
         <v>308</v>
       </c>
@@ -9367,7 +9365,7 @@
       <c r="Z125" s="4"/>
       <c r="AA125" s="4"/>
     </row>
-    <row r="126" ht="15.75" hidden="1" customHeight="1">
+    <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="3" t="s">
         <v>312</v>
       </c>
@@ -34101,13 +34099,6 @@
       <c r="Z1000" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$R$126">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="core"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <conditionalFormatting sqref="E2:E126">
     <cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="co">
       <formula>LEFT((E2),LEN("co"))=("co")</formula>

</xml_diff>

<commit_message>
Fase 4.2-B — Annexo 4.1 items 3+13: purpose + split família prancha
Item 3: Slide Board Lateral
  purpose: 'explosive' → 'compound'
  (deslizamento lateral unilateral = composto, não explosivo)

Item 13: 7 pranchas frontais + 1 lateral
  Prancha / Alternada / Bola / Feijao / Renegade / Slideboard:
    variacao_de: 'prancha' → 'prancha frontal'
  Prancha Lateral:
    variacao_de: 'prancha' → 'prancha lateral'

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -5930,7 +5930,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha frontal</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6004,7 +6004,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha frontal</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha frontal</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6152,7 +6152,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha frontal</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha lateral</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha frontal</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>prancha</t>
+          <t>prancha frontal</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -8122,7 +8122,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>explosive</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">

</xml_diff>

<commit_message>
Fase 4 Sub-C — setup estrutural: 5 colunas dim + loader ativo/variante_pontual
XLSX: colunas pegada, plano_corporal, equipamento_grupo, variante_pontual, ativo
adicionadas como vazias (18 → 23 cols). gerador_treino.py: helper _bool_xlsx,
campo Exercicio.ativo (default True), carregar_banco() lê variante_pontual +
ativo e filtra inativos. NO-OP confirmado: 175 passed, 13 snapshots, harness
16/16 OK (4.1 = 21.54% informativo, inalterado).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R126"/>
+  <dimension ref="A1:W126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,6 +507,31 @@
           <t>demanda_core</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>pegada</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>plano_corporal</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>equipamento_grupo</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>variante_pontual</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ativo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -524,7 +549,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>core</t>
@@ -571,7 +595,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
@@ -598,7 +621,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>lower</t>
@@ -645,7 +667,6 @@
           <t>glúteo médio</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>1</v>
       </c>
@@ -672,7 +693,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>lower</t>
@@ -719,7 +739,6 @@
           <t>adutores</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>1</v>
       </c>
@@ -746,7 +765,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>lower</t>
@@ -793,7 +811,6 @@
           <t>adutores, glúteo médio</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>1</v>
       </c>
@@ -810,13 +827,11 @@
           <t>Agachamento Búlgaro</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>lower</t>
@@ -863,7 +878,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>1</v>
       </c>
@@ -890,7 +904,6 @@
           <t>Halter</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>lower</t>
@@ -937,7 +950,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>1</v>
       </c>
@@ -964,7 +976,6 @@
           <t>Rack + barra olímpica</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>lower</t>
@@ -1011,7 +1022,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>1</v>
       </c>
@@ -1038,7 +1048,6 @@
           <t>Barra Smith (crossover)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>lower</t>
@@ -1085,7 +1094,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>1</v>
       </c>
@@ -1112,7 +1120,6 @@
           <t>Air Bike</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>cardio</t>
@@ -1159,7 +1166,6 @@
           <t>full body, cardiovascular</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>1</v>
       </c>
@@ -1186,7 +1192,6 @@
           <t>Air Bike</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>cardio</t>
@@ -1233,7 +1238,6 @@
           <t>full body, cardiovascular</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>1</v>
       </c>
@@ -1255,8 +1259,6 @@
           <t>Apoio</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1303,7 +1305,6 @@
           <t>peitoral, tríceps</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>0</v>
       </c>
@@ -1325,8 +1326,6 @@
           <t>Apoio</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1373,7 +1372,6 @@
           <t>peitoral, tríceps</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
         <v>0</v>
       </c>
@@ -1395,8 +1393,6 @@
           <t>Apoio</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1443,7 +1439,6 @@
           <t>peitoral, tríceps</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>0</v>
       </c>
@@ -1470,7 +1465,6 @@
           <t>Barra fixa (crossover)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1517,7 +1511,6 @@
           <t>dorsal, bíceps</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>3</v>
       </c>
@@ -1544,7 +1537,6 @@
           <t>Barra fixa (crossover)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1591,7 +1583,6 @@
           <t>dorsal, bíceps</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
         <v>3</v>
       </c>
@@ -1618,7 +1609,6 @@
           <t>Barra olímpica</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1665,7 +1655,6 @@
           <t>bíceps</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>1</v>
       </c>
@@ -1743,7 +1732,6 @@
           <t>bíceps</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>1</v>
       </c>
@@ -1770,7 +1758,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1817,7 +1804,6 @@
           <t>bíceps</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>1</v>
       </c>
@@ -1844,7 +1830,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1891,7 +1876,6 @@
           <t>bíceps</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>1</v>
       </c>
@@ -1918,7 +1902,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>upper</t>
@@ -1965,7 +1948,6 @@
           <t>bíceps</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>1</v>
       </c>
@@ -1992,7 +1974,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>upper</t>
@@ -2039,7 +2020,6 @@
           <t>bíceps, braquiorradial</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>1</v>
       </c>
@@ -2056,13 +2036,11 @@
           <t>Box Jump</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Caixa pliométrica</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>lower</t>
@@ -2109,7 +2087,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
@@ -2126,13 +2103,11 @@
           <t>Cadeira Extensora</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Cadeira extensora</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>lower</t>
@@ -2179,7 +2154,6 @@
           <t>quadríceps</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>0</v>
       </c>
@@ -2196,13 +2170,11 @@
           <t>Cadeira Flexora</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Cadeira flexora</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>lower</t>
@@ -2249,7 +2221,6 @@
           <t>isquiotibiais</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
         <v>0</v>
       </c>
@@ -2266,13 +2237,11 @@
           <t>Canoinha</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Banco</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>core</t>
@@ -2319,7 +2288,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
         <v>0</v>
       </c>
@@ -2397,7 +2365,6 @@
           <t>adutores</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
         <v>0</v>
       </c>
@@ -2424,7 +2391,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>upper</t>
@@ -2471,7 +2437,6 @@
           <t>peitoral</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
         <v>1</v>
       </c>
@@ -2549,7 +2514,6 @@
           <t>peitoral</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
         <v>1</v>
       </c>
@@ -2627,7 +2591,6 @@
           <t>peitoral</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
         <v>1</v>
       </c>
@@ -2644,13 +2607,11 @@
           <t>Crucifíxo Invertido</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>upper</t>
@@ -2697,7 +2658,6 @@
           <t>deltóide posterior</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="n">
         <v>1</v>
       </c>
@@ -2724,7 +2684,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>core</t>
@@ -2771,7 +2730,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="n">
         <v>0</v>
       </c>
@@ -2798,7 +2756,6 @@
           <t>Bola</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>core</t>
@@ -2845,7 +2802,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
         <v>0</v>
       </c>
@@ -2872,7 +2828,6 @@
           <t>Polia</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>core</t>
@@ -2919,7 +2874,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="n">
         <v>1</v>
       </c>
@@ -2946,7 +2900,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>core</t>
@@ -2993,7 +2946,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="n">
         <v>0</v>
       </c>
@@ -3071,7 +3023,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="n">
         <v>1</v>
       </c>
@@ -3098,7 +3049,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>core</t>
@@ -3145,7 +3095,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="n">
         <v>0</v>
       </c>
@@ -3223,7 +3172,6 @@
           <t>deltóide, tríceps</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="n">
         <v>1</v>
       </c>
@@ -3301,7 +3249,6 @@
           <t>deltóide, tríceps</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="n">
         <v>1</v>
       </c>
@@ -3379,7 +3326,6 @@
           <t>deltóide, tríceps</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="n">
         <v>1</v>
       </c>
@@ -3457,7 +3403,6 @@
           <t>deltóide, tríceps</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="n">
         <v>1</v>
       </c>
@@ -3484,7 +3429,6 @@
           <t>Barra Smith (crossover)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>upper</t>
@@ -3531,7 +3475,6 @@
           <t>deltóide, tríceps</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="n">
         <v>1</v>
       </c>
@@ -3548,13 +3491,11 @@
           <t>Desloc. Lateral c/ Band</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>Glute band</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>lower</t>
@@ -3601,7 +3542,6 @@
           <t>glúteo médio</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="n">
         <v>0</v>
       </c>
@@ -3628,7 +3568,6 @@
           <t>Rack</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>lower</t>
@@ -3675,7 +3614,6 @@
           <t>gastrocnêmio</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
         <v>0</v>
       </c>
@@ -3702,7 +3640,6 @@
           <t>Anilha</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>upper</t>
@@ -3749,7 +3686,6 @@
           <t>deltóide anterior</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="n">
         <v>1</v>
       </c>
@@ -3776,7 +3712,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>upper</t>
@@ -3823,7 +3758,6 @@
           <t>deltóide anterior</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="n">
         <v>1</v>
       </c>
@@ -3850,7 +3784,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>upper</t>
@@ -3897,7 +3830,6 @@
           <t>deltóide lateral</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
         <v>1</v>
       </c>
@@ -3924,7 +3856,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>upper</t>
@@ -3971,7 +3902,6 @@
           <t>deltóide lateral</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
         <v>1</v>
       </c>
@@ -4049,7 +3979,6 @@
           <t>deltóide lateral</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
         <v>1</v>
       </c>
@@ -4076,7 +4005,6 @@
           <t>Rack</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>lower</t>
@@ -4123,7 +4051,6 @@
           <t>gastrocnêmio</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
         <v>0</v>
       </c>
@@ -4140,7 +4067,6 @@
           <t>Face Pull (Polia)</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>Crossover</t>
@@ -4197,7 +4123,6 @@
           <t>deltóide posterior, manguito</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="n">
         <v>1</v>
       </c>
@@ -4224,7 +4149,6 @@
           <t>feijao</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>lower</t>
@@ -4271,7 +4195,6 @@
           <t>isquiotibiais</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" t="n">
         <v>0</v>
       </c>
@@ -4298,7 +4221,6 @@
           <t>slideboard</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>lower</t>
@@ -4345,7 +4267,6 @@
           <t>isquiotibiais</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
       <c r="P53" t="n">
         <v>0</v>
       </c>
@@ -4372,7 +4293,6 @@
           <t>Barra olímpica</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>lower</t>
@@ -4419,7 +4339,6 @@
           <t>isquiotibiais, eretores</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
       <c r="P54" t="n">
         <v>0</v>
       </c>
@@ -4497,7 +4416,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
       <c r="P55" t="n">
         <v>0</v>
       </c>
@@ -4575,7 +4493,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
       <c r="P56" t="n">
         <v>0</v>
       </c>
@@ -4597,7 +4514,6 @@
           <t>Hip thrust</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Colchonete</t>
@@ -4649,7 +4565,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr"/>
       <c r="P57" t="n">
         <v>0</v>
       </c>
@@ -4666,13 +4581,11 @@
           <t>Hiperextensão 45°</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>Banco romano</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>lower</t>
@@ -4719,7 +4632,6 @@
           <t>eretores, glúteos, isquios</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
       <c r="P58" t="n">
         <v>0</v>
       </c>
@@ -4736,13 +4648,11 @@
           <t>Hollow Hold</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>core</t>
@@ -4789,7 +4699,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
       <c r="P59" t="n">
         <v>0</v>
       </c>
@@ -4806,13 +4715,11 @@
           <t>Leg Press</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>Leg Press</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>lower</t>
@@ -4859,7 +4766,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
       <c r="P60" t="n">
         <v>0</v>
       </c>
@@ -4937,7 +4843,6 @@
           <t>isquiotibiais, glúteos, eretores</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
       <c r="P61" t="n">
         <v>3</v>
       </c>
@@ -4964,7 +4869,6 @@
           <t>suporte anilhas</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>lower</t>
@@ -5011,7 +4915,6 @@
           <t>isquiotibiais, glúteos</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
       <c r="P62" t="n">
         <v>2</v>
       </c>
@@ -5089,7 +4992,6 @@
           <t>isquiotibiais, glúteos, eretores</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr"/>
       <c r="P63" t="n">
         <v>3</v>
       </c>
@@ -5106,9 +5008,6 @@
           <t>Nordic Curl</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>lower</t>
@@ -5155,7 +5054,6 @@
           <t>isquiotibiais</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr"/>
       <c r="P64" t="n">
         <v>0</v>
       </c>
@@ -5172,13 +5070,11 @@
           <t>Pallof Press</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>core</t>
@@ -5225,7 +5121,6 @@
           <t>core anti-rotação</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr"/>
       <c r="P65" t="n">
         <v>1</v>
       </c>
@@ -5252,7 +5147,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>lower</t>
@@ -5299,7 +5193,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
       <c r="P66" t="n">
         <v>1</v>
       </c>
@@ -5377,7 +5270,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr"/>
       <c r="P67" t="n">
         <v>1</v>
       </c>
@@ -5455,7 +5347,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr"/>
       <c r="P68" t="n">
         <v>0</v>
       </c>
@@ -5533,7 +5424,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr"/>
       <c r="P69" t="n">
         <v>0</v>
       </c>
@@ -5611,7 +5501,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr"/>
       <c r="P70" t="n">
         <v>0</v>
       </c>
@@ -5689,7 +5578,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr"/>
       <c r="P71" t="n">
         <v>0</v>
       </c>
@@ -5767,7 +5655,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr"/>
       <c r="P72" t="n">
         <v>0</v>
       </c>
@@ -5789,7 +5676,6 @@
           <t>ponte</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>Colchonete</t>
@@ -5841,7 +5727,6 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr"/>
       <c r="P73" t="n">
         <v>0</v>
       </c>
@@ -5858,13 +5743,11 @@
           <t>Posterior Ombro Polia</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>Polia</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
           <t>upper</t>
@@ -5911,7 +5794,6 @@
           <t>deltóide posterior</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr"/>
       <c r="P74" t="n">
         <v>1</v>
       </c>
@@ -5938,7 +5820,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
           <t>core</t>
@@ -5985,7 +5866,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr"/>
       <c r="P75" t="n">
         <v>0</v>
       </c>
@@ -6012,7 +5892,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
           <t>core</t>
@@ -6059,7 +5938,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr"/>
       <c r="P76" t="n">
         <v>0</v>
       </c>
@@ -6086,7 +5964,6 @@
           <t>bola</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>core</t>
@@ -6133,7 +6010,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr"/>
       <c r="P77" t="n">
         <v>0</v>
       </c>
@@ -6160,7 +6036,6 @@
           <t>feijao</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>core</t>
@@ -6207,7 +6082,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr"/>
       <c r="P78" t="n">
         <v>0</v>
       </c>
@@ -6234,7 +6108,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>core</t>
@@ -6271,13 +6144,11 @@
           <t>não</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr">
         <is>
           <t>oblíquos</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr"/>
       <c r="P79" t="n">
         <v>0</v>
       </c>
@@ -6304,7 +6175,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>core</t>
@@ -6351,7 +6221,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr"/>
       <c r="P80" t="n">
         <v>1</v>
       </c>
@@ -6373,7 +6242,6 @@
           <t>prancha frontal</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>slideboard</t>
@@ -6425,7 +6293,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr"/>
       <c r="P81" t="n">
         <v>0</v>
       </c>
@@ -6503,7 +6370,6 @@
           <t>dorsal, serrátil</t>
         </is>
       </c>
-      <c r="O82" t="inlineStr"/>
       <c r="P82" t="n">
         <v>1</v>
       </c>
@@ -6530,7 +6396,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>upper</t>
@@ -6577,7 +6442,6 @@
           <t>dorsal, serrátil</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr"/>
       <c r="P83" t="n">
         <v>1</v>
       </c>
@@ -6655,7 +6519,6 @@
           <t>dorsal, bíceps</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr"/>
       <c r="P84" t="n">
         <v>2</v>
       </c>
@@ -6733,7 +6596,6 @@
           <t>dorsal, bíceps</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr"/>
       <c r="P85" t="n">
         <v>2</v>
       </c>
@@ -6760,7 +6622,6 @@
           <t xml:space="preserve">Puxada </t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>upper</t>
@@ -6807,7 +6668,6 @@
           <t>dorsal, bíceps</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr"/>
       <c r="P86" t="n">
         <v>2</v>
       </c>
@@ -6834,7 +6694,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>lower</t>
@@ -6881,7 +6740,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr"/>
       <c r="P87" t="n">
         <v>1</v>
       </c>
@@ -6908,7 +6766,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>lower</t>
@@ -6955,7 +6812,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr"/>
       <c r="P88" t="n">
         <v>1</v>
       </c>
@@ -6982,7 +6838,6 @@
           <t>Barra</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>lower</t>
@@ -7029,7 +6884,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr"/>
       <c r="P89" t="n">
         <v>0</v>
       </c>
@@ -7051,8 +6905,6 @@
           <t>trx</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7099,7 +6951,6 @@
           <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr"/>
       <c r="P90" t="n">
         <v>2</v>
       </c>
@@ -7177,7 +7028,6 @@
           <t>dorsal, romboides</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="n">
         <v>2</v>
       </c>
@@ -7255,7 +7105,6 @@
           <t>dorsal, romboides</t>
         </is>
       </c>
-      <c r="O92" t="inlineStr"/>
       <c r="P92" t="n">
         <v>3</v>
       </c>
@@ -7333,7 +7182,6 @@
           <t>dorsal, romboides</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr"/>
       <c r="P93" t="n">
         <v>3</v>
       </c>
@@ -7360,7 +7208,6 @@
           <t>Barra olímpica</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7407,7 +7254,6 @@
           <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr"/>
       <c r="P94" t="n">
         <v>3</v>
       </c>
@@ -7434,7 +7280,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7481,7 +7326,6 @@
           <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr"/>
       <c r="P95" t="n">
         <v>2</v>
       </c>
@@ -7508,7 +7352,6 @@
           <t>barra smith</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7555,7 +7398,6 @@
           <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
-      <c r="O96" t="inlineStr"/>
       <c r="P96" t="n">
         <v>2</v>
       </c>
@@ -7633,7 +7475,6 @@
           <t>dorsal, romboides</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr"/>
       <c r="P97" t="n">
         <v>3</v>
       </c>
@@ -7655,8 +7496,6 @@
           <t>trx</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7703,7 +7542,6 @@
           <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr"/>
       <c r="P98" t="n">
         <v>2</v>
       </c>
@@ -7730,7 +7568,6 @@
           <t>Banco reto</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7777,7 +7614,6 @@
           <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr"/>
       <c r="P99" t="n">
         <v>2</v>
       </c>
@@ -7804,7 +7640,6 @@
           <t>Polia</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>upper</t>
@@ -7851,7 +7686,6 @@
           <t>dorsal, romboides</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr"/>
       <c r="P100" t="n">
         <v>2</v>
       </c>
@@ -7868,7 +7702,6 @@
           <t>Roda Abdominal</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
           <t>Ab wheel</t>
@@ -7925,7 +7758,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O101" t="inlineStr"/>
       <c r="P101" t="n">
         <v>1</v>
       </c>
@@ -8003,7 +7835,6 @@
           <t>dorsal, romboides</t>
         </is>
       </c>
-      <c r="O102" t="inlineStr"/>
       <c r="P102" t="n">
         <v>2</v>
       </c>
@@ -8020,7 +7851,6 @@
           <t>Side Clams</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
           <t>Glute band</t>
@@ -8077,7 +7907,6 @@
           <t>glúteo médio</t>
         </is>
       </c>
-      <c r="O103" t="inlineStr"/>
       <c r="P103" t="n">
         <v>0</v>
       </c>
@@ -8104,7 +7933,6 @@
           <t>Slide board</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>lower</t>
@@ -8151,7 +7979,6 @@
           <t>adutores, glúteo médio</t>
         </is>
       </c>
-      <c r="O104" t="inlineStr"/>
       <c r="P104" t="n">
         <v>0</v>
       </c>
@@ -8229,7 +8056,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O105" t="inlineStr"/>
       <c r="P105" t="n">
         <v>1</v>
       </c>
@@ -8307,7 +8133,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O106" t="inlineStr"/>
       <c r="P106" t="n">
         <v>1</v>
       </c>
@@ -8334,7 +8159,6 @@
           <t>barra smith</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>lower</t>
@@ -8381,7 +8205,6 @@
           <t>isquiotibiais, glúteos</t>
         </is>
       </c>
-      <c r="O107" t="inlineStr"/>
       <c r="P107" t="n">
         <v>2</v>
       </c>
@@ -8408,7 +8231,6 @@
           <t>Barra olímpica</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>lower</t>
@@ -8455,7 +8277,6 @@
           <t>isquiotibiais, glúteos</t>
         </is>
       </c>
-      <c r="O108" t="inlineStr"/>
       <c r="P108" t="n">
         <v>3</v>
       </c>
@@ -8482,7 +8303,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>lower</t>
@@ -8529,7 +8349,6 @@
           <t>isquiotibiais, glúteos</t>
         </is>
       </c>
-      <c r="O109" t="inlineStr"/>
       <c r="P109" t="n">
         <v>2</v>
       </c>
@@ -8556,7 +8375,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
           <t>lower</t>
@@ -8603,7 +8421,6 @@
           <t>isquiotibiais, glúteos</t>
         </is>
       </c>
-      <c r="O110" t="inlineStr"/>
       <c r="P110" t="n">
         <v>2</v>
       </c>
@@ -8630,7 +8447,6 @@
           <t>barra smith</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
           <t>lower</t>
@@ -8677,7 +8493,6 @@
           <t>isquiotibiais, glúteos</t>
         </is>
       </c>
-      <c r="O111" t="inlineStr"/>
       <c r="P111" t="n">
         <v>1</v>
       </c>
@@ -8755,7 +8570,6 @@
           <t>peitoral, tríceps, deltóide ant.</t>
         </is>
       </c>
-      <c r="O112" t="inlineStr"/>
       <c r="P112" t="n">
         <v>1</v>
       </c>
@@ -8833,7 +8647,6 @@
           <t>peitoral, tríceps, deltóide ant.</t>
         </is>
       </c>
-      <c r="O113" t="inlineStr"/>
       <c r="P113" t="n">
         <v>1</v>
       </c>
@@ -8911,7 +8724,6 @@
           <t>peitoral, tríceps, deltóide ant.</t>
         </is>
       </c>
-      <c r="O114" t="inlineStr"/>
       <c r="P114" t="n">
         <v>1</v>
       </c>
@@ -8989,7 +8801,6 @@
           <t>peitoral, tríceps</t>
         </is>
       </c>
-      <c r="O115" t="inlineStr"/>
       <c r="P115" t="n">
         <v>1</v>
       </c>
@@ -9016,7 +8827,6 @@
           <t>Halter</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
           <t>upper</t>
@@ -9063,7 +8873,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O116" t="inlineStr"/>
       <c r="P116" t="n">
         <v>1</v>
       </c>
@@ -9090,7 +8899,6 @@
           <t>polia</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
           <t>upper</t>
@@ -9137,7 +8945,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O117" t="inlineStr"/>
       <c r="P117" t="n">
         <v>1</v>
       </c>
@@ -9215,7 +9022,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O118" t="inlineStr"/>
       <c r="P118" t="n">
         <v>1</v>
       </c>
@@ -9242,7 +9048,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
           <t>upper</t>
@@ -9289,7 +9094,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O119" t="inlineStr"/>
       <c r="P119" t="n">
         <v>1</v>
       </c>
@@ -9316,7 +9120,6 @@
           <t>Banco reto</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
           <t>upper</t>
@@ -9363,7 +9166,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O120" t="inlineStr"/>
       <c r="P120" t="n">
         <v>1</v>
       </c>
@@ -9441,7 +9243,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O121" t="inlineStr"/>
       <c r="P121" t="n">
         <v>1</v>
       </c>
@@ -9519,7 +9320,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O122" t="inlineStr"/>
       <c r="P122" t="n">
         <v>1</v>
       </c>
@@ -9546,7 +9346,6 @@
           <t>Crossover</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
           <t>upper</t>
@@ -9593,7 +9392,6 @@
           <t>tríceps</t>
         </is>
       </c>
-      <c r="O123" t="inlineStr"/>
       <c r="P123" t="n">
         <v>1</v>
       </c>
@@ -9620,7 +9418,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
           <t>core</t>
@@ -9667,7 +9464,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O124" t="inlineStr"/>
       <c r="P124" t="n">
         <v>0</v>
       </c>
@@ -9694,7 +9490,6 @@
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
           <t>core</t>
@@ -9741,7 +9536,6 @@
           <t>core anterior</t>
         </is>
       </c>
-      <c r="O125" t="inlineStr"/>
       <c r="P125" t="n">
         <v>0</v>
       </c>
@@ -9768,7 +9562,6 @@
           <t>Halteres</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>lower</t>
@@ -9815,7 +9608,6 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O126" t="inlineStr"/>
       <c r="P126" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Fase 4 Sub-D — cadastrar 11 mock_futuros + expandir rotacao_tronco dyn
XLSX: +11 linhas (Apoio Fechado, Supino Fechado, Supino Inclinado Halteres,
Barra Aberta, Barra Supinada, Recuo do Estepe, Russian Twist, INFRA
Alternado/Suspenso/Chão/Roll-Up). Banco cresce de 125 → 136 exercícios.

gerador_treino.py:
- PADRAO_PARA_SUBREGIAO["rotacao_tronco"]: {"core_isometrico"} → {"core_isometrico", "core_dinamico"}
- _PADROES_LEGADOS["core_dinamico"]: adiciona "rotacao_tronco" (Russian Twist ativo)

Testes: seed SEED=3→1 (par Lev.Terra+Remada Baixa Aberta), contagens de carga
atualizadas (82/102/109 → 89/111/118), 8 snapshots regenerados. 175 passed.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W126"/>
+  <dimension ref="A1:W137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9618,6 +9618,929 @@
         <v>2</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Apoio Fechado</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Apoio</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Sem equipamento</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>peito</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>empurrar_compostos</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J127" t="n">
+        <v>2</v>
+      </c>
+      <c r="K127" t="n">
+        <v>3</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>horizontal_press_compound</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="P127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>1</v>
+      </c>
+      <c r="R127" t="n">
+        <v>1</v>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V127" t="b">
+        <v>1</v>
+      </c>
+      <c r="W127" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Supino Fechado</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Supino Reto</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>peito</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>empurrar_compostos</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J128" t="n">
+        <v>3</v>
+      </c>
+      <c r="K128" t="n">
+        <v>4</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>horizontal_press_compound</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="P128" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>0</v>
+      </c>
+      <c r="R128" t="n">
+        <v>0</v>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V128" t="b">
+        <v>1</v>
+      </c>
+      <c r="W128" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Supino Inclinado Halteres</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Supino Inclinado</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Halteres + Banco inclinado</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>peito</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>empurrar_compostos</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J129" t="n">
+        <v>3</v>
+      </c>
+      <c r="K129" t="n">
+        <v>3</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>horizontal_press_compound</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>peitoral, tríceps, deltóide ant.</t>
+        </is>
+      </c>
+      <c r="P129" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>0</v>
+      </c>
+      <c r="R129" t="n">
+        <v>0</v>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>inclinado</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V129" t="b">
+        <v>0</v>
+      </c>
+      <c r="W129" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Barra Aberta</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Barra fixa (crossover)</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>costas</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>puxadas</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J130" t="n">
+        <v>4</v>
+      </c>
+      <c r="K130" t="n">
+        <v>4</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>vertical_pull_compound</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>dorsal, bíceps</t>
+        </is>
+      </c>
+      <c r="P130" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>1</v>
+      </c>
+      <c r="R130" t="n">
+        <v>2</v>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>aberta</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V130" t="b">
+        <v>0</v>
+      </c>
+      <c r="W130" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Barra Supinada</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Barra fixa (crossover)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>costas</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>puxadas</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>4</v>
+      </c>
+      <c r="K131" t="n">
+        <v>4</v>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>vertical_pull_compound</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>dorsal, bíceps</t>
+        </is>
+      </c>
+      <c r="P131" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>1</v>
+      </c>
+      <c r="R131" t="n">
+        <v>2</v>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>supinada</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V131" t="b">
+        <v>0</v>
+      </c>
+      <c r="W131" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Recuo do Estepe</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>subida_elevada</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Halteres + Caixa</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>perna_anterior</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>squat_unilateral</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>unilateral</t>
+        </is>
+      </c>
+      <c r="J132" t="n">
+        <v>3</v>
+      </c>
+      <c r="K132" t="n">
+        <v>3</v>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>squat_unilateral_compound</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>Glúteos, Quadríceps</t>
+        </is>
+      </c>
+      <c r="P132" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>1</v>
+      </c>
+      <c r="R132" t="n">
+        <v>1</v>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="V132" t="b">
+        <v>0</v>
+      </c>
+      <c r="W132" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Russian Twist</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>russian twist</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Halteres</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>core_dinamico</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>rotacao_tronco</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>isolation</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J133" t="n">
+        <v>3</v>
+      </c>
+      <c r="K133" t="n">
+        <v>3</v>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>core_antirotation</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>obliquos, reto abdominal</t>
+        </is>
+      </c>
+      <c r="P133" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>1</v>
+      </c>
+      <c r="R133" t="n">
+        <v>2</v>
+      </c>
+      <c r="V133" t="b">
+        <v>0</v>
+      </c>
+      <c r="W133" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>INFRA Alternado</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Colchonete</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>core_dinamico</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>flexao_quadril</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>isolation</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>unilateral</t>
+        </is>
+      </c>
+      <c r="J134" t="n">
+        <v>2</v>
+      </c>
+      <c r="K134" t="n">
+        <v>2</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>core_flexion</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>iliopsoas, reto abdominal</t>
+        </is>
+      </c>
+      <c r="P134" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>1</v>
+      </c>
+      <c r="R134" t="n">
+        <v>2</v>
+      </c>
+      <c r="V134" t="b">
+        <v>0</v>
+      </c>
+      <c r="W134" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>INFRA Suspenso</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Barra fixa (crossover)</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>core_dinamico</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>flexao_quadril</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>isolation</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J135" t="n">
+        <v>4</v>
+      </c>
+      <c r="K135" t="n">
+        <v>3</v>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>core_flexion</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>iliopsoas, reto abdominal</t>
+        </is>
+      </c>
+      <c r="P135" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>1</v>
+      </c>
+      <c r="R135" t="n">
+        <v>3</v>
+      </c>
+      <c r="V135" t="b">
+        <v>0</v>
+      </c>
+      <c r="W135" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>INFRA Chão</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Colchonete</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>core_dinamico</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>flexao_quadril</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>isolation</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J136" t="n">
+        <v>2</v>
+      </c>
+      <c r="K136" t="n">
+        <v>2</v>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>core_flexion</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>iliopsoas, reto abdominal</t>
+        </is>
+      </c>
+      <c r="P136" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q136" t="n">
+        <v>1</v>
+      </c>
+      <c r="R136" t="n">
+        <v>3</v>
+      </c>
+      <c r="V136" t="b">
+        <v>0</v>
+      </c>
+      <c r="W136" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>INFRA Roll-Up</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Colchonete</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>core_dinamico</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>flexao_quadril</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>isolation</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>3</v>
+      </c>
+      <c r="K137" t="n">
+        <v>3</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>core_flexion</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>iliopsoas, reto abdominal</t>
+        </is>
+      </c>
+      <c r="P137" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>1</v>
+      </c>
+      <c r="R137" t="n">
+        <v>3</v>
+      </c>
+      <c r="V137" t="b">
+        <v>0</v>
+      </c>
+      <c r="W137" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4 Sub-E — port 66 entradas YAML → XLSX (5 colunas dims)
Atualiza variacao_de + pegada + plano_corporal + equipamento_grupo +
variante_pontual para todos os 66 exercícios cadastrado do YAML overlay.

Mudanças de variacao_de notáveis:
- Supinos: "Supino" → "Supino Reto" / "Supino Inclinado" (Anexo 15-bis)
- Step Up / Passada Dos Steps: → "subida_elevada" (Anexo 15-quinquies)
- Remada Curvada: "remada curvada" → "curvada"

Override nominal (Q1 desta sessão):
- Supino Com Anilha: equipamento_grupo = null (C4-exc2; anilha bilateral
  não aproxima por eixo de equipamento — não é família terra)

9 snapshots regenerados (mudanças de variacao_de afetam predicado
_compativel_intra, alterando saída determinística com seeds fixos).
175 passed.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -604,6 +604,9 @@
       <c r="R2" t="n">
         <v>2</v>
       </c>
+      <c r="V2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -820,6 +823,14 @@
       <c r="R5" t="n">
         <v>1</v>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -887,6 +898,14 @@
       <c r="R6" t="n">
         <v>3</v>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -959,6 +978,14 @@
       <c r="R7" t="n">
         <v>1</v>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1031,6 +1058,14 @@
       <c r="R8" t="n">
         <v>2</v>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1103,6 +1138,14 @@
       <c r="R9" t="n">
         <v>1</v>
       </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
+        </is>
+      </c>
+      <c r="V9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1314,6 +1357,19 @@
       <c r="R12" t="n">
         <v>1</v>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1381,6 +1437,19 @@
       <c r="R13" t="n">
         <v>1</v>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1448,6 +1517,19 @@
       <c r="R14" t="n">
         <v>1</v>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1520,6 +1602,19 @@
       <c r="R15" t="n">
         <v>2</v>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>aberta</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1592,6 +1687,19 @@
       <c r="R16" t="n">
         <v>2</v>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>aberta</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2096,6 +2204,9 @@
       <c r="R23" t="n">
         <v>2</v>
       </c>
+      <c r="V23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2163,6 +2274,14 @@
       <c r="R24" t="n">
         <v>0</v>
       </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>maquina</t>
+        </is>
+      </c>
+      <c r="V24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2297,6 +2416,9 @@
       <c r="R26" t="n">
         <v>2</v>
       </c>
+      <c r="V26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2446,6 +2568,24 @@
       <c r="R28" t="n">
         <v>1</v>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2523,6 +2663,24 @@
       <c r="R29" t="n">
         <v>0</v>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2600,6 +2758,24 @@
       <c r="R30" t="n">
         <v>0</v>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2739,6 +2915,9 @@
       <c r="R32" t="n">
         <v>1</v>
       </c>
+      <c r="V32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2811,6 +2990,9 @@
       <c r="R33" t="n">
         <v>2</v>
       </c>
+      <c r="V33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2883,6 +3065,9 @@
       <c r="R34" t="n">
         <v>2</v>
       </c>
+      <c r="V34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2955,6 +3140,9 @@
       <c r="R35" t="n">
         <v>2</v>
       </c>
+      <c r="V35" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3032,6 +3220,9 @@
       <c r="R36" t="n">
         <v>3</v>
       </c>
+      <c r="V36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3104,6 +3295,9 @@
       <c r="R37" t="n">
         <v>2</v>
       </c>
+      <c r="V37" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4708,6 +4902,9 @@
       <c r="R59" t="n">
         <v>2</v>
       </c>
+      <c r="V59" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4775,6 +4972,14 @@
       <c r="R60" t="n">
         <v>0</v>
       </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>maquina</t>
+        </is>
+      </c>
+      <c r="V60" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5130,6 +5335,9 @@
       <c r="R65" t="n">
         <v>2</v>
       </c>
+      <c r="V65" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5202,6 +5410,14 @@
       <c r="R66" t="n">
         <v>1</v>
       </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V66" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5211,7 +5427,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>passada</t>
+          <t>subida_elevada</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -5279,6 +5495,14 @@
       <c r="R67" t="n">
         <v>1</v>
       </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="V67" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5875,6 +6099,9 @@
       <c r="R75" t="n">
         <v>1</v>
       </c>
+      <c r="V75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5947,6 +6174,9 @@
       <c r="R76" t="n">
         <v>2</v>
       </c>
+      <c r="V76" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6019,6 +6249,9 @@
       <c r="R77" t="n">
         <v>2</v>
       </c>
+      <c r="V77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6091,6 +6324,9 @@
       <c r="R78" t="n">
         <v>2</v>
       </c>
+      <c r="V78" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6158,6 +6394,9 @@
       <c r="R79" t="n">
         <v>2</v>
       </c>
+      <c r="V79" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6230,6 +6469,9 @@
       <c r="R80" t="n">
         <v>2</v>
       </c>
+      <c r="V80" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6302,6 +6544,9 @@
       <c r="R81" t="n">
         <v>3</v>
       </c>
+      <c r="V81" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6379,6 +6624,24 @@
       <c r="R82" t="n">
         <v>2</v>
       </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>pullover</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V82" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6451,6 +6714,24 @@
       <c r="R83" t="n">
         <v>2</v>
       </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>pullover</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V83" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6528,6 +6809,19 @@
       <c r="R84" t="n">
         <v>1</v>
       </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>aberta</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V84" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6605,6 +6899,19 @@
       <c r="R85" t="n">
         <v>1</v>
       </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V85" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6677,6 +6984,19 @@
       <c r="R86" t="n">
         <v>1</v>
       </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>supinada</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V86" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6749,6 +7069,14 @@
       <c r="R87" t="n">
         <v>1</v>
       </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V87" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6821,6 +7149,14 @@
       <c r="R88" t="n">
         <v>1</v>
       </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V88" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6893,6 +7229,14 @@
       <c r="R89" t="n">
         <v>1</v>
       </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V89" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6960,6 +7304,19 @@
       <c r="R90" t="n">
         <v>1</v>
       </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>aberta</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>suspensao</t>
+        </is>
+      </c>
+      <c r="V90" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6969,7 +7326,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Remada horizontal</t>
+          <t>apoiado</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7035,6 +7392,24 @@
         <v>0</v>
       </c>
       <c r="R91" t="n">
+        <v>0</v>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>apoiada</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V91" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7046,7 +7421,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>remada baixa</t>
+          <t>baixa</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -7113,6 +7488,24 @@
       </c>
       <c r="R92" t="n">
         <v>2</v>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>aberta</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>baixa_sentada</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V92" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -7123,7 +7516,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Remada horizontal</t>
+          <t>baixa</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -7190,6 +7583,24 @@
       </c>
       <c r="R93" t="n">
         <v>2</v>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>baixa_sentada</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V93" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -7200,7 +7611,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>remada curvada</t>
+          <t>curvada</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -7263,6 +7674,24 @@
       <c r="R94" t="n">
         <v>3</v>
       </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>curvada</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V94" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7272,7 +7701,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>remada curvada</t>
+          <t>curvada</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -7335,6 +7764,24 @@
       <c r="R95" t="n">
         <v>3</v>
       </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>curvada</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V95" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7344,7 +7791,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>remada curvada</t>
+          <t>curvada</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -7407,6 +7854,24 @@
       <c r="R96" t="n">
         <v>2</v>
       </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>curvada</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
+        </is>
+      </c>
+      <c r="V96" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7416,7 +7881,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Remada horizontal</t>
+          <t>curvada</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -7483,6 +7948,24 @@
       </c>
       <c r="R97" t="n">
         <v>3</v>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>curvada</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V97" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -7551,6 +8034,19 @@
       <c r="R98" t="n">
         <v>1</v>
       </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>suspensao</t>
+        </is>
+      </c>
+      <c r="V98" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7560,7 +8056,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Remada horizontal</t>
+          <t>seal</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -7623,6 +8119,24 @@
       <c r="R99" t="n">
         <v>0</v>
       </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>apoiada</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V99" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7632,7 +8146,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Remada unilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -7694,6 +8208,24 @@
       </c>
       <c r="R100" t="n">
         <v>1</v>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>unilateral_apoiada</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V100" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -7767,6 +8299,9 @@
       <c r="R101" t="n">
         <v>3</v>
       </c>
+      <c r="V101" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7776,7 +8311,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Remada unilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7844,6 +8379,24 @@
       <c r="R102" t="n">
         <v>2</v>
       </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>unilateral_apoiada</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V102" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7988,6 +8541,9 @@
       <c r="R104" t="n">
         <v>1</v>
       </c>
+      <c r="V104" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7997,7 +8553,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Step up</t>
+          <t>subida_elevada</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -8064,6 +8620,14 @@
       </c>
       <c r="R105" t="n">
         <v>1</v>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="V105" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -8074,7 +8638,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Step up</t>
+          <t>subida_elevada</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -8141,6 +8705,14 @@
       </c>
       <c r="R106" t="n">
         <v>1</v>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="V106" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -8511,7 +9083,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Supino</t>
+          <t>Supino Reto</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -8577,6 +9149,19 @@
         <v>0</v>
       </c>
       <c r="R112" t="n">
+        <v>0</v>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="V112" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8588,7 +9173,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Supino</t>
+          <t>Supino Reto</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -8654,6 +9239,24 @@
         <v>0</v>
       </c>
       <c r="R113" t="n">
+        <v>0</v>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V113" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8665,7 +9268,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Supino</t>
+          <t>Supino Reto</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -8731,6 +9334,24 @@
         <v>0</v>
       </c>
       <c r="R114" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>reto</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V114" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8742,7 +9363,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Supino</t>
+          <t>Supino Inclinado</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -8808,6 +9429,24 @@
         <v>0</v>
       </c>
       <c r="R115" t="n">
+        <v>0</v>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>inclinado</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
+        </is>
+      </c>
+      <c r="V115" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9473,6 +10112,9 @@
       <c r="R124" t="n">
         <v>3</v>
       </c>
+      <c r="V124" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -9545,6 +10187,9 @@
       <c r="R125" t="n">
         <v>2</v>
       </c>
+      <c r="V125" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9616,6 +10261,14 @@
       </c>
       <c r="R126" t="n">
         <v>2</v>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V126" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="127">

</xml_diff>

<commit_message>
Fase 4 Sub-F — preencher dims para 59 exercícios non-YAML
Aplica 5 colunas dims (pegada, plano_corporal, equipamento_grupo,
variante_pontual; variacao_de intocado) para todos os 59 exercícios
que não estavam no YAML da Etapa 6.

Regras aplicadas:
- hinge em_pe: Stiffs (5), Lev. Terra (3), Good Morning, Hiperextensão 45°
- hinge deitado: Hip Thrusts (3), Pontes (6)
- Decisões C1-C7: Landmine→pegada=neutra, Feijão/Slide→equip=null,
  Hip Thrust Uni./Ponte Uni./Copenhagen→corporal, Hiperext.→em_pe,
  Lev. Terra Anilha→barra (C4-exc), Elevação Panturrilha→corporal
- ombro/bíceps/tríceps: pegada=null (conservador + G7); equip por eq_primario
- cardio: all null

Consequências:
- 6 snapshots atualizados (score-aware agora tem dims em todo banco)
- HIB2 seed: 1→4; par: Lev.Terra+Remada Baixa Aberta→Lev.Terra+Barra Isométrica
- 175 passed, 1 skipped (igual Etapa 8)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -679,6 +679,14 @@
       <c r="R3" t="n">
         <v>1</v>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -751,6 +759,14 @@
       <c r="R4" t="n">
         <v>1</v>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1218,6 +1234,9 @@
       <c r="R10" t="n">
         <v>1</v>
       </c>
+      <c r="V10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1290,6 +1309,9 @@
       <c r="R11" t="n">
         <v>1</v>
       </c>
+      <c r="V11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1772,6 +1794,14 @@
       <c r="R17" t="n">
         <v>1</v>
       </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1849,6 +1879,14 @@
       <c r="R18" t="n">
         <v>0</v>
       </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1921,6 +1959,14 @@
       <c r="R19" t="n">
         <v>1</v>
       </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1993,6 +2039,14 @@
       <c r="R20" t="n">
         <v>1</v>
       </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2065,6 +2119,14 @@
       <c r="R21" t="n">
         <v>1</v>
       </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2137,6 +2199,14 @@
       <c r="R22" t="n">
         <v>1</v>
       </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2349,6 +2419,14 @@
       <c r="R25" t="n">
         <v>0</v>
       </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>maquina</t>
+        </is>
+      </c>
+      <c r="V25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2496,6 +2574,14 @@
       <c r="R27" t="n">
         <v>3</v>
       </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2843,6 +2929,14 @@
       <c r="R31" t="n">
         <v>2</v>
       </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V31" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3375,6 +3469,14 @@
       <c r="R38" t="n">
         <v>1</v>
       </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V38" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3452,6 +3554,14 @@
       <c r="R39" t="n">
         <v>1</v>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V39" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3529,6 +3639,19 @@
       <c r="R40" t="n">
         <v>1</v>
       </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V40" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3606,6 +3729,14 @@
       <c r="R41" t="n">
         <v>1</v>
       </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V41" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3678,6 +3809,14 @@
       <c r="R42" t="n">
         <v>1</v>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
+        </is>
+      </c>
+      <c r="V42" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3745,6 +3884,14 @@
       <c r="R43" t="n">
         <v>1</v>
       </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>banda_elastica</t>
+        </is>
+      </c>
+      <c r="V43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3817,6 +3964,14 @@
       <c r="R44" t="n">
         <v>1</v>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V44" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3889,6 +4044,14 @@
       <c r="R45" t="n">
         <v>1</v>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V45" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3961,6 +4124,14 @@
       <c r="R46" t="n">
         <v>1</v>
       </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V46" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4033,6 +4204,14 @@
       <c r="R47" t="n">
         <v>1</v>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V47" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4105,6 +4284,14 @@
       <c r="R48" t="n">
         <v>1</v>
       </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V48" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4182,6 +4369,14 @@
       <c r="R49" t="n">
         <v>0</v>
       </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V49" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4254,6 +4449,14 @@
       <c r="R50" t="n">
         <v>1</v>
       </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V50" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4326,6 +4529,14 @@
       <c r="R51" t="n">
         <v>1</v>
       </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V51" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4398,6 +4609,9 @@
       <c r="R52" t="n">
         <v>2</v>
       </c>
+      <c r="V52" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4470,6 +4684,9 @@
       <c r="R53" t="n">
         <v>3</v>
       </c>
+      <c r="V53" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4542,6 +4759,19 @@
       <c r="R54" t="n">
         <v>3</v>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V54" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4619,6 +4849,19 @@
       <c r="R55" t="n">
         <v>1</v>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V55" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4696,6 +4939,19 @@
       <c r="R56" t="n">
         <v>1</v>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>banda_elastica</t>
+        </is>
+      </c>
+      <c r="V56" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4768,6 +5024,19 @@
       <c r="R57" t="n">
         <v>1</v>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V57" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4835,6 +5104,19 @@
       <c r="R58" t="n">
         <v>2</v>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>maquina</t>
+        </is>
+      </c>
+      <c r="V58" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5057,6 +5339,19 @@
       <c r="R61" t="n">
         <v>3</v>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V61" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5129,6 +5424,19 @@
       <c r="R62" t="n">
         <v>2</v>
       </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V62" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5206,6 +5514,19 @@
       <c r="R63" t="n">
         <v>3</v>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V63" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5268,6 +5589,14 @@
       <c r="R64" t="n">
         <v>3</v>
       </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V64" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5580,6 +5909,19 @@
       <c r="R68" t="n">
         <v>1</v>
       </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V68" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5657,6 +5999,19 @@
       <c r="R69" t="n">
         <v>1</v>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V69" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5734,6 +6089,19 @@
       <c r="R70" t="n">
         <v>1</v>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>banda_elastica</t>
+        </is>
+      </c>
+      <c r="V70" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5811,6 +6179,19 @@
       <c r="R71" t="n">
         <v>1</v>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="V71" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5888,6 +6269,19 @@
       <c r="R72" t="n">
         <v>1</v>
       </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
+      </c>
+      <c r="V72" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5960,6 +6354,19 @@
       <c r="R73" t="n">
         <v>1</v>
       </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>deitado</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V73" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6027,6 +6434,14 @@
       <c r="R74" t="n">
         <v>0</v>
       </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V74" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8469,6 +8884,14 @@
       <c r="R103" t="n">
         <v>1</v>
       </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>banda_elastica</t>
+        </is>
+      </c>
+      <c r="V103" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8786,6 +9209,19 @@
       <c r="R107" t="n">
         <v>3</v>
       </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
+        </is>
+      </c>
+      <c r="V107" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8858,6 +9294,19 @@
       <c r="R108" t="n">
         <v>3</v>
       </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="V108" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8930,6 +9379,19 @@
       <c r="R109" t="n">
         <v>3</v>
       </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V109" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9002,6 +9464,19 @@
       <c r="R110" t="n">
         <v>3</v>
       </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V110" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9074,6 +9549,19 @@
       <c r="R111" t="n">
         <v>3</v>
       </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
+        </is>
+      </c>
+      <c r="V111" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9521,6 +10009,14 @@
       <c r="R116" t="n">
         <v>1</v>
       </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V116" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9593,6 +10089,14 @@
       <c r="R117" t="n">
         <v>1</v>
       </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V117" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9670,6 +10174,14 @@
       <c r="R118" t="n">
         <v>1</v>
       </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V118" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -9742,6 +10254,14 @@
       <c r="R119" t="n">
         <v>0</v>
       </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V119" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -9814,6 +10334,14 @@
       <c r="R120" t="n">
         <v>1</v>
       </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>corporal</t>
+        </is>
+      </c>
+      <c r="V120" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -9891,6 +10419,14 @@
       <c r="R121" t="n">
         <v>1</v>
       </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V121" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -9968,6 +10504,14 @@
       <c r="R122" t="n">
         <v>0</v>
       </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>halter</t>
+        </is>
+      </c>
+      <c r="V122" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -10039,6 +10583,14 @@
       </c>
       <c r="R123" t="n">
         <v>1</v>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
+      </c>
+      <c r="V123" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="124">

</xml_diff>

<commit_message>
Fase 4 Sub-H — Remada Landmine split (Annexo 4.1 item 1)
Renomeia 'Remada Landmine' para 'Remada LM Neutra' e insere nova linha
'Remada LM Aberta' logo após (pegada=aberta, demais dims idênticas).
Ambas mantêm variacao_de='curvada' (família curvada existente).

Banco: 137 exercícios (136 → 137).
Contadores carga: 90/112/119 grip/lombar/core (era 89/111/118).
3 snapshots atualizados. 175 passed, 1 skipped.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W137"/>
+  <dimension ref="A1:W138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8291,7 +8291,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Remada Landmine</t>
+          <t>Remada LM Neutra</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -8386,12 +8386,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Remada Neutra Trx</t>
+          <t>Remada LM Aberta</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>trx</t>
+          <t>curvada</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Barra landmine</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Suporte remada landmine</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -8416,11 +8426,11 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K98" t="n">
         <v>3</v>
@@ -8437,46 +8447,49 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>dorsal, romboides, bíceps</t>
+          <t>dorsal, romboides</t>
         </is>
       </c>
       <c r="P98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q98" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R98" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>neutra</t>
+          <t>aberta</t>
         </is>
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>suspensao</t>
+          <t>curvada</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>barra</t>
         </is>
       </c>
       <c r="V98" t="b">
         <v>0</v>
+      </c>
+      <c r="W98" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Remada Seal Halteres</t>
+          <t>Remada Neutra Trx</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>seal</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Banco reto</t>
+          <t>trx</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8505,7 +8518,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K99" t="n">
         <v>3</v>
@@ -8529,10 +8542,10 @@
         <v>2</v>
       </c>
       <c r="Q99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S99" t="inlineStr">
         <is>
@@ -8541,12 +8554,7 @@
       </c>
       <c r="T99" t="inlineStr">
         <is>
-          <t>apoiada</t>
-        </is>
-      </c>
-      <c r="U99" t="inlineStr">
-        <is>
-          <t>halter</t>
+          <t>suspensao</t>
         </is>
       </c>
       <c r="V99" t="b">
@@ -8556,17 +8564,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Remada Uni Polia</t>
+          <t>Remada Seal Halteres</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>seal</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Polia</t>
+          <t>Banco reto</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -8591,11 +8599,11 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K100" t="n">
         <v>3</v>
@@ -8612,17 +8620,17 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>dorsal, romboides</t>
+          <t>dorsal, romboides, bíceps</t>
         </is>
       </c>
       <c r="P100" t="n">
         <v>2</v>
       </c>
       <c r="Q100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S100" t="inlineStr">
         <is>
@@ -8631,12 +8639,12 @@
       </c>
       <c r="T100" t="inlineStr">
         <is>
-          <t>unilateral_apoiada</t>
+          <t>apoiada</t>
         </is>
       </c>
       <c r="U100" t="inlineStr">
         <is>
-          <t>polia</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V100" t="b">
@@ -8646,49 +8654,49 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Roda Abdominal</t>
+          <t>Remada Uni Polia</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Ab wheel</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Colchonete</t>
+          <t>Polia</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>upper</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>core_isometrico</t>
+          <t>costas</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>flexao_tronco</t>
+          <t>remadas</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>stability</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -8697,22 +8705,37 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>core_antiextension</t>
+          <t>horizontal_pull_compound</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>core anterior</t>
+          <t>dorsal, romboides</t>
         </is>
       </c>
       <c r="P101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q101" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R101" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>unilateral_apoiada</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
       </c>
       <c r="V101" t="b">
         <v>0</v>
@@ -8721,47 +8744,42 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Serrote</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>unilateral</t>
+          <t>Roda Abdominal</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Halteres</t>
+          <t>Ab wheel</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Banco reto</t>
+          <t>Colchonete</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>upper</t>
+          <t>core</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>costas</t>
+          <t>core_isometrico</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>remadas</t>
+          <t>flexao_tronco</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>compound</t>
+          <t>stability</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J102" t="n">
@@ -8777,37 +8795,22 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>horizontal_pull_compound</t>
+          <t>core_antiextension</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>dorsal, romboides</t>
+          <t>core anterior</t>
         </is>
       </c>
       <c r="P102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R102" t="n">
-        <v>2</v>
-      </c>
-      <c r="S102" t="inlineStr">
-        <is>
-          <t>neutra</t>
-        </is>
-      </c>
-      <c r="T102" t="inlineStr">
-        <is>
-          <t>unilateral_apoiada</t>
-        </is>
-      </c>
-      <c r="U102" t="inlineStr">
-        <is>
-          <t>halter</t>
-        </is>
+        <v>3</v>
       </c>
       <c r="V102" t="b">
         <v>0</v>
@@ -8816,77 +8819,92 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Side Clams</t>
+          <t>Serrote</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Glute band</t>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Colchonete</t>
+          <t>Banco reto</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>upper</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>perna_posterior</t>
+          <t>costas</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>abduction</t>
+          <t>remadas</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>isolation</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K103" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>hip_abduction_isolation</t>
+          <t>horizontal_pull_compound</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>glúteo médio</t>
+          <t>dorsal, romboides</t>
         </is>
       </c>
       <c r="P103" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q103" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R103" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>neutra</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>unilateral_apoiada</t>
+        </is>
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>banda_elastica</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V103" t="b">
@@ -8896,17 +8914,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Slide Board Lateral</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>agach. lateral</t>
+          <t>Side Clams</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Slide board</t>
+          <t>Glute band</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Colchonete</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -8916,29 +8934,29 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>perna_anterior</t>
+          <t>perna_posterior</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>squat_unilateral</t>
+          <t>abduction</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>compound</t>
+          <t>isolation</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L104" t="inlineStr">
         <is>
@@ -8947,22 +8965,27 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>squat_unilateral_compound</t>
+          <t>hip_abduction_isolation</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>adutores, glúteo médio</t>
+          <t>glúteo médio</t>
         </is>
       </c>
       <c r="P104" t="n">
         <v>0</v>
       </c>
       <c r="Q104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R104" t="n">
         <v>1</v>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>banda_elastica</t>
+        </is>
       </c>
       <c r="V104" t="b">
         <v>0</v>
@@ -8971,22 +8994,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Step Up</t>
+          <t>Slide Board Lateral</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>subida_elevada</t>
+          <t>agach. lateral</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Caixa</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Halteres</t>
+          <t>Slide board</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -9032,22 +9050,17 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>quadríceps, glúteos</t>
+          <t>adutores, glúteo médio</t>
         </is>
       </c>
       <c r="P105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q105" t="n">
         <v>1</v>
       </c>
       <c r="R105" t="n">
         <v>1</v>
-      </c>
-      <c r="U105" t="inlineStr">
-        <is>
-          <t>caixa</t>
-        </is>
       </c>
       <c r="V105" t="b">
         <v>0</v>
@@ -9056,7 +9069,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Step Up Alt.</t>
+          <t>Step Up</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -9141,17 +9154,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Stiff Barra Smith</t>
+          <t>Step Up Alt.</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>stiff</t>
+          <t>subida_elevada</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>barra smith</t>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -9161,12 +9179,12 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>perna_posterior</t>
+          <t>perna_anterior</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>hinge</t>
+          <t>squat_unilateral</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -9176,47 +9194,42 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J107" t="n">
         <v>3</v>
       </c>
       <c r="K107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>hip_hinge_compound</t>
+          <t>squat_unilateral_compound</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>isquiotibiais, glúteos</t>
+          <t>quadríceps, glúteos</t>
         </is>
       </c>
       <c r="P107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R107" t="n">
-        <v>3</v>
-      </c>
-      <c r="T107" t="inlineStr">
-        <is>
-          <t>em_pe</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>barra_guiada</t>
+          <t>caixa</t>
         </is>
       </c>
       <c r="V107" t="b">
@@ -9226,7 +9239,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Stiff Barra Livre</t>
+          <t>Stiff Barra Smith</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -9236,7 +9249,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Barra olímpica</t>
+          <t>barra smith</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -9286,7 +9299,7 @@
         </is>
       </c>
       <c r="P108" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q108" t="n">
         <v>3</v>
@@ -9301,7 +9314,7 @@
       </c>
       <c r="U108" t="inlineStr">
         <is>
-          <t>barra</t>
+          <t>barra_guiada</t>
         </is>
       </c>
       <c r="V108" t="b">
@@ -9311,7 +9324,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Stiff Halteres</t>
+          <t>Stiff Barra Livre</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9321,7 +9334,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Halteres</t>
+          <t>Barra olímpica</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9353,7 +9366,7 @@
         <v>3</v>
       </c>
       <c r="K109" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9371,7 +9384,7 @@
         </is>
       </c>
       <c r="P109" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q109" t="n">
         <v>3</v>
@@ -9386,7 +9399,7 @@
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>halter</t>
+          <t>barra</t>
         </is>
       </c>
       <c r="V109" t="b">
@@ -9396,7 +9409,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Stiff Uni. Halteres</t>
+          <t>Stiff Halteres</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9431,7 +9444,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -9481,7 +9494,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Stiff Uni. Smith</t>
+          <t>Stiff Uni. Halteres</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9491,7 +9504,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>barra smith</t>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -9541,7 +9554,7 @@
         </is>
       </c>
       <c r="P111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q111" t="n">
         <v>3</v>
@@ -9556,7 +9569,7 @@
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>barra_guiada</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V111" t="b">
@@ -9566,37 +9579,32 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Supino Com Anilha</t>
+          <t>Stiff Uni. Smith</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Supino Reto</t>
+          <t>stiff</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Banco reto</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Anilha</t>
+          <t>barra smith</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>upper</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>peito</t>
+          <t>perna_posterior</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>empurrar_compostos</t>
+          <t>hinge</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -9606,11 +9614,11 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K112" t="n">
         <v>3</v>
@@ -9622,31 +9630,31 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>horizontal_press_compound</t>
+          <t>hip_hinge_compound</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>peitoral, tríceps, deltóide ant.</t>
+          <t>isquiotibiais, glúteos</t>
         </is>
       </c>
       <c r="P112" t="n">
         <v>1</v>
       </c>
       <c r="Q112" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R112" t="n">
-        <v>0</v>
-      </c>
-      <c r="S112" t="inlineStr">
-        <is>
-          <t>pronada</t>
-        </is>
+        <v>3</v>
       </c>
       <c r="T112" t="inlineStr">
         <is>
-          <t>reto</t>
+          <t>em_pe</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>barra_guiada</t>
         </is>
       </c>
       <c r="V112" t="b">
@@ -9656,7 +9664,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Supino Com Barra</t>
+          <t>Supino Com Anilha</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -9666,12 +9674,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Rack + barra olímpica</t>
+          <t>Banco reto</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Banco reto</t>
+          <t>Anilha</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -9700,7 +9708,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K113" t="n">
         <v>3</v>
@@ -9737,11 +9745,6 @@
       <c r="T113" t="inlineStr">
         <is>
           <t>reto</t>
-        </is>
-      </c>
-      <c r="U113" t="inlineStr">
-        <is>
-          <t>barra</t>
         </is>
       </c>
       <c r="V113" t="b">
@@ -9751,7 +9754,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Supino Com Halteres</t>
+          <t>Supino Com Barra</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -9761,14 +9764,14 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
+          <t>Rack + barra olímpica</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
           <t>Banco reto</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Halteres</t>
-        </is>
-      </c>
       <c r="E114" t="inlineStr">
         <is>
           <t>upper</t>
@@ -9836,7 +9839,7 @@
       </c>
       <c r="U114" t="inlineStr">
         <is>
-          <t>halter</t>
+          <t>barra</t>
         </is>
       </c>
       <c r="V114" t="b">
@@ -9846,22 +9849,22 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Supino Smith Inclinado</t>
+          <t>Supino Com Halteres</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Supino Inclinado</t>
+          <t>Supino Reto</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Barra Smith (crossover)</t>
+          <t>Banco reto</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Banco inclinável</t>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -9890,7 +9893,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K115" t="n">
         <v>3</v>
@@ -9907,7 +9910,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>peitoral, tríceps</t>
+          <t>peitoral, tríceps, deltóide ant.</t>
         </is>
       </c>
       <c r="P115" t="n">
@@ -9926,12 +9929,12 @@
       </c>
       <c r="T115" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>reto</t>
         </is>
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>barra_guiada</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V115" t="b">
@@ -9941,17 +9944,22 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Tríceps Coice Com Halter</t>
+          <t>Supino Smith Inclinado</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Tríceps Coice</t>
+          <t>Supino Inclinado</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Halter</t>
+          <t>Barra Smith (crossover)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Banco inclinável</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -9961,17 +9969,17 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>bracos</t>
+          <t>peito</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>triceps</t>
+          <t>empurrar_compostos</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>isolation</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -9983,7 +9991,7 @@
         <v>2</v>
       </c>
       <c r="K116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -9992,26 +10000,36 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>elbow_extension_isolation</t>
+          <t>horizontal_press_compound</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>tríceps</t>
+          <t>peitoral, tríceps</t>
         </is>
       </c>
       <c r="P116" t="n">
         <v>1</v>
       </c>
       <c r="Q116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R116" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>inclinado</t>
+        </is>
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>halter</t>
+          <t>barra_guiada</t>
         </is>
       </c>
       <c r="V116" t="b">
@@ -10021,7 +10039,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Tríceps Coice Polia</t>
+          <t>Tríceps Coice Com Halter</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -10031,7 +10049,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>polia</t>
+          <t>Halter</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -10056,7 +10074,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J117" t="n">
@@ -10091,7 +10109,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>polia</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V117" t="b">
@@ -10101,22 +10119,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Tríceps Corda</t>
+          <t>Tríceps Coice Polia</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Tríceps Pushdown</t>
+          <t>Tríceps Coice</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Polia</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>Corda</t>
+          <t>polia</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -10141,18 +10154,18 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K118" t="n">
         <v>2</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -10186,17 +10199,22 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Tríceps Francês</t>
+          <t>Tríceps Corda</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tríceps Francês</t>
+          <t>Tríceps Pushdown</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Halteres</t>
+          <t>Polia</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Corda</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -10221,18 +10239,18 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K119" t="n">
         <v>2</v>
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -10249,14 +10267,14 @@
         <v>1</v>
       </c>
       <c r="Q119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>halter</t>
+          <t>polia</t>
         </is>
       </c>
       <c r="V119" t="b">
@@ -10266,17 +10284,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Tríceps Mergulho Banco</t>
+          <t>Tríceps Francês</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Tríceps Mergulho</t>
+          <t>Tríceps Francês</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Banco reto</t>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -10301,18 +10319,18 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J120" t="n">
         <v>2</v>
       </c>
       <c r="K120" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
@@ -10332,11 +10350,11 @@
         <v>0</v>
       </c>
       <c r="R120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>corporal</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V120" t="b">
@@ -10346,22 +10364,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Tríceps Polia Alta</t>
+          <t>Tríceps Mergulho Banco</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Tríceps Pushdown</t>
+          <t>Tríceps Mergulho</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Crossover</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>Barra reta pequena</t>
+          <t>Banco reto</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -10390,14 +10403,14 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
@@ -10414,14 +10427,14 @@
         <v>1</v>
       </c>
       <c r="Q121" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R121" t="n">
         <v>1</v>
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>polia</t>
+          <t>corporal</t>
         </is>
       </c>
       <c r="V121" t="b">
@@ -10431,22 +10444,22 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Tríceps Testa Halteres</t>
+          <t>Tríceps Polia Alta</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Tríceps Testa</t>
+          <t>Tríceps Pushdown</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Halteres</t>
+          <t>Crossover</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Banco reto</t>
+          <t>Barra reta pequena</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -10475,7 +10488,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K122" t="n">
         <v>2</v>
@@ -10499,14 +10512,14 @@
         <v>1</v>
       </c>
       <c r="Q122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>halter</t>
+          <t>polia</t>
         </is>
       </c>
       <c r="V122" t="b">
@@ -10516,17 +10529,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Tríceps Unilateral Polia</t>
+          <t>Tríceps Testa Halteres</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Tríceps Pushdown</t>
+          <t>Tríceps Testa</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Crossover</t>
+          <t>Halteres</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Banco reto</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -10551,11 +10569,11 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K123" t="n">
         <v>2</v>
@@ -10579,14 +10597,14 @@
         <v>1</v>
       </c>
       <c r="Q123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U123" t="inlineStr">
         <is>
-          <t>polia</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V123" t="b">
@@ -10596,32 +10614,32 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>V-Up</t>
+          <t>Tríceps Unilateral Polia</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>v-up</t>
+          <t>Tríceps Pushdown</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Colchonete</t>
+          <t>Crossover</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>upper</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>core_dinamico</t>
+          <t>bracos</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>flexao_quadril</t>
+          <t>triceps</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -10631,38 +10649,43 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J124" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K124" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>core_flexion</t>
+          <t>elbow_extension_isolation</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>core anterior</t>
+          <t>tríceps</t>
         </is>
       </c>
       <c r="P124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q124" t="n">
         <v>1</v>
       </c>
       <c r="R124" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>polia</t>
+        </is>
       </c>
       <c r="V124" t="b">
         <v>0</v>
@@ -10671,7 +10694,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>V-Up Unilateral</t>
+          <t>V-Up</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -10706,14 +10729,14 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J125" t="n">
         <v>2</v>
       </c>
       <c r="K125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -10737,7 +10760,7 @@
         <v>1</v>
       </c>
       <c r="R125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V125" t="b">
         <v>0</v>
@@ -10746,37 +10769,37 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Walking Lunges</t>
+          <t>V-Up Unilateral</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>walking lunges</t>
+          <t>v-up</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Halteres</t>
+          <t>Colchonete</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>core</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>perna_anterior</t>
+          <t>core_dinamico</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>squat_unilateral</t>
+          <t>flexao_quadril</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>compound</t>
+          <t>isolation</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -10785,7 +10808,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K126" t="n">
         <v>3</v>
@@ -10797,27 +10820,22 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>squat_unilateral_compound</t>
+          <t>core_flexion</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>quadríceps, glúteos</t>
+          <t>core anterior</t>
         </is>
       </c>
       <c r="P126" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q126" t="n">
         <v>1</v>
       </c>
       <c r="R126" t="n">
         <v>2</v>
-      </c>
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>halter</t>
-        </is>
       </c>
       <c r="V126" t="b">
         <v>0</v>
@@ -10826,32 +10844,32 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Apoio Fechado</t>
+          <t>Walking Lunges</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Apoio</t>
+          <t>walking lunges</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Sem equipamento</t>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>upper</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>peito</t>
+          <t>perna_anterior</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>empurrar_compostos</t>
+          <t>squat_unilateral</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -10861,11 +10879,11 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K127" t="n">
         <v>3</v>
@@ -10877,54 +10895,46 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>horizontal_press_compound</t>
+          <t>squat_unilateral_compound</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>quadríceps, glúteos</t>
         </is>
       </c>
       <c r="P127" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q127" t="n">
         <v>1</v>
       </c>
       <c r="R127" t="n">
-        <v>1</v>
-      </c>
-      <c r="S127" t="inlineStr">
-        <is>
-          <t>pronada</t>
-        </is>
+        <v>2</v>
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>corporal</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V127" t="b">
-        <v>1</v>
-      </c>
-      <c r="W127" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Supino Fechado</t>
+          <t>Apoio Fechado</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Supino Reto</t>
+          <t>Apoio</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Barra</t>
+          <t>Sem equipamento</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -10953,14 +10963,14 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K128" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
@@ -10974,27 +10984,22 @@
         </is>
       </c>
       <c r="P128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
           <t>pronada</t>
         </is>
       </c>
-      <c r="T128" t="inlineStr">
-        <is>
-          <t>reto</t>
-        </is>
-      </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>barra</t>
+          <t>corporal</t>
         </is>
       </c>
       <c r="V128" t="b">
@@ -11007,17 +11012,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Supino Inclinado Halteres</t>
+          <t>Supino Fechado</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Supino Inclinado</t>
+          <t>Supino Reto</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Halteres + Banco inclinado</t>
+          <t>Barra</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -11049,7 +11054,7 @@
         <v>3</v>
       </c>
       <c r="K129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L129" t="inlineStr">
         <is>
@@ -11063,7 +11068,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>peitoral, tríceps, deltóide ant.</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="P129" t="n">
@@ -11082,16 +11087,16 @@
       </c>
       <c r="T129" t="inlineStr">
         <is>
-          <t>inclinado</t>
+          <t>reto</t>
         </is>
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>halter</t>
+          <t>barra</t>
         </is>
       </c>
       <c r="V129" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W129" t="b">
         <v>1</v>
@@ -11100,17 +11105,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Barra Aberta</t>
+          <t>Supino Inclinado Halteres</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Barra</t>
+          <t>Supino Inclinado</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Barra fixa (crossover)</t>
+          <t>Halteres + Banco inclinado</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -11120,12 +11125,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>costas</t>
+          <t>peito</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>puxadas</t>
+          <t>empurrar_compostos</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -11139,43 +11144,48 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K130" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>vertical_pull_compound</t>
+          <t>horizontal_press_compound</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>dorsal, bíceps</t>
+          <t>peitoral, tríceps, deltóide ant.</t>
         </is>
       </c>
       <c r="P130" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R130" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>aberta</t>
+          <t>pronada</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>inclinado</t>
         </is>
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>corporal</t>
+          <t>halter</t>
         </is>
       </c>
       <c r="V130" t="b">
@@ -11188,7 +11198,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Barra Supinada</t>
+          <t>Barra Aberta</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11258,7 +11268,7 @@
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>supinada</t>
+          <t>aberta</t>
         </is>
       </c>
       <c r="U131" t="inlineStr">
@@ -11276,32 +11286,32 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Recuo do Estepe</t>
+          <t>Barra Supinada</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>subida_elevada</t>
+          <t>Barra</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Halteres + Caixa</t>
+          <t>Barra fixa (crossover)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>upper</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>perna_anterior</t>
+          <t>costas</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>squat_unilateral</t>
+          <t>puxadas</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -11311,14 +11321,14 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
@@ -11327,26 +11337,31 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>squat_unilateral_compound</t>
+          <t>vertical_pull_compound</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>Glúteos, Quadríceps</t>
+          <t>dorsal, bíceps</t>
         </is>
       </c>
       <c r="P132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q132" t="n">
         <v>1</v>
       </c>
       <c r="R132" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>supinada</t>
+        </is>
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>caixa</t>
+          <t>corporal</t>
         </is>
       </c>
       <c r="V132" t="b">
@@ -11359,42 +11374,42 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Russian Twist</t>
+          <t>Recuo do Estepe</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>russian twist</t>
+          <t>subida_elevada</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Halteres</t>
+          <t>Halteres + Caixa</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>core</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>core_dinamico</t>
+          <t>perna_anterior</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>rotacao_tronco</t>
+          <t>squat_unilateral</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>isolation</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J133" t="n">
@@ -11410,12 +11425,12 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>core_antirotation</t>
+          <t>squat_unilateral_compound</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>obliquos, reto abdominal</t>
+          <t>Glúteos, Quadríceps</t>
         </is>
       </c>
       <c r="P133" t="n">
@@ -11425,7 +11440,12 @@
         <v>1</v>
       </c>
       <c r="R133" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>caixa</t>
+        </is>
       </c>
       <c r="V133" t="b">
         <v>0</v>
@@ -11437,17 +11457,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>INFRA Alternado</t>
+          <t>Russian Twist</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>INFRA</t>
+          <t>russian twist</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Colchonete</t>
+          <t>Halteres</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -11462,7 +11482,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>flexao_quadril</t>
+          <t>rotacao_tronco</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -11472,14 +11492,14 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>unilateral</t>
+          <t>bilateral</t>
         </is>
       </c>
       <c r="J134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L134" t="inlineStr">
         <is>
@@ -11488,16 +11508,16 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>core_flexion</t>
+          <t>core_antirotation</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>iliopsoas, reto abdominal</t>
+          <t>obliquos, reto abdominal</t>
         </is>
       </c>
       <c r="P134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q134" t="n">
         <v>1</v>
@@ -11515,7 +11535,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>INFRA Suspenso</t>
+          <t>INFRA Alternado</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -11525,7 +11545,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Barra fixa (crossover)</t>
+          <t>Colchonete</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -11550,14 +11570,14 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>bilateral</t>
+          <t>unilateral</t>
         </is>
       </c>
       <c r="J135" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -11575,13 +11595,13 @@
         </is>
       </c>
       <c r="P135" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q135" t="n">
         <v>1</v>
       </c>
       <c r="R135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V135" t="b">
         <v>0</v>
@@ -11593,7 +11613,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>INFRA Chão</t>
+          <t>INFRA Suspenso</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -11603,7 +11623,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Colchonete</t>
+          <t>Barra fixa (crossover)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -11632,10 +11652,10 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
@@ -11653,7 +11673,7 @@
         </is>
       </c>
       <c r="P136" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q136" t="n">
         <v>1</v>
@@ -11671,78 +11691,156 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>INFRA Chão</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Colchonete</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>core_dinamico</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>flexao_quadril</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>isolation</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>bilateral</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>2</v>
+      </c>
+      <c r="K137" t="n">
+        <v>2</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>core_flexion</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>iliopsoas, reto abdominal</t>
+        </is>
+      </c>
+      <c r="P137" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>1</v>
+      </c>
+      <c r="R137" t="n">
+        <v>3</v>
+      </c>
+      <c r="V137" t="b">
+        <v>0</v>
+      </c>
+      <c r="W137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
           <t>INFRA Roll-Up</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B138" t="inlineStr">
         <is>
           <t>INFRA</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
+      <c r="C138" t="inlineStr">
         <is>
           <t>Colchonete</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr">
+      <c r="E138" t="inlineStr">
         <is>
           <t>core</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr">
+      <c r="F138" t="inlineStr">
         <is>
           <t>core_dinamico</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr">
+      <c r="G138" t="inlineStr">
         <is>
           <t>flexao_quadril</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr">
+      <c r="H138" t="inlineStr">
         <is>
           <t>isolation</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
+      <c r="I138" t="inlineStr">
         <is>
           <t>bilateral</t>
         </is>
       </c>
-      <c r="J137" t="n">
-        <v>3</v>
-      </c>
-      <c r="K137" t="n">
-        <v>3</v>
-      </c>
-      <c r="L137" t="inlineStr">
+      <c r="J138" t="n">
+        <v>3</v>
+      </c>
+      <c r="K138" t="n">
+        <v>3</v>
+      </c>
+      <c r="L138" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr">
+      <c r="M138" t="inlineStr">
         <is>
           <t>core_flexion</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr">
+      <c r="N138" t="inlineStr">
         <is>
           <t>iliopsoas, reto abdominal</t>
         </is>
       </c>
-      <c r="P137" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q137" t="n">
-        <v>1</v>
-      </c>
-      <c r="R137" t="n">
-        <v>3</v>
-      </c>
-      <c r="V137" t="b">
-        <v>0</v>
-      </c>
-      <c r="W137" t="b">
+      <c r="P138" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q138" t="n">
+        <v>1</v>
+      </c>
+      <c r="R138" t="n">
+        <v>3</v>
+      </c>
+      <c r="V138" t="b">
+        <v>0</v>
+      </c>
+      <c r="W138" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
banco(pre-mvp): correções de cadastro pré-Fatia 1 (knee_extension + inativos + notas)
- knee_extension: novo padrão (perna_anterior/quad) em PADRAO_PARA_SUBREGIAO
  e GRUPO_MUSCULAR_PADRAO; Cadeira Extensora movida de squat_bilateral
- Hip Thrust base: purpose compound -> isolation (alinha 9 variações)
- Box Jump, Air Bike (Sprint/Steady State): ativo=False
- Agach. Lateral: corrigido explosive -> compound, mantido ativo
- docs/refatoracao/notas_cadastro.md: registro das decisões clínicas
- testes: counts de carga (98/118/125) + re-pin seed pair + snapshots
- inclui os dois bancos .xlsx de backup (Copy removido, pre CSP adicionado)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/banco_exercicios.xlsx
+++ b/banco_exercicios.xlsx
@@ -761,7 +761,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>explosive</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -1226,7 +1226,11 @@
           <t>full body, cardiovascular</t>
         </is>
       </c>
-      <c r="O10" s="2" t="n"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>inativo em 2026-05-21. Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P10" s="4" t="n">
         <v>1</v>
       </c>
@@ -1242,7 +1246,9 @@
       <c r="V10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="W10" s="2" t="n"/>
+      <c r="W10" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="X10" s="2" t="n"/>
       <c r="Y10" s="2" t="n"/>
       <c r="Z10" s="2" t="n"/>
@@ -1310,7 +1316,11 @@
           <t>full body, cardiovascular</t>
         </is>
       </c>
-      <c r="O11" s="2" t="n"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>inativo em 2026-05-21. Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P11" s="4" t="n">
         <v>1</v>
       </c>
@@ -1326,7 +1336,9 @@
       <c r="V11" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="W11" s="2" t="n"/>
+      <c r="W11" s="2" t="b">
+        <v>0</v>
+      </c>
       <c r="X11" s="2" t="n"/>
       <c r="Y11" s="2" t="n"/>
       <c r="Z11" s="2" t="n"/>
@@ -2382,7 +2394,11 @@
           <t>quadríceps, glúteos</t>
         </is>
       </c>
-      <c r="O23" s="2" t="n"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>inativo em 2026-05-21. Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P23" s="4" t="n">
         <v>0</v>
       </c>
@@ -2430,7 +2446,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>squat_bilateral</t>
+          <t>knee_extension</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2464,7 +2480,11 @@
           <t>quadríceps</t>
         </is>
       </c>
-      <c r="O24" s="2" t="n"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>padrão knee_extension criado em 2026-05-21 (movido de squat_bilateral). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P24" s="4" t="n">
         <v>0</v>
       </c>
@@ -5183,7 +5203,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>compound</t>
+          <t>isolation</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -5212,7 +5232,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O55" s="2" t="n"/>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P55" s="4" t="n">
         <v>0</v>
       </c>
@@ -5308,7 +5332,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O56" s="2" t="n"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
@@ -5400,7 +5428,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O57" s="2" t="n"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P57" s="4" t="n">
         <v>0</v>
       </c>
@@ -6372,7 +6404,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O68" s="2" t="n"/>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P68" s="4" t="n">
         <v>0</v>
       </c>
@@ -6468,7 +6504,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O69" s="2" t="n"/>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P69" s="4" t="n">
         <v>0</v>
       </c>
@@ -6564,7 +6604,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O70" s="2" t="n"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P70" s="4" t="n">
         <v>0</v>
       </c>
@@ -6660,7 +6704,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O71" s="2" t="n"/>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P71" s="4" t="n">
         <v>0</v>
       </c>
@@ -6756,7 +6804,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O72" s="2" t="n"/>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
@@ -6848,7 +6900,11 @@
           <t>glúteos</t>
         </is>
       </c>
-      <c r="O73" s="2" t="n"/>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>purpose=isolation deliberado (não erro). Ver notas_cadastro.md.</t>
+        </is>
+      </c>
       <c r="P73" s="4" t="n">
         <v>0</v>
       </c>

</xml_diff>